<commit_message>
Update dividend calendar 2026-03-09
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -561,7 +561,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estimated Dividend Increase Announcement Calendar - 03/06/2026</t>
+          <t>Estimated Dividend Increase Announcement Calendar - 03/09/2026</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         <v>46096</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>46300</v>
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="L6" s="9" t="n">
-        <v>0.02091029465724359</v>
+        <v>0.02123442826954228</v>
       </c>
     </row>
     <row r="7">
@@ -712,7 +712,7 @@
         <v>46096</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>46196</v>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.05013927363491755</v>
+        <v>0.05043193807276123</v>
       </c>
     </row>
     <row r="8">
@@ -758,7 +758,7 @@
         <v>46122</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>46132</v>
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.02760692241919218</v>
+        <v>0.02742783112167496</v>
       </c>
     </row>
     <row r="9">
@@ -804,7 +804,7 @@
         <v>46127</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>46503</v>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>0.01863128817928794</v>
+        <v>0.01920125840726826</v>
       </c>
     </row>
     <row r="10">
@@ -850,7 +850,7 @@
         <v>46128</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>46165</v>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.02179425374964139</v>
+        <v>0.02153164487221803</v>
       </c>
     </row>
     <row r="11">
@@ -896,7 +896,7 @@
         <v>46134</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46161</v>
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.03100775159142471</v>
+        <v>0.03071620865694696</v>
       </c>
     </row>
     <row r="12">
@@ -942,7 +942,7 @@
         <v>46141</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>46191</v>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0.05029091984291129</v>
+        <v>0.04996858131518413</v>
       </c>
     </row>
     <row r="13">
@@ -988,7 +988,7 @@
         <v>46143</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>46152</v>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>0.04367386099191616</v>
+        <v>0.04428952183157404</v>
       </c>
     </row>
     <row r="14">
@@ -1034,7 +1034,7 @@
         <v>46162</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>46198</v>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.03125000094443982</v>
+        <v>0.03135003990293934</v>
       </c>
     </row>
     <row r="15">
@@ -1080,7 +1080,7 @@
         <v>46176</v>
       </c>
       <c r="I15" s="20" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="J15" s="19" t="n">
         <v>46197</v>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="L15" s="18" t="n">
-        <v>0.03963385818268213</v>
+        <v>0.03995053847357968</v>
       </c>
     </row>
     <row r="16">
@@ -1126,7 +1126,7 @@
         <v>46218</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>46248</v>
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="L16" s="9" t="n">
-        <v>0.01803942519245617</v>
+        <v>0.01847529122044088</v>
       </c>
     </row>
     <row r="17">
@@ -1172,7 +1172,7 @@
         <v>46220</v>
       </c>
       <c r="I17" s="13" t="n">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>46264</v>
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.02161061800994751</v>
+        <v>0.02209016195988108</v>
       </c>
     </row>
     <row r="18">
@@ -1218,7 +1218,7 @@
         <v>46227</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>46267</v>
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.04412839732925053</v>
+        <v>0.04586268860329277</v>
       </c>
     </row>
     <row r="19">
@@ -1264,7 +1264,7 @@
         <v>46232</v>
       </c>
       <c r="I19" s="13" t="n">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>46246</v>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0.0434896963373957</v>
+        <v>0.04514220705346985</v>
       </c>
     </row>
     <row r="20">
@@ -1310,7 +1310,7 @@
         <v>46232</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>46264</v>
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0.02961427247426216</v>
+        <v>0.02994460207493484</v>
       </c>
     </row>
     <row r="21">
@@ -1356,7 +1356,7 @@
         <v>46263</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46297</v>
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.02880983789161461</v>
+        <v>0.02911414781981898</v>
       </c>
     </row>
     <row r="22">
@@ -1402,7 +1402,7 @@
         <v>46267</v>
       </c>
       <c r="I22" s="13" t="n">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="J22" s="10" t="n">
         <v>46303</v>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="L22" s="9" t="n">
-        <v>0.05433605865719647</v>
+        <v>0.05419734985467445</v>
       </c>
     </row>
     <row r="23">
@@ -1448,7 +1448,7 @@
         <v>46278</v>
       </c>
       <c r="I23" s="13" t="n">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>46344</v>
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0.008881514816818951</v>
+        <v>0.008929447230883993</v>
       </c>
     </row>
     <row r="24">
@@ -1494,7 +1494,7 @@
         <v>46285</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="J24" s="10" t="n">
         <v>46325</v>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="L24" s="9" t="n">
-        <v>0.02941633490976144</v>
+        <v>0.02961572656987358</v>
       </c>
     </row>
     <row r="25">
@@ -1540,7 +1540,7 @@
         <v>46305</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>46339</v>
@@ -1551,7 +1551,7 @@
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>0.0384657892455476</v>
+        <v>0.03938879524734049</v>
       </c>
     </row>
     <row r="26">
@@ -1586,7 +1586,7 @@
         <v>46311</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>46386</v>
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0.01197083029429245</v>
+        <v>0.01218125357404984</v>
       </c>
     </row>
     <row r="27">
@@ -1632,7 +1632,7 @@
         <v>46317</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>46351</v>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="L27" s="9" t="n">
-        <v>0.01280653322421403</v>
+        <v>0.01305087977945609</v>
       </c>
     </row>
     <row r="28">
@@ -1678,7 +1678,7 @@
         <v>46322</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>46338</v>
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="L28" s="9" t="n">
-        <v>0.02432535207111895</v>
+        <v>0.0247438625812264</v>
       </c>
     </row>
     <row r="29">
@@ -1724,7 +1724,7 @@
         <v>46329</v>
       </c>
       <c r="I29" s="13" t="n">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>46338</v>
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>0.00670822057103366</v>
+        <v>0.006716574317527649</v>
       </c>
     </row>
     <row r="30">
@@ -1770,7 +1770,7 @@
         <v>46332</v>
       </c>
       <c r="I30" s="13" t="n">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="J30" s="10" t="n">
         <v>46346</v>
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="L30" s="9" t="n">
-        <v>0.02614869390488948</v>
+        <v>0.02662955919332545</v>
       </c>
     </row>
     <row r="31">
@@ -1816,7 +1816,7 @@
         <v>46341</v>
       </c>
       <c r="I31" s="13" t="n">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>46339</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="n">
-        <v>0.02711775290341838</v>
+        <v>0.02687365511453597</v>
       </c>
     </row>
     <row r="32">
@@ -1862,7 +1862,7 @@
         <v>46344</v>
       </c>
       <c r="I32" s="13" t="n">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>46385</v>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="L32" s="9" t="n">
-        <v>0.02969378118246405</v>
+        <v>0.02996960741873846</v>
       </c>
     </row>
     <row r="33">
@@ -1908,7 +1908,7 @@
         <v>46347</v>
       </c>
       <c r="I33" s="13" t="n">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>46358</v>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>0.02873412138550337</v>
+        <v>0.0293796246055187</v>
       </c>
     </row>
     <row r="34">
@@ -1954,7 +1954,7 @@
         <v>46352</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>46400</v>
@@ -1965,7 +1965,7 @@
         </is>
       </c>
       <c r="L34" s="9" t="n">
-        <v>0.04825030695041271</v>
+        <v>0.04913016233452121</v>
       </c>
     </row>
     <row r="35">
@@ -2000,7 +2000,7 @@
         <v>46360</v>
       </c>
       <c r="I35" s="13" t="n">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>46371</v>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0.04750459268387158</v>
+        <v>0.04944084822343214</v>
       </c>
     </row>
     <row r="36">
@@ -2046,7 +2046,7 @@
         <v>46366</v>
       </c>
       <c r="I36" s="13" t="n">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>46432</v>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="L36" s="9" t="n">
-        <v>0.0273942735353147</v>
+        <v>0.02715992761331142</v>
       </c>
     </row>
     <row r="37">
@@ -2092,7 +2092,7 @@
         <v>46370</v>
       </c>
       <c r="I37" s="13" t="n">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>46413</v>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>0.06450402928726036</v>
+        <v>0.0649056603773585</v>
       </c>
     </row>
     <row r="38">
@@ -2138,7 +2138,7 @@
         <v>46371</v>
       </c>
       <c r="I38" s="13" t="n">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>46344</v>
@@ -2149,7 +2149,7 @@
         </is>
       </c>
       <c r="L38" s="9" t="n">
-        <v>0.02107191945064864</v>
+        <v>0.02131603343958685</v>
       </c>
     </row>
     <row r="39">
@@ -2184,7 +2184,7 @@
         <v>46411</v>
       </c>
       <c r="I39" s="13" t="n">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>46435</v>
@@ -2195,7 +2195,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.03827412485747456</v>
+        <v>0.03888005694645721</v>
       </c>
     </row>
     <row r="40">
@@ -2230,7 +2230,7 @@
         <v>46416</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="J40" s="10" t="n">
         <v>46483</v>
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.01596288658098838</v>
+        <v>0.01616161616161616</v>
       </c>
     </row>
     <row r="41">
@@ -2276,7 +2276,7 @@
         <v>46417</v>
       </c>
       <c r="I41" s="13" t="n">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>46433</v>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>0.03753690570923929</v>
+        <v>0.03728334269512545</v>
       </c>
     </row>
     <row r="42">
@@ -2322,7 +2322,7 @@
         <v>46419</v>
       </c>
       <c r="I42" s="13" t="n">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="J42" s="10" t="n">
         <v>46472</v>
@@ -2333,7 +2333,7 @@
         </is>
       </c>
       <c r="L42" s="9" t="n">
-        <v>0.03025906855367032</v>
+        <v>0.02953970594222538</v>
       </c>
     </row>
     <row r="43">
@@ -2368,7 +2368,7 @@
         <v>46423</v>
       </c>
       <c r="I43" s="13" t="n">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>46435</v>
@@ -2379,7 +2379,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>0.06470066120416362</v>
+        <v>0.06718558010043858</v>
       </c>
     </row>
     <row r="44">
@@ -2414,7 +2414,7 @@
         <v>46428</v>
       </c>
       <c r="I44" s="13" t="n">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="J44" s="10" t="n">
         <v>46452</v>
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="L44" s="9" t="n">
-        <v>0.01441483983229846</v>
+        <v>0.01437492589275465</v>
       </c>
     </row>
     <row r="45">
@@ -2460,7 +2460,7 @@
         <v>46430</v>
       </c>
       <c r="I45" s="13" t="n">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="J45" s="10" t="n">
         <v>46460</v>
@@ -2471,13 +2471,13 @@
         </is>
       </c>
       <c r="L45" s="9" t="n">
-        <v>0.05657330701696998</v>
+        <v>0.05776665748201185</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>RHI</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
@@ -2487,29 +2487,29 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="D46" s="7" t="n">
-        <v>0.59</v>
+        <v>0.41</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>0.53</v>
+        <v>0.4</v>
       </c>
       <c r="F46" s="8" t="n">
-        <v>0.1132075471698112</v>
+        <v>0.02499999999999988</v>
       </c>
       <c r="G46" s="9" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="H46" s="10" t="n">
-        <v>46431</v>
+        <v>46432</v>
       </c>
       <c r="I46" s="13" t="n">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="J46" s="10" t="n">
-        <v>46442</v>
+        <v>46481</v>
       </c>
       <c r="K46" s="12" t="inlineStr">
         <is>
@@ -2517,45 +2517,45 @@
         </is>
       </c>
       <c r="L46" s="9" t="n">
-        <v>0.09570154154918477</v>
+        <v>0.02167305457492465</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Quarterly</t>
+          <t>Semi-Annual</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="D47" s="7" t="n">
-        <v>0.41</v>
+        <v>1.883</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>0.4</v>
+        <v>1.864</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>0.02499999999999988</v>
+        <v>0.01019313304721025</v>
       </c>
       <c r="G47" s="9" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="H47" s="10" t="n">
-        <v>46432</v>
+        <v>46433</v>
       </c>
       <c r="I47" s="13" t="n">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="J47" s="10" t="n">
-        <v>46481</v>
+        <v>46425</v>
       </c>
       <c r="K47" s="12" t="inlineStr">
         <is>
@@ -2563,45 +2563,45 @@
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>0.02076212234906543</v>
+        <v>0.002867978565556691</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Semi-Annual</t>
+          <t>Quarterly</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Dec</t>
         </is>
       </c>
       <c r="D48" s="7" t="n">
-        <v>1.883</v>
+        <v>1.25</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>1.864</v>
+        <v>1.15</v>
       </c>
       <c r="F48" s="8" t="n">
-        <v>0.01019313304721025</v>
+        <v>4.043478260869565</v>
       </c>
       <c r="G48" s="9" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="H48" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="I48" s="13" t="n">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="J48" s="10" t="n">
-        <v>46425</v>
+        <v>46383</v>
       </c>
       <c r="K48" s="12" t="inlineStr">
         <is>
@@ -2609,13 +2609,13 @@
         </is>
       </c>
       <c r="L48" s="9" t="n">
-        <v>0.002844991090000402</v>
+        <v>0.0157497678726076</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>DVN</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
@@ -2625,17 +2625,17 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Dec</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="D49" s="7" t="n">
-        <v>1.25</v>
+        <v>0.24</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>1.15</v>
+        <v>0.22</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>4.043478260869565</v>
+        <v>0.09090909090909087</v>
       </c>
       <c r="G49" s="9" t="n">
         <v>0.06</v>
@@ -2644,10 +2644,10 @@
         <v>46433</v>
       </c>
       <c r="I49" s="13" t="n">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="J49" s="10" t="n">
-        <v>46383</v>
+        <v>46276</v>
       </c>
       <c r="K49" s="12" t="inlineStr">
         <is>
@@ -2655,13 +2655,13 @@
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>0.01577112918840002</v>
+        <v>0.0209422706286886</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>DVN</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
@@ -2671,17 +2671,17 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="D50" s="7" t="n">
-        <v>0.24</v>
+        <v>1.423</v>
       </c>
       <c r="E50" s="7" t="n">
-        <v>0.22</v>
+        <v>1.355</v>
       </c>
       <c r="F50" s="8" t="n">
-        <v>0.09090909090909087</v>
+        <v>0.05018450184501849</v>
       </c>
       <c r="G50" s="9" t="n">
         <v>0.06</v>
@@ -2690,10 +2690,10 @@
         <v>46433</v>
       </c>
       <c r="I50" s="13" t="n">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="J50" s="10" t="n">
-        <v>46276</v>
+        <v>46177</v>
       </c>
       <c r="K50" s="12" t="inlineStr">
         <is>
@@ -2701,13 +2701,13 @@
         </is>
       </c>
       <c r="L50" s="9" t="n">
-        <v>0.02145011679340417</v>
+        <v>0.035575</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>PFG</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
@@ -2717,29 +2717,29 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="D51" s="7" t="n">
-        <v>1.423</v>
+        <v>0.79</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>1.355</v>
+        <v>0.78</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>0.05018450184501849</v>
+        <v>0.01282051282051283</v>
       </c>
       <c r="G51" s="9" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="H51" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="I51" s="13" t="n">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="J51" s="10" t="n">
-        <v>46177</v>
+        <v>46270</v>
       </c>
       <c r="K51" s="12" t="inlineStr">
         <is>
@@ -2747,13 +2747,13 @@
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>0.03607783384584436</v>
+        <v>0.03556355726313094</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>PFG</t>
+          <t>UL</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -2763,29 +2763,29 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>Aug</t>
         </is>
       </c>
       <c r="D52" s="7" t="n">
-        <v>0.79</v>
+        <v>0.555</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>0.78</v>
+        <v>0.588964</v>
       </c>
       <c r="F52" s="8" t="n">
-        <v>0.01282051282051283</v>
+        <v>0.005735494868956323</v>
       </c>
       <c r="G52" s="9" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="H52" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="I52" s="13" t="n">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="J52" s="10" t="n">
-        <v>46270</v>
+        <v>46243</v>
       </c>
       <c r="K52" s="12" t="inlineStr">
         <is>
@@ -2793,13 +2793,13 @@
         </is>
       </c>
       <c r="L52" s="9" t="n">
-        <v>0.0346111708036702</v>
+        <v>0.03373347640718918</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>UL</t>
+          <t>ALSN</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -2809,29 +2809,29 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Aug</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
-        <v>0.555</v>
+        <v>0.27</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>0.588964</v>
+        <v>0.25</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>0.005735494868956323</v>
+        <v>0.08000000000000007</v>
       </c>
       <c r="G53" s="9" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="H53" s="10" t="n">
-        <v>46433</v>
+        <v>46440</v>
       </c>
       <c r="I53" s="13" t="n">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="J53" s="10" t="n">
-        <v>46243</v>
+        <v>46449</v>
       </c>
       <c r="K53" s="12" t="inlineStr">
         <is>
@@ -2839,13 +2839,13 @@
         </is>
       </c>
       <c r="L53" s="9" t="n">
-        <v>0.03333834092339166</v>
+        <v>0.0095566762196685</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>ALSN</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -2859,25 +2859,25 @@
         </is>
       </c>
       <c r="D54" s="7" t="n">
-        <v>0.27</v>
+        <v>2.3</v>
       </c>
       <c r="E54" s="7" t="n">
-        <v>0.25</v>
+        <v>2.25</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>0.08000000000000007</v>
+        <v>0.02222222222222214</v>
       </c>
       <c r="G54" s="9" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="H54" s="10" t="n">
         <v>46440</v>
       </c>
       <c r="I54" s="13" t="n">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="J54" s="10" t="n">
-        <v>46449</v>
+        <v>46455</v>
       </c>
       <c r="K54" s="12" t="inlineStr">
         <is>
@@ -2885,13 +2885,13 @@
         </is>
       </c>
       <c r="L54" s="9" t="n">
-        <v>0.009166525231687333</v>
+        <v>0.02635385774024195</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>GD</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
@@ -2901,29 +2901,29 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="D55" s="7" t="n">
-        <v>2.3</v>
+        <v>1.5</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>2.25</v>
+        <v>1.42</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>0.02222222222222214</v>
+        <v>0.05633802816901413</v>
       </c>
       <c r="G55" s="9" t="n">
         <v>0.08</v>
       </c>
       <c r="H55" s="10" t="n">
-        <v>46440</v>
+        <v>46451</v>
       </c>
       <c r="I55" s="13" t="n">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="J55" s="10" t="n">
-        <v>46455</v>
+        <v>46487</v>
       </c>
       <c r="K55" s="12" t="inlineStr">
         <is>
@@ -2931,53 +2931,7 @@
         </is>
       </c>
       <c r="L55" s="9" t="n">
-        <v>0.02575155278654199</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>Apr</t>
-        </is>
-      </c>
-      <c r="D56" s="7" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E56" s="7" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="F56" s="8" t="n">
-        <v>0.05633802816901413</v>
-      </c>
-      <c r="G56" s="9" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="H56" s="10" t="n">
-        <v>46451</v>
-      </c>
-      <c r="I56" s="13" t="n">
-        <v>364</v>
-      </c>
-      <c r="J56" s="10" t="n">
-        <v>46487</v>
-      </c>
-      <c r="K56" s="12" t="inlineStr">
-        <is>
-          <t>Notion + yfinance</t>
-        </is>
-      </c>
-      <c r="L56" s="9" t="n">
-        <v>0.01658031088082901</v>
+        <v>0.01678087038133019</v>
       </c>
     </row>
   </sheetData>
@@ -2991,7 +2945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3012,7 +2966,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Expected Increase Announcements by Month - 03/06/2026</t>
+          <t>Expected Increase Announcements by Month - 03/09/2026</t>
         </is>
       </c>
     </row>
@@ -4447,20 +4401,20 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>RHI</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B79" s="10" t="n">
-        <v>46431</v>
+        <v>46432</v>
       </c>
       <c r="C79" s="10" t="n">
-        <v>46442</v>
+        <v>46481</v>
       </c>
       <c r="D79" s="7" t="n">
-        <v>0.59</v>
+        <v>0.41</v>
       </c>
       <c r="E79" s="8" t="n">
-        <v>0.1132075471698112</v>
+        <v>0.02499999999999988</v>
       </c>
       <c r="F79" s="12" t="inlineStr">
         <is>
@@ -4471,20 +4425,20 @@
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B80" s="10" t="n">
-        <v>46432</v>
+        <v>46433</v>
       </c>
       <c r="C80" s="10" t="n">
-        <v>46481</v>
+        <v>46425</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>0.41</v>
+        <v>1.883</v>
       </c>
       <c r="E80" s="8" t="n">
-        <v>0.02499999999999988</v>
+        <v>0.01019313304721025</v>
       </c>
       <c r="F80" s="12" t="inlineStr">
         <is>
@@ -4495,20 +4449,20 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="B81" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="C81" s="10" t="n">
-        <v>46425</v>
+        <v>46383</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>1.883</v>
+        <v>1.25</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>0.01019313304721025</v>
+        <v>4.043478260869565</v>
       </c>
       <c r="F81" s="12" t="inlineStr">
         <is>
@@ -4519,20 +4473,20 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>DVN</t>
         </is>
       </c>
       <c r="B82" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="C82" s="10" t="n">
-        <v>46383</v>
+        <v>46276</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>1.25</v>
+        <v>0.24</v>
       </c>
       <c r="E82" s="8" t="n">
-        <v>4.043478260869565</v>
+        <v>0.09090909090909087</v>
       </c>
       <c r="F82" s="12" t="inlineStr">
         <is>
@@ -4543,20 +4497,20 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>DVN</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B83" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="C83" s="10" t="n">
-        <v>46276</v>
+        <v>46177</v>
       </c>
       <c r="D83" s="7" t="n">
-        <v>0.24</v>
+        <v>1.423</v>
       </c>
       <c r="E83" s="8" t="n">
-        <v>0.09090909090909087</v>
+        <v>0.05018450184501849</v>
       </c>
       <c r="F83" s="12" t="inlineStr">
         <is>
@@ -4567,20 +4521,20 @@
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>PFG</t>
         </is>
       </c>
       <c r="B84" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="C84" s="10" t="n">
-        <v>46177</v>
+        <v>46270</v>
       </c>
       <c r="D84" s="7" t="n">
-        <v>1.423</v>
+        <v>0.79</v>
       </c>
       <c r="E84" s="8" t="n">
-        <v>0.05018450184501849</v>
+        <v>0.01282051282051283</v>
       </c>
       <c r="F84" s="12" t="inlineStr">
         <is>
@@ -4591,20 +4545,20 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>PFG</t>
+          <t>UL</t>
         </is>
       </c>
       <c r="B85" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="C85" s="10" t="n">
-        <v>46270</v>
+        <v>46243</v>
       </c>
       <c r="D85" s="7" t="n">
-        <v>0.79</v>
+        <v>0.555</v>
       </c>
       <c r="E85" s="8" t="n">
-        <v>0.01282051282051283</v>
+        <v>0.005735494868956323</v>
       </c>
       <c r="F85" s="12" t="inlineStr">
         <is>
@@ -4615,20 +4569,20 @@
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>UL</t>
+          <t>ALSN</t>
         </is>
       </c>
       <c r="B86" s="10" t="n">
-        <v>46433</v>
+        <v>46440</v>
       </c>
       <c r="C86" s="10" t="n">
-        <v>46243</v>
+        <v>46449</v>
       </c>
       <c r="D86" s="7" t="n">
-        <v>0.555</v>
+        <v>0.27</v>
       </c>
       <c r="E86" s="8" t="n">
-        <v>0.005735494868956323</v>
+        <v>0.08000000000000007</v>
       </c>
       <c r="F86" s="12" t="inlineStr">
         <is>
@@ -4639,20 +4593,20 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>ALSN</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B87" s="10" t="n">
         <v>46440</v>
       </c>
       <c r="C87" s="10" t="n">
-        <v>46449</v>
+        <v>46455</v>
       </c>
       <c r="D87" s="7" t="n">
-        <v>0.27</v>
+        <v>2.3</v>
       </c>
       <c r="E87" s="8" t="n">
-        <v>0.08000000000000007</v>
+        <v>0.02222222222222214</v>
       </c>
       <c r="F87" s="12" t="inlineStr">
         <is>
@@ -4660,88 +4614,64 @@
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="5" t="inlineStr">
-        <is>
-          <t>HD</t>
-        </is>
-      </c>
-      <c r="B88" s="10" t="n">
-        <v>46440</v>
-      </c>
-      <c r="C88" s="10" t="n">
-        <v>46455</v>
-      </c>
-      <c r="D88" s="7" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="E88" s="8" t="n">
-        <v>0.02222222222222214</v>
-      </c>
-      <c r="F88" s="12" t="inlineStr">
-        <is>
-          <t>Notion + yfinance</t>
+    <row r="89">
+      <c r="A89" s="22" t="inlineStr">
+        <is>
+          <t>March 2027</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="22" t="inlineStr">
-        <is>
-          <t>March 2027</t>
+      <c r="A90" s="23" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B90" s="23" t="inlineStr">
+        <is>
+          <t>Est. Announce</t>
+        </is>
+      </c>
+      <c r="C90" s="23" t="inlineStr">
+        <is>
+          <t>Est. Ex-Date</t>
+        </is>
+      </c>
+      <c r="D90" s="23" t="inlineStr">
+        <is>
+          <t>Last Amount</t>
+        </is>
+      </c>
+      <c r="E90" s="23" t="inlineStr">
+        <is>
+          <t>Last Change</t>
+        </is>
+      </c>
+      <c r="F90" s="23" t="inlineStr">
+        <is>
+          <t>Source</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="23" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B91" s="23" t="inlineStr">
-        <is>
-          <t>Est. Announce</t>
-        </is>
-      </c>
-      <c r="C91" s="23" t="inlineStr">
-        <is>
-          <t>Est. Ex-Date</t>
-        </is>
-      </c>
-      <c r="D91" s="23" t="inlineStr">
-        <is>
-          <t>Last Amount</t>
-        </is>
-      </c>
-      <c r="E91" s="23" t="inlineStr">
-        <is>
-          <t>Last Change</t>
-        </is>
-      </c>
-      <c r="F91" s="23" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="5" t="inlineStr">
+      <c r="A91" s="5" t="inlineStr">
         <is>
           <t>GD</t>
         </is>
       </c>
-      <c r="B92" s="10" t="n">
+      <c r="B91" s="10" t="n">
         <v>46451</v>
       </c>
-      <c r="C92" s="10" t="n">
+      <c r="C91" s="10" t="n">
         <v>46487</v>
       </c>
-      <c r="D92" s="7" t="n">
+      <c r="D91" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="E92" s="8" t="n">
+      <c r="E91" s="8" t="n">
         <v>0.05633802816901413</v>
       </c>
-      <c r="F92" s="12" t="inlineStr">
+      <c r="F91" s="12" t="inlineStr">
         <is>
           <t>Notion + yfinance</t>
         </is>
@@ -4758,7 +4688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M55"/>
+  <dimension ref="A1:M54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4786,7 +4716,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete Holdings Dividend Summary - 03/06/2026</t>
+          <t>Complete Holdings Dividend Summary - 03/09/2026</t>
         </is>
       </c>
     </row>
@@ -4890,7 +4820,7 @@
         <v>1.08</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.009166525231687333</v>
+        <v>0.0095566762196685</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>45982</v>
@@ -4943,7 +4873,7 @@
         <v>10.08</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.0273942735353147</v>
+        <v>0.02715992761331142</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>46066</v>
@@ -4996,7 +4926,7 @@
         <v>3.766</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.002844991090000402</v>
+        <v>0.002867978565556691</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>46063</v>
@@ -5049,7 +4979,7 @@
         <v>2.812</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.03827412485747456</v>
+        <v>0.03888005694645721</v>
       </c>
       <c r="I8" s="10" t="n">
         <v>46070</v>
@@ -5102,7 +5032,7 @@
         <v>4</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.02961427247426216</v>
+        <v>0.02994460207493484</v>
       </c>
       <c r="I9" s="10" t="n">
         <v>46080</v>
@@ -5155,7 +5085,7 @@
         <v>4.96</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.0434896963373957</v>
+        <v>0.04514220705346985</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>46050</v>
@@ -5208,7 +5138,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.01577112918840002</v>
+        <v>0.0157497678726076</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>46003</v>
@@ -5261,7 +5191,7 @@
         <v>0.92</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.02107191945064864</v>
+        <v>0.02131603343958685</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>46072</v>
@@ -5314,7 +5244,7 @@
         <v>2.4</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0.00670822057103366</v>
+        <v>0.006716574317527649</v>
       </c>
       <c r="I13" s="10" t="n">
         <v>46066</v>
@@ -5367,7 +5297,7 @@
         <v>1.64</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0.02076212234906543</v>
+        <v>0.02167305457492465</v>
       </c>
       <c r="I14" s="10" t="n">
         <v>46024</v>
@@ -5420,7 +5350,7 @@
         <v>7.12</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.03753690570923929</v>
+        <v>0.03728334269512545</v>
       </c>
       <c r="I15" s="10" t="n">
         <v>46070</v>
@@ -5473,7 +5403,7 @@
         <v>3.2</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.01596288658098838</v>
+        <v>0.01616161616161616</v>
       </c>
       <c r="I16" s="10" t="n">
         <v>46035</v>
@@ -5526,7 +5456,7 @@
         <v>0.96</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.02145011679340417</v>
+        <v>0.0209422706286886</v>
       </c>
       <c r="I17" s="10" t="n">
         <v>46006</v>
@@ -5579,7 +5509,7 @@
         <v>3.36</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.04750459268387158</v>
+        <v>0.04944084822343214</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>46006</v>
@@ -5632,7 +5562,7 @@
         <v>2.56</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.02432535207111895</v>
+        <v>0.0247438625812264</v>
       </c>
       <c r="I19" s="10" t="n">
         <v>46062</v>
@@ -5685,7 +5615,7 @@
         <v>6</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.01658031088082901</v>
+        <v>0.01678087038133019</v>
       </c>
       <c r="I20" s="10" t="n">
         <v>46038</v>
@@ -5738,7 +5668,7 @@
         <v>9.199999999999999</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.02575155278654199</v>
+        <v>0.02635385774024195</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>45995</v>
@@ -5791,7 +5721,7 @@
         <v>5.52</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>0.01280653322421403</v>
+        <v>0.01305087977945609</v>
       </c>
       <c r="I22" s="10" t="n">
         <v>46080</v>
@@ -5844,7 +5774,7 @@
         <v>1.172</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.04825030695041271</v>
+        <v>0.04913016233452121</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>46034</v>
@@ -5897,7 +5827,7 @@
         <v>3.28</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>0.02880983789161461</v>
+        <v>0.02911414781981898</v>
       </c>
       <c r="I24" s="10" t="n">
         <v>46024</v>
@@ -5950,7 +5880,7 @@
         <v>2.44</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.01441483983229846</v>
+        <v>0.01437492589275465</v>
       </c>
       <c r="I25" s="10" t="n">
         <v>46086</v>
@@ -6003,7 +5933,7 @@
         <v>5.2</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>0.02179425374964139</v>
+        <v>0.02153164487221803</v>
       </c>
       <c r="I26" s="10" t="n">
         <v>46077</v>
@@ -6056,7 +5986,7 @@
         <v>6</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.02091029465724359</v>
+        <v>0.02123442826954228</v>
       </c>
       <c r="I27" s="10" t="n">
         <v>46028</v>
@@ -6109,7 +6039,7 @@
         <v>1.952</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0.01863128817928794</v>
+        <v>0.01920125840726826</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>45853</v>
@@ -6162,7 +6092,7 @@
         <v>3.16</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.01197083029429245</v>
+        <v>0.01218125357404984</v>
       </c>
       <c r="I29" s="10" t="n">
         <v>46022</v>
@@ -6215,7 +6145,7 @@
         <v>2.84</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.03125000094443982</v>
+        <v>0.03135003990293934</v>
       </c>
       <c r="I30" s="10" t="n">
         <v>46017</v>
@@ -6268,7 +6198,7 @@
         <v>1.92</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0.02969378118246405</v>
+        <v>0.02996960741873846</v>
       </c>
       <c r="I31" s="10" t="n">
         <v>46020</v>
@@ -6321,7 +6251,7 @@
         <v>3.64</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.008881514816818951</v>
+        <v>0.008929447230883993</v>
       </c>
       <c r="I32" s="10" t="n">
         <v>46072</v>
@@ -6374,7 +6304,7 @@
         <v>3.48</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0.0384657892455476</v>
+        <v>0.03938879524734049</v>
       </c>
       <c r="I33" s="10" t="n">
         <v>46036</v>
@@ -6427,7 +6357,7 @@
         <v>1.64</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0.02873412138550337</v>
+        <v>0.0293796246055187</v>
       </c>
       <c r="I34" s="10" t="n">
         <v>46083</v>
@@ -6480,7 +6410,7 @@
         <v>1.168</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0.03025906855367032</v>
+        <v>0.02953970594222538</v>
       </c>
       <c r="I35" s="10" t="n">
         <v>45887</v>
@@ -6533,7 +6463,7 @@
         <v>3.24</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0.05013927363491755</v>
+        <v>0.05043193807276123</v>
       </c>
       <c r="I36" s="10" t="n">
         <v>46080</v>
@@ -6586,7 +6516,7 @@
         <v>4.32</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.04367386099191616</v>
+        <v>0.04428952183157404</v>
       </c>
       <c r="I37" s="10" t="n">
         <v>46050</v>
@@ -6639,10 +6569,10 @@
         <v>5.692</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0.03607783384584436</v>
+        <v>0.035575</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>45996</v>
+        <v>46087</v>
       </c>
       <c r="J38" s="8" t="n">
         <v>0.05018450184501849</v>
@@ -6692,7 +6622,7 @@
         <v>1.72</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.06450402928726036</v>
+        <v>0.0649056603773585</v>
       </c>
       <c r="I39" s="10" t="n">
         <v>46045</v>
@@ -6745,7 +6675,7 @@
         <v>3.16</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.0346111708036702</v>
+        <v>0.03556355726313094</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>45994</v>
@@ -6798,7 +6728,7 @@
         <v>4.228</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0.02760692241919218</v>
+        <v>0.02742783112167496</v>
       </c>
       <c r="I41" s="10" t="n">
         <v>46045</v>
@@ -6851,7 +6781,7 @@
         <v>2.1</v>
       </c>
       <c r="H42" s="18" t="n">
-        <v>0.03963385818268213</v>
+        <v>0.03995053847357968</v>
       </c>
       <c r="I42" s="19" t="n">
         <v>46013</v>
@@ -6904,7 +6834,7 @@
         <v>5.08</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0.03100775159142471</v>
+        <v>0.03071620865694696</v>
       </c>
       <c r="I43" s="10" t="n">
         <v>46076</v>
@@ -6957,7 +6887,7 @@
         <v>3.72</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.01803942519245617</v>
+        <v>0.01847529122044088</v>
       </c>
       <c r="I44" s="10" t="n">
         <v>46070</v>
@@ -6980,7 +6910,7 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>RHI</t>
+          <t>SNA</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
@@ -7000,29 +6930,29 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Nov</t>
         </is>
       </c>
       <c r="F45" s="7" t="n">
-        <v>0.59</v>
+        <v>2.44</v>
       </c>
       <c r="G45" s="24" t="n">
-        <v>2.36</v>
+        <v>9.76</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>0.09570154154918477</v>
+        <v>0.02662955919332545</v>
       </c>
       <c r="I45" s="10" t="n">
-        <v>46078</v>
+        <v>46077</v>
       </c>
       <c r="J45" s="8" t="n">
-        <v>0.1132075471698112</v>
+        <v>0.1401869158878504</v>
       </c>
       <c r="K45" s="10" t="n">
-        <v>46431</v>
+        <v>46332</v>
       </c>
       <c r="L45" s="10" t="n">
-        <v>46442</v>
+        <v>46346</v>
       </c>
       <c r="M45" s="12" t="inlineStr">
         <is>
@@ -7033,7 +6963,7 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>SNA</t>
+          <t>SWK</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
@@ -7048,34 +6978,34 @@
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>Feb/May/Aug/Nov</t>
+          <t>Mar/Jun/Sep/Nov</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>Nov</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="F46" s="7" t="n">
-        <v>2.44</v>
+        <v>0.83</v>
       </c>
       <c r="G46" s="24" t="n">
-        <v>9.76</v>
+        <v>3.32</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.02614869390488948</v>
+        <v>0.04586268860329277</v>
       </c>
       <c r="I46" s="10" t="n">
-        <v>46077</v>
+        <v>45992</v>
       </c>
       <c r="J46" s="8" t="n">
-        <v>0.1401869158878504</v>
+        <v>0.01219512195121952</v>
       </c>
       <c r="K46" s="10" t="n">
-        <v>46332</v>
+        <v>46227</v>
       </c>
       <c r="L46" s="10" t="n">
-        <v>46346</v>
+        <v>46267</v>
       </c>
       <c r="M46" s="12" t="inlineStr">
         <is>
@@ -7086,7 +7016,7 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>SWK</t>
+          <t>TROW</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
@@ -7101,34 +7031,34 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Mar/Jun/Sep/Nov</t>
+          <t>Mar/Jun/Sep/Dec</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="F47" s="7" t="n">
-        <v>0.83</v>
+        <v>1.27</v>
       </c>
       <c r="G47" s="24" t="n">
-        <v>3.32</v>
+        <v>5.08</v>
       </c>
       <c r="H47" s="9" t="n">
-        <v>0.04412839732925053</v>
+        <v>0.05776665748201185</v>
       </c>
       <c r="I47" s="10" t="n">
-        <v>45992</v>
+        <v>46006</v>
       </c>
       <c r="J47" s="8" t="n">
-        <v>0.01219512195121952</v>
+        <v>0.02419354838709679</v>
       </c>
       <c r="K47" s="10" t="n">
-        <v>46227</v>
+        <v>46430</v>
       </c>
       <c r="L47" s="10" t="n">
-        <v>46267</v>
+        <v>46460</v>
       </c>
       <c r="M47" s="12" t="inlineStr">
         <is>
@@ -7139,7 +7069,7 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>TROW</t>
+          <t>TTE</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
@@ -7159,29 +7089,29 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="F48" s="7" t="n">
-        <v>1.27</v>
+        <v>0.994</v>
       </c>
       <c r="G48" s="24" t="n">
-        <v>5.08</v>
+        <v>3.976</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>0.05657330701696998</v>
+        <v>0.04996858131518413</v>
       </c>
       <c r="I48" s="10" t="n">
-        <v>46006</v>
+        <v>45930</v>
       </c>
       <c r="J48" s="8" t="n">
-        <v>0.02419354838709679</v>
+        <v>0.2021660649819495</v>
       </c>
       <c r="K48" s="10" t="n">
-        <v>46430</v>
+        <v>46141</v>
       </c>
       <c r="L48" s="10" t="n">
-        <v>46460</v>
+        <v>46191</v>
       </c>
       <c r="M48" s="12" t="inlineStr">
         <is>
@@ -7192,7 +7122,7 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
@@ -7207,34 +7137,34 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Mar/Jun/Sep/Dec</t>
+          <t>Jan/May/Jul/Oct</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Oct</t>
         </is>
       </c>
       <c r="F49" s="7" t="n">
-        <v>0.994</v>
+        <v>1.42</v>
       </c>
       <c r="G49" s="24" t="n">
-        <v>3.976</v>
+        <v>5.68</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.05029091984291129</v>
+        <v>0.02961572656987358</v>
       </c>
       <c r="I49" s="10" t="n">
-        <v>45930</v>
+        <v>45961</v>
       </c>
       <c r="J49" s="8" t="n">
-        <v>0.2021660649819495</v>
+        <v>0.0441176470588234</v>
       </c>
       <c r="K49" s="10" t="n">
-        <v>46141</v>
+        <v>46285</v>
       </c>
       <c r="L49" s="10" t="n">
-        <v>46191</v>
+        <v>46325</v>
       </c>
       <c r="M49" s="12" t="inlineStr">
         <is>
@@ -7245,7 +7175,7 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>UL</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
@@ -7260,34 +7190,34 @@
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Jan/May/Jul/Oct</t>
+          <t>Feb/May/Aug/Nov</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Oct</t>
+          <t>Aug</t>
         </is>
       </c>
       <c r="F50" s="7" t="n">
-        <v>1.42</v>
+        <v>0.555</v>
       </c>
       <c r="G50" s="24" t="n">
-        <v>5.68</v>
+        <v>2.22</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.02941633490976144</v>
+        <v>0.03373347640718918</v>
       </c>
       <c r="I50" s="10" t="n">
-        <v>45961</v>
+        <v>46080</v>
       </c>
       <c r="J50" s="8" t="n">
-        <v>0.0441176470588234</v>
+        <v>0.005735494868956323</v>
       </c>
       <c r="K50" s="10" t="n">
-        <v>46285</v>
+        <v>46433</v>
       </c>
       <c r="L50" s="10" t="n">
-        <v>46325</v>
+        <v>46243</v>
       </c>
       <c r="M50" s="12" t="inlineStr">
         <is>
@@ -7298,7 +7228,7 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>UL</t>
+          <t>UNP</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
@@ -7313,7 +7243,7 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Feb/May/Aug/Nov</t>
+          <t>Feb/May/Aug/Dec</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
@@ -7322,25 +7252,25 @@
         </is>
       </c>
       <c r="F51" s="7" t="n">
-        <v>0.555</v>
+        <v>1.38</v>
       </c>
       <c r="G51" s="24" t="n">
-        <v>2.22</v>
+        <v>5.52</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.03333834092339166</v>
+        <v>0.02209016195988108</v>
       </c>
       <c r="I51" s="10" t="n">
         <v>46080</v>
       </c>
       <c r="J51" s="8" t="n">
-        <v>0.005735494868956323</v>
+        <v>0.02985074626865658</v>
       </c>
       <c r="K51" s="10" t="n">
-        <v>46433</v>
+        <v>46220</v>
       </c>
       <c r="L51" s="10" t="n">
-        <v>46243</v>
+        <v>46264</v>
       </c>
       <c r="M51" s="12" t="inlineStr">
         <is>
@@ -7351,7 +7281,7 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>UNP</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -7366,34 +7296,34 @@
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Feb/May/Aug/Dec</t>
+          <t>Feb/May/Aug/Nov</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Aug</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="F52" s="7" t="n">
-        <v>1.38</v>
+        <v>1.64</v>
       </c>
       <c r="G52" s="24" t="n">
-        <v>5.52</v>
+        <v>6.56</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.02161061800994751</v>
+        <v>0.06718558010043858</v>
       </c>
       <c r="I52" s="10" t="n">
-        <v>46080</v>
+        <v>46070</v>
       </c>
       <c r="J52" s="8" t="n">
-        <v>0.02985074626865658</v>
+        <v>0.00613496932515338</v>
       </c>
       <c r="K52" s="10" t="n">
-        <v>46220</v>
+        <v>46423</v>
       </c>
       <c r="L52" s="10" t="n">
-        <v>46264</v>
+        <v>46435</v>
       </c>
       <c r="M52" s="12" t="inlineStr">
         <is>
@@ -7404,7 +7334,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>VZ</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -7419,34 +7349,34 @@
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Feb/May/Aug/Nov</t>
+          <t>Jan/Apr/Jul/Oct</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Oct</t>
         </is>
       </c>
       <c r="F53" s="7" t="n">
-        <v>1.64</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G53" s="24" t="n">
-        <v>6.56</v>
+        <v>2.76</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>0.06470066120416362</v>
+        <v>0.05419734985467445</v>
       </c>
       <c r="I53" s="10" t="n">
-        <v>46070</v>
+        <v>46034</v>
       </c>
       <c r="J53" s="8" t="n">
-        <v>0.00613496932515338</v>
+        <v>0.01769911504424764</v>
       </c>
       <c r="K53" s="10" t="n">
-        <v>46423</v>
+        <v>46267</v>
       </c>
       <c r="L53" s="10" t="n">
-        <v>46435</v>
+        <v>46303</v>
       </c>
       <c r="M53" s="12" t="inlineStr">
         <is>
@@ -7457,7 +7387,7 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>VZ</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -7472,89 +7402,36 @@
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Jan/Apr/Jul/Oct</t>
+          <t>Feb/May/Aug/Nov</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Oct</t>
+          <t>Nov</t>
         </is>
       </c>
       <c r="F54" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.03</v>
       </c>
       <c r="G54" s="24" t="n">
-        <v>2.76</v>
+        <v>4.12</v>
       </c>
       <c r="H54" s="9" t="n">
-        <v>0.05433605865719647</v>
+        <v>0.02687365511453597</v>
       </c>
       <c r="I54" s="10" t="n">
-        <v>46034</v>
+        <v>46065</v>
       </c>
       <c r="J54" s="8" t="n">
-        <v>0.01769911504424764</v>
+        <v>0.04040404040404044</v>
       </c>
       <c r="K54" s="10" t="n">
-        <v>46267</v>
+        <v>46341</v>
       </c>
       <c r="L54" s="10" t="n">
-        <v>46303</v>
+        <v>46339</v>
       </c>
       <c r="M54" s="12" t="inlineStr">
-        <is>
-          <t>Notion + yfinance</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>XOM</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>Quality Dividend</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>Feb/May/Aug/Nov</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>Nov</t>
-        </is>
-      </c>
-      <c r="F55" s="7" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="G55" s="24" t="n">
-        <v>4.12</v>
-      </c>
-      <c r="H55" s="9" t="n">
-        <v>0.02711775290341838</v>
-      </c>
-      <c r="I55" s="10" t="n">
-        <v>46065</v>
-      </c>
-      <c r="J55" s="8" t="n">
-        <v>0.04040404040404044</v>
-      </c>
-      <c r="K55" s="10" t="n">
-        <v>46341</v>
-      </c>
-      <c r="L55" s="10" t="n">
-        <v>46339</v>
-      </c>
-      <c r="M55" s="12" t="inlineStr">
         <is>
           <t>Notion + yfinance</t>
         </is>
@@ -7563,252 +7440,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
-    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
-    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
-                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
-                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54D7E5A6-E20A-4DF3-BFF2-95F97C57AE72}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF21B2D4-F516-4342-87AE-293F72731B69}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59FB35DC-1CBC-48BE-AD11-52F29A542886}"/>
 </file>
</xml_diff>

<commit_message>
Clear pycache, force fresh module load
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -7510,4 +7510,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{161435CF-554B-4E9C-8EF7-D306330B17B9}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94120F72-60DA-490F-BAAC-86AA11994D08}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8340C35D-F94E-472C-A02F-046046F1B44A}"/>
 </file>
</xml_diff>

<commit_message>
Update dividend calendar 2026-03-30
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="167" formatCode="MM/DD/YYYY"/>
     <numFmt numFmtId="168" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,6 +72,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00856404"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="00666666"/>
       <sz val="9"/>
     </font>
@@ -88,7 +94,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -98,6 +104,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001a3a5c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
     <fill>
@@ -123,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -131,16 +142,19 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,10 +164,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -547,7 +561,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estimated Dividend Calendar: Anticipated Announcements - 03/23/2026</t>
+          <t>Estimated Dividend Calendar: Anticipated Announcements - 03/30/2026</t>
         </is>
       </c>
     </row>
@@ -652,7 +666,7 @@
         <v>46122</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>46132</v>
@@ -663,7 +677,7 @@
         </is>
       </c>
       <c r="L6" s="9" t="n">
-        <v>0.0291535954348521</v>
+        <v>0.02939990314843966</v>
       </c>
     </row>
     <row r="7">
@@ -697,8 +711,8 @@
       <c r="H7" s="10" t="n">
         <v>46127</v>
       </c>
-      <c r="I7" s="11" t="n">
-        <v>23</v>
+      <c r="I7" s="13" t="n">
+        <v>16</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>46503</v>
@@ -709,7 +723,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.02049343832020997</v>
+        <v>0.02049244854572341</v>
       </c>
     </row>
     <row r="8">
@@ -743,8 +757,8 @@
       <c r="H8" s="10" t="n">
         <v>46128</v>
       </c>
-      <c r="I8" s="11" t="n">
-        <v>24</v>
+      <c r="I8" s="13" t="n">
+        <v>17</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>46165</v>
@@ -755,7 +769,7 @@
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.02203016500553975</v>
+        <v>0.02150270835143434</v>
       </c>
     </row>
     <row r="9">
@@ -789,8 +803,8 @@
       <c r="H9" s="10" t="n">
         <v>46134</v>
       </c>
-      <c r="I9" s="11" t="n">
-        <v>30</v>
+      <c r="I9" s="13" t="n">
+        <v>23</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>46161</v>
@@ -801,7 +815,7 @@
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>0.02895742012250174</v>
+        <v>0.02688399565783459</v>
       </c>
     </row>
     <row r="10">
@@ -835,8 +849,8 @@
       <c r="H10" s="10" t="n">
         <v>46140</v>
       </c>
-      <c r="I10" s="11" t="n">
-        <v>36</v>
+      <c r="I10" s="13" t="n">
+        <v>29</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>46190</v>
@@ -847,7 +861,7 @@
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.04551803170526622</v>
+        <v>0.0429535990399483</v>
       </c>
     </row>
     <row r="11">
@@ -881,8 +895,8 @@
       <c r="H11" s="10" t="n">
         <v>46143</v>
       </c>
-      <c r="I11" s="11" t="n">
-        <v>39</v>
+      <c r="I11" s="13" t="n">
+        <v>32</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46152</v>
@@ -893,7 +907,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.04596967353172818</v>
+        <v>0.04682926829268293</v>
       </c>
     </row>
     <row r="12">
@@ -927,8 +941,8 @@
       <c r="H12" s="10" t="n">
         <v>46162</v>
       </c>
-      <c r="I12" s="11" t="n">
-        <v>58</v>
+      <c r="I12" s="13" t="n">
+        <v>51</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>46198</v>
@@ -939,53 +953,53 @@
         </is>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0.03268124223397447</v>
+        <v>0.03263617685080991</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>POR</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="16" t="n">
         <v>0.525</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="F13" s="16" t="n">
+      <c r="F13" s="17" t="n">
         <v>0.05000000000000004</v>
       </c>
-      <c r="G13" s="17" t="n">
+      <c r="G13" s="18" t="n">
         <v>0.04</v>
       </c>
-      <c r="H13" s="18" t="n">
+      <c r="H13" s="19" t="n">
         <v>46176</v>
       </c>
-      <c r="I13" s="19" t="n">
-        <v>72</v>
-      </c>
-      <c r="J13" s="18" t="n">
+      <c r="I13" s="20" t="n">
+        <v>65</v>
+      </c>
+      <c r="J13" s="19" t="n">
         <v>46197</v>
       </c>
-      <c r="K13" s="20" t="inlineStr">
+      <c r="K13" s="21" t="inlineStr">
         <is>
           <t>yfinance</t>
         </is>
       </c>
-      <c r="L13" s="17" t="n">
-        <v>0.04154713772034981</v>
+      <c r="L13" s="18" t="n">
+        <v>0.0402723172224527</v>
       </c>
     </row>
     <row r="14">
@@ -1019,8 +1033,8 @@
       <c r="H14" s="10" t="n">
         <v>46218</v>
       </c>
-      <c r="I14" s="11" t="n">
-        <v>114</v>
+      <c r="I14" s="13" t="n">
+        <v>107</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>46248</v>
@@ -1031,7 +1045,7 @@
         </is>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.01846291281599689</v>
+        <v>0.01864755074222239</v>
       </c>
     </row>
     <row r="15">
@@ -1065,8 +1079,8 @@
       <c r="H15" s="10" t="n">
         <v>46218</v>
       </c>
-      <c r="I15" s="11" t="n">
-        <v>114</v>
+      <c r="I15" s="13" t="n">
+        <v>107</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>46248</v>
@@ -1077,7 +1091,7 @@
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>0.01846291281599689</v>
+        <v>0.01864755074222239</v>
       </c>
     </row>
     <row r="16">
@@ -1111,8 +1125,8 @@
       <c r="H16" s="10" t="n">
         <v>46220</v>
       </c>
-      <c r="I16" s="11" t="n">
-        <v>116</v>
+      <c r="I16" s="13" t="n">
+        <v>109</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>46264</v>
@@ -1123,7 +1137,7 @@
         </is>
       </c>
       <c r="L16" s="9" t="n">
-        <v>0.02307065393635178</v>
+        <v>0.02292834890965732</v>
       </c>
     </row>
     <row r="17">
@@ -1157,8 +1171,8 @@
       <c r="H17" s="10" t="n">
         <v>46227</v>
       </c>
-      <c r="I17" s="11" t="n">
-        <v>123</v>
+      <c r="I17" s="13" t="n">
+        <v>116</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>46267</v>
@@ -1169,7 +1183,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.04739810245968331</v>
+        <v>0.04879482591603472</v>
       </c>
     </row>
     <row r="18">
@@ -1203,8 +1217,8 @@
       <c r="H18" s="10" t="n">
         <v>46232</v>
       </c>
-      <c r="I18" s="11" t="n">
-        <v>128</v>
+      <c r="I18" s="13" t="n">
+        <v>121</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>46264</v>
@@ -1215,7 +1229,7 @@
         </is>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.03003454137242492</v>
+        <v>0.02967138990015516</v>
       </c>
     </row>
     <row r="19">
@@ -1249,8 +1263,8 @@
       <c r="H19" s="10" t="n">
         <v>46232</v>
       </c>
-      <c r="I19" s="11" t="n">
-        <v>128</v>
+      <c r="I19" s="13" t="n">
+        <v>121</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>46246</v>
@@ -1261,7 +1275,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0.04611808330319646</v>
+        <v>0.04900701556039189</v>
       </c>
     </row>
     <row r="20">
@@ -1295,8 +1309,8 @@
       <c r="H20" s="10" t="n">
         <v>46263</v>
       </c>
-      <c r="I20" s="11" t="n">
-        <v>159</v>
+      <c r="I20" s="13" t="n">
+        <v>152</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>46297</v>
@@ -1307,7 +1321,7 @@
         </is>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0.02994613381315931</v>
+        <v>0.02918668873610638</v>
       </c>
     </row>
     <row r="21">
@@ -1341,8 +1355,8 @@
       <c r="H21" s="10" t="n">
         <v>46267</v>
       </c>
-      <c r="I21" s="11" t="n">
-        <v>163</v>
+      <c r="I21" s="13" t="n">
+        <v>156</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46303</v>
@@ -1353,7 +1367,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.0552</v>
+        <v>0.05448429504518887</v>
       </c>
     </row>
     <row r="22">
@@ -1387,8 +1401,8 @@
       <c r="H22" s="10" t="n">
         <v>46278</v>
       </c>
-      <c r="I22" s="11" t="n">
-        <v>174</v>
+      <c r="I22" s="13" t="n">
+        <v>167</v>
       </c>
       <c r="J22" s="10" t="n">
         <v>46344</v>
@@ -1399,7 +1413,7 @@
         </is>
       </c>
       <c r="L22" s="9" t="n">
-        <v>0.009441793172158741</v>
+        <v>0.01011349878049246</v>
       </c>
     </row>
     <row r="23">
@@ -1433,8 +1447,8 @@
       <c r="H23" s="10" t="n">
         <v>46285</v>
       </c>
-      <c r="I23" s="11" t="n">
-        <v>181</v>
+      <c r="I23" s="13" t="n">
+        <v>174</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>46325</v>
@@ -1445,7 +1459,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0.0297506811988012</v>
+        <v>0.02987833617940912</v>
       </c>
     </row>
     <row r="24">
@@ -1479,8 +1493,8 @@
       <c r="H24" s="10" t="n">
         <v>46305</v>
       </c>
-      <c r="I24" s="11" t="n">
-        <v>201</v>
+      <c r="I24" s="13" t="n">
+        <v>194</v>
       </c>
       <c r="J24" s="10" t="n">
         <v>46339</v>
@@ -1491,7 +1505,7 @@
         </is>
       </c>
       <c r="L24" s="9" t="n">
-        <v>0.04068272109836166</v>
+        <v>0.03850409499617897</v>
       </c>
     </row>
     <row r="25">
@@ -1525,8 +1539,8 @@
       <c r="H25" s="10" t="n">
         <v>46311</v>
       </c>
-      <c r="I25" s="11" t="n">
-        <v>207</v>
+      <c r="I25" s="13" t="n">
+        <v>200</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>46386</v>
@@ -1537,7 +1551,7 @@
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>0.01230577473752138</v>
+        <v>0.01275659546945501</v>
       </c>
     </row>
     <row r="26">
@@ -1571,8 +1585,8 @@
       <c r="H26" s="10" t="n">
         <v>46317</v>
       </c>
-      <c r="I26" s="11" t="n">
-        <v>213</v>
+      <c r="I26" s="13" t="n">
+        <v>206</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>46351</v>
@@ -1583,7 +1597,7 @@
         </is>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0.01366336633663366</v>
+        <v>0.0146463000754747</v>
       </c>
     </row>
     <row r="27">
@@ -1617,8 +1631,8 @@
       <c r="H27" s="10" t="n">
         <v>46322</v>
       </c>
-      <c r="I27" s="11" t="n">
-        <v>218</v>
+      <c r="I27" s="13" t="n">
+        <v>211</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>46338</v>
@@ -1629,7 +1643,7 @@
         </is>
       </c>
       <c r="L27" s="9" t="n">
-        <v>0.02537542692959548</v>
+        <v>0.02327378459090542</v>
       </c>
     </row>
     <row r="28">
@@ -1663,8 +1677,8 @@
       <c r="H28" s="10" t="n">
         <v>46329</v>
       </c>
-      <c r="I28" s="11" t="n">
-        <v>225</v>
+      <c r="I28" s="13" t="n">
+        <v>218</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>46338</v>
@@ -1675,7 +1689,7 @@
         </is>
       </c>
       <c r="L28" s="9" t="n">
-        <v>0.007356208990148843</v>
+        <v>0.007635530491459991</v>
       </c>
     </row>
     <row r="29">
@@ -1709,8 +1723,8 @@
       <c r="H29" s="10" t="n">
         <v>46332</v>
       </c>
-      <c r="I29" s="11" t="n">
-        <v>228</v>
+      <c r="I29" s="13" t="n">
+        <v>221</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>46346</v>
@@ -1721,7 +1735,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>0.0268223978014428</v>
+        <v>0.02719988759972165</v>
       </c>
     </row>
     <row r="30">
@@ -1755,8 +1769,8 @@
       <c r="H30" s="10" t="n">
         <v>46341</v>
       </c>
-      <c r="I30" s="11" t="n">
-        <v>237</v>
+      <c r="I30" s="13" t="n">
+        <v>230</v>
       </c>
       <c r="J30" s="10" t="n">
         <v>46339</v>
@@ -1767,7 +1781,7 @@
         </is>
       </c>
       <c r="L30" s="9" t="n">
-        <v>0.02607182508545984</v>
+        <v>0.02356574933849925</v>
       </c>
     </row>
     <row r="31">
@@ -1801,8 +1815,8 @@
       <c r="H31" s="10" t="n">
         <v>46344</v>
       </c>
-      <c r="I31" s="11" t="n">
-        <v>240</v>
+      <c r="I31" s="13" t="n">
+        <v>233</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>46385</v>
@@ -1813,7 +1827,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="n">
-        <v>0.0359617910086034</v>
+        <v>0.0361990943977892</v>
       </c>
     </row>
     <row r="32">
@@ -1847,8 +1861,8 @@
       <c r="H32" s="10" t="n">
         <v>46347</v>
       </c>
-      <c r="I32" s="11" t="n">
-        <v>243</v>
+      <c r="I32" s="13" t="n">
+        <v>236</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>46358</v>
@@ -1859,7 +1873,7 @@
         </is>
       </c>
       <c r="L32" s="9" t="n">
-        <v>0.03073463233210399</v>
+        <v>0.03174603183979984</v>
       </c>
     </row>
     <row r="33">
@@ -1893,8 +1907,8 @@
       <c r="H33" s="10" t="n">
         <v>46352</v>
       </c>
-      <c r="I33" s="11" t="n">
-        <v>248</v>
+      <c r="I33" s="13" t="n">
+        <v>241</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>46400</v>
@@ -1905,7 +1919,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>0.05265049361856506</v>
+        <v>0.05067012721677747</v>
       </c>
     </row>
     <row r="34">
@@ -1939,8 +1953,8 @@
       <c r="H34" s="10" t="n">
         <v>46360</v>
       </c>
-      <c r="I34" s="11" t="n">
-        <v>256</v>
+      <c r="I34" s="13" t="n">
+        <v>249</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>46371</v>
@@ -1951,7 +1965,7 @@
         </is>
       </c>
       <c r="L34" s="9" t="n">
-        <v>0.04986272751327035</v>
+        <v>0.04632565912794535</v>
       </c>
     </row>
     <row r="35">
@@ -1985,8 +1999,8 @@
       <c r="H35" s="10" t="n">
         <v>46366</v>
       </c>
-      <c r="I35" s="11" t="n">
-        <v>262</v>
+      <c r="I35" s="13" t="n">
+        <v>255</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>46432</v>
@@ -1997,7 +2011,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0.02869097539422992</v>
+        <v>0.02867628152814483</v>
       </c>
     </row>
     <row r="36">
@@ -2031,8 +2045,8 @@
       <c r="H36" s="10" t="n">
         <v>46370</v>
       </c>
-      <c r="I36" s="11" t="n">
-        <v>266</v>
+      <c r="I36" s="13" t="n">
+        <v>259</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>46413</v>
@@ -2043,7 +2057,7 @@
         </is>
       </c>
       <c r="L36" s="9" t="n">
-        <v>0.06394052135283915</v>
+        <v>0.06281177656172118</v>
       </c>
     </row>
     <row r="37">
@@ -2077,8 +2091,8 @@
       <c r="H37" s="10" t="n">
         <v>46371</v>
       </c>
-      <c r="I37" s="11" t="n">
-        <v>267</v>
+      <c r="I37" s="13" t="n">
+        <v>260</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>46344</v>
@@ -2089,7 +2103,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>0.02188391959954028</v>
+        <v>0.0214252452124615</v>
       </c>
     </row>
     <row r="38">
@@ -2123,8 +2137,8 @@
       <c r="H38" s="10" t="n">
         <v>46411</v>
       </c>
-      <c r="I38" s="11" t="n">
-        <v>307</v>
+      <c r="I38" s="13" t="n">
+        <v>300</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>46435</v>
@@ -2135,7 +2149,7 @@
         </is>
       </c>
       <c r="L38" s="9" t="n">
-        <v>0.04124678949944683</v>
+        <v>0.040594776039757</v>
       </c>
     </row>
     <row r="39">
@@ -2169,8 +2183,8 @@
       <c r="H39" s="10" t="n">
         <v>46416</v>
       </c>
-      <c r="I39" s="11" t="n">
-        <v>312</v>
+      <c r="I39" s="13" t="n">
+        <v>305</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>46483</v>
@@ -2181,7 +2195,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.01629162014983631</v>
+        <v>0.01634988749254875</v>
       </c>
     </row>
     <row r="40">
@@ -2215,8 +2229,8 @@
       <c r="H40" s="10" t="n">
         <v>46417</v>
       </c>
-      <c r="I40" s="11" t="n">
-        <v>313</v>
+      <c r="I40" s="13" t="n">
+        <v>306</v>
       </c>
       <c r="J40" s="10" t="n">
         <v>46433</v>
@@ -2227,7 +2241,7 @@
         </is>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.03538327635252886</v>
+        <v>0.03326092504050905</v>
       </c>
     </row>
     <row r="41">
@@ -2261,8 +2275,8 @@
       <c r="H41" s="10" t="n">
         <v>46419</v>
       </c>
-      <c r="I41" s="11" t="n">
-        <v>315</v>
+      <c r="I41" s="13" t="n">
+        <v>308</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>46472</v>
@@ -2273,7 +2287,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>0.03161028351510873</v>
+        <v>0.03309719381407237</v>
       </c>
     </row>
     <row r="42">
@@ -2307,8 +2321,8 @@
       <c r="H42" s="10" t="n">
         <v>46423</v>
       </c>
-      <c r="I42" s="11" t="n">
-        <v>319</v>
+      <c r="I42" s="13" t="n">
+        <v>312</v>
       </c>
       <c r="J42" s="10" t="n">
         <v>46435</v>
@@ -2319,7 +2333,7 @@
         </is>
       </c>
       <c r="L42" s="9" t="n">
-        <v>0.06706880854454768</v>
+        <v>0.06847598946793178</v>
       </c>
     </row>
     <row r="43">
@@ -2353,8 +2367,8 @@
       <c r="H43" s="10" t="n">
         <v>46428</v>
       </c>
-      <c r="I43" s="11" t="n">
-        <v>324</v>
+      <c r="I43" s="13" t="n">
+        <v>317</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>46452</v>
@@ -2365,7 +2379,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>0.01475211662660081</v>
+        <v>0.01577348219982237</v>
       </c>
     </row>
     <row r="44">
@@ -2399,8 +2413,8 @@
       <c r="H44" s="10" t="n">
         <v>46428</v>
       </c>
-      <c r="I44" s="11" t="n">
-        <v>324</v>
+      <c r="I44" s="13" t="n">
+        <v>317</v>
       </c>
       <c r="J44" s="10" t="n">
         <v>46460</v>
@@ -2411,45 +2425,45 @@
         </is>
       </c>
       <c r="L44" s="9" t="n">
-        <v>0.05940820373037564</v>
+        <v>0.0581557898200166</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>Semi-Annual</t>
+          <t>Quarterly</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="D45" s="7" t="n">
-        <v>1.883</v>
+        <v>0.41</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>1.864</v>
+        <v>0.4</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>0.01019313304721025</v>
+        <v>0.02499999999999988</v>
       </c>
       <c r="G45" s="9" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="H45" s="10" t="n">
-        <v>46433</v>
-      </c>
-      <c r="I45" s="11" t="n">
-        <v>329</v>
+        <v>46432</v>
+      </c>
+      <c r="I45" s="13" t="n">
+        <v>321</v>
       </c>
       <c r="J45" s="10" t="n">
-        <v>46425</v>
+        <v>46481</v>
       </c>
       <c r="K45" s="12" t="inlineStr">
         <is>
@@ -2457,45 +2471,45 @@
         </is>
       </c>
       <c r="L45" s="9" t="n">
-        <v>0.002723282372501188</v>
+        <v>0.02077527171622906</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Quarterly</t>
+          <t>Semi-Annual</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Dec</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="D46" s="7" t="n">
-        <v>7.45</v>
+        <v>1.883</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>1.25</v>
+        <v>1.864</v>
       </c>
       <c r="F46" s="8" t="n">
-        <v>4.96</v>
+        <v>0.01019313304721025</v>
       </c>
       <c r="G46" s="9" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="H46" s="10" t="n">
         <v>46433</v>
       </c>
-      <c r="I46" s="11" t="n">
-        <v>329</v>
+      <c r="I46" s="13" t="n">
+        <v>322</v>
       </c>
       <c r="J46" s="10" t="n">
-        <v>46383</v>
+        <v>46425</v>
       </c>
       <c r="K46" s="12" t="inlineStr">
         <is>
@@ -2503,13 +2517,13 @@
         </is>
       </c>
       <c r="L46" s="9" t="n">
-        <v>0.09735221224892325</v>
+        <v>0.00296196100543417</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>DVN</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
@@ -2519,17 +2533,17 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>Dec</t>
         </is>
       </c>
       <c r="D47" s="7" t="n">
-        <v>0.24</v>
+        <v>7.45</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>0.22</v>
+        <v>1.25</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>0.09090909090909087</v>
+        <v>4.96</v>
       </c>
       <c r="G47" s="9" t="n">
         <v>0.06</v>
@@ -2537,11 +2551,11 @@
       <c r="H47" s="10" t="n">
         <v>46433</v>
       </c>
-      <c r="I47" s="11" t="n">
-        <v>329</v>
+      <c r="I47" s="13" t="n">
+        <v>322</v>
       </c>
       <c r="J47" s="10" t="n">
-        <v>46276</v>
+        <v>46383</v>
       </c>
       <c r="K47" s="12" t="inlineStr">
         <is>
@@ -2549,13 +2563,13 @@
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>0.02006479204737895</v>
+        <v>0.1007675883168235</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>DVN</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
@@ -2565,17 +2579,17 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="D48" s="7" t="n">
-        <v>1.423</v>
+        <v>0.24</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>1.355</v>
+        <v>0.22</v>
       </c>
       <c r="F48" s="8" t="n">
-        <v>0.05018450184501849</v>
+        <v>0.09090909090909087</v>
       </c>
       <c r="G48" s="9" t="n">
         <v>0.06</v>
@@ -2583,11 +2597,11 @@
       <c r="H48" s="10" t="n">
         <v>46433</v>
       </c>
-      <c r="I48" s="11" t="n">
-        <v>329</v>
+      <c r="I48" s="13" t="n">
+        <v>322</v>
       </c>
       <c r="J48" s="10" t="n">
-        <v>46177</v>
+        <v>46276</v>
       </c>
       <c r="K48" s="12" t="inlineStr">
         <is>
@@ -2595,13 +2609,13 @@
         </is>
       </c>
       <c r="L48" s="9" t="n">
-        <v>0.03783686339934728</v>
+        <v>0.01829616881390908</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>PFG</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
@@ -2611,29 +2625,29 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="D49" s="7" t="n">
-        <v>0.8</v>
+        <v>1.423</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>0.79</v>
+        <v>1.355</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>0.01265822784810128</v>
+        <v>0.05018450184501849</v>
       </c>
       <c r="G49" s="9" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="H49" s="10" t="n">
         <v>46433</v>
       </c>
-      <c r="I49" s="11" t="n">
-        <v>329</v>
+      <c r="I49" s="13" t="n">
+        <v>322</v>
       </c>
       <c r="J49" s="10" t="n">
-        <v>46270</v>
+        <v>46177</v>
       </c>
       <c r="K49" s="12" t="inlineStr">
         <is>
@@ -2641,13 +2655,13 @@
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>0.03720497524150213</v>
+        <v>0.03653519090405939</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>UL</t>
+          <t>PFG</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
@@ -2657,29 +2671,29 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Aug</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="D50" s="7" t="n">
-        <v>0.555</v>
+        <v>0.8</v>
       </c>
       <c r="E50" s="7" t="n">
-        <v>0.588964</v>
+        <v>0.79</v>
       </c>
       <c r="F50" s="8" t="n">
-        <v>0.005735494868956323</v>
+        <v>0.01265822784810128</v>
       </c>
       <c r="G50" s="9" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="H50" s="10" t="n">
         <v>46433</v>
       </c>
-      <c r="I50" s="11" t="n">
-        <v>329</v>
+      <c r="I50" s="13" t="n">
+        <v>322</v>
       </c>
       <c r="J50" s="10" t="n">
-        <v>46243</v>
+        <v>46270</v>
       </c>
       <c r="K50" s="12" t="inlineStr">
         <is>
@@ -2687,13 +2701,13 @@
         </is>
       </c>
       <c r="L50" s="9" t="n">
-        <v>0.03599513623773182</v>
+        <v>0.03650051405080914</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>ALSN</t>
+          <t>UL</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
@@ -2703,29 +2717,29 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Aug</t>
         </is>
       </c>
       <c r="D51" s="7" t="n">
-        <v>0.29</v>
+        <v>0.555</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>0.27</v>
+        <v>0.588964</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>0.07407407407407393</v>
+        <v>0.005735494868956323</v>
       </c>
       <c r="G51" s="9" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="H51" s="10" t="n">
-        <v>46440</v>
-      </c>
-      <c r="I51" s="11" t="n">
-        <v>336</v>
+        <v>46433</v>
+      </c>
+      <c r="I51" s="13" t="n">
+        <v>322</v>
       </c>
       <c r="J51" s="10" t="n">
-        <v>46450</v>
+        <v>46243</v>
       </c>
       <c r="K51" s="12" t="inlineStr">
         <is>
@@ -2733,13 +2747,13 @@
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>0.01011774953826027</v>
+        <v>0.03716103009083437</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>ALSN</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -2753,25 +2767,25 @@
         </is>
       </c>
       <c r="D52" s="7" t="n">
-        <v>2.33</v>
+        <v>0.29</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>2.3</v>
+        <v>0.27</v>
       </c>
       <c r="F52" s="8" t="n">
-        <v>0.01304347826086967</v>
+        <v>0.07407407407407393</v>
       </c>
       <c r="G52" s="9" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="H52" s="10" t="n">
-        <v>46441</v>
-      </c>
-      <c r="I52" s="11" t="n">
-        <v>337</v>
+        <v>46440</v>
+      </c>
+      <c r="I52" s="13" t="n">
+        <v>329</v>
       </c>
       <c r="J52" s="10" t="n">
-        <v>46456</v>
+        <v>46450</v>
       </c>
       <c r="K52" s="12" t="inlineStr">
         <is>
@@ -2779,13 +2793,13 @@
         </is>
       </c>
       <c r="L52" s="9" t="n">
-        <v>0.02796825186337326</v>
+        <v>0.01014074662286406</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>GD</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -2795,83 +2809,83 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
-        <v>1.5</v>
+        <v>2.33</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>1.42</v>
+        <v>2.3</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>0.05633802816901413</v>
+        <v>0.01304347826086967</v>
       </c>
       <c r="G53" s="9" t="n">
         <v>0.08</v>
       </c>
       <c r="H53" s="10" t="n">
+        <v>46441</v>
+      </c>
+      <c r="I53" s="13" t="n">
+        <v>330</v>
+      </c>
+      <c r="J53" s="10" t="n">
+        <v>46456</v>
+      </c>
+      <c r="K53" s="12" t="inlineStr">
+        <is>
+          <t>Notion + yfinance</t>
+        </is>
+      </c>
+      <c r="L53" s="9" t="n">
+        <v>0.02851809941441286</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>GD</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="F54" s="8" t="n">
+        <v>0.05633802816901413</v>
+      </c>
+      <c r="G54" s="9" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H54" s="10" t="n">
         <v>46451</v>
       </c>
-      <c r="I53" s="11" t="n">
-        <v>347</v>
-      </c>
-      <c r="J53" s="10" t="n">
+      <c r="I54" s="13" t="n">
+        <v>340</v>
+      </c>
+      <c r="J54" s="10" t="n">
         <v>46487</v>
       </c>
-      <c r="K53" s="12" t="inlineStr">
-        <is>
-          <t>Notion + yfinance</t>
-        </is>
-      </c>
-      <c r="L53" s="9" t="n">
-        <v>0.0174218562737619</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="13" t="inlineStr">
-        <is>
-          <t>CSCO</t>
-        </is>
-      </c>
-      <c r="B54" s="14" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="C54" s="14" t="inlineStr">
-        <is>
-          <t>Apr</t>
-        </is>
-      </c>
-      <c r="D54" s="15" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="E54" s="15" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F54" s="16" t="n">
-        <v>0.02499999999999988</v>
-      </c>
-      <c r="G54" s="17" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="H54" s="18" t="n">
-        <v>46460</v>
-      </c>
-      <c r="I54" s="19" t="n">
-        <v>356</v>
-      </c>
-      <c r="J54" s="18" t="n">
-        <v>46481</v>
-      </c>
-      <c r="K54" s="20" t="inlineStr">
-        <is>
-          <t>yfinance</t>
-        </is>
-      </c>
-      <c r="L54" s="17" t="n">
-        <v>0.02079898581784063</v>
+      <c r="K54" s="12" t="inlineStr">
+        <is>
+          <t>Notion + yfinance</t>
+        </is>
+      </c>
+      <c r="L54" s="9" t="n">
+        <v>0.01724782270450997</v>
       </c>
     </row>
     <row r="55">
@@ -2905,8 +2919,8 @@
       <c r="H55" s="10" t="n">
         <v>46461</v>
       </c>
-      <c r="I55" s="11" t="n">
-        <v>357</v>
+      <c r="I55" s="13" t="n">
+        <v>350</v>
       </c>
       <c r="J55" s="10" t="n">
         <v>46300</v>
@@ -2917,7 +2931,7 @@
         </is>
       </c>
       <c r="L55" s="9" t="n">
-        <v>0.02058107236004315</v>
+        <v>0.02104414080461985</v>
       </c>
     </row>
     <row r="56">
@@ -2951,8 +2965,8 @@
       <c r="H56" s="10" t="n">
         <v>46461</v>
       </c>
-      <c r="I56" s="11" t="n">
-        <v>357</v>
+      <c r="I56" s="13" t="n">
+        <v>350</v>
       </c>
       <c r="J56" s="10" t="n">
         <v>46196</v>
@@ -2963,7 +2977,7 @@
         </is>
       </c>
       <c r="L56" s="9" t="n">
-        <v>0.05314088789783094</v>
+        <v>0.05277732582200233</v>
       </c>
     </row>
   </sheetData>
@@ -2998,44 +3012,44 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Expected Increase Announcements by Month - 03/23/2026</t>
+          <t>Expected Increase Announcements by Month - 03/30/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>April 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C5" s="22" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D5" s="22" t="inlineStr">
+      <c r="D5" s="23" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E5" s="22" t="inlineStr">
+      <c r="E5" s="23" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F5" s="22" t="inlineStr">
+      <c r="F5" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3162,39 +3176,39 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>May 2026</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C13" s="22" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D13" s="22" t="inlineStr">
+      <c r="D13" s="23" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E13" s="22" t="inlineStr">
+      <c r="E13" s="23" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F13" s="22" t="inlineStr">
+      <c r="F13" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3249,102 +3263,102 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>June 2026</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B18" s="23" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C18" s="22" t="inlineStr">
+      <c r="C18" s="23" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D18" s="22" t="inlineStr">
+      <c r="D18" s="23" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E18" s="22" t="inlineStr">
+      <c r="E18" s="23" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F18" s="22" t="inlineStr">
+      <c r="F18" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>POR</t>
         </is>
       </c>
-      <c r="B19" s="18" t="n">
+      <c r="B19" s="19" t="n">
         <v>46176</v>
       </c>
-      <c r="C19" s="18" t="n">
+      <c r="C19" s="19" t="n">
         <v>46197</v>
       </c>
-      <c r="D19" s="15" t="n">
+      <c r="D19" s="16" t="n">
         <v>0.525</v>
       </c>
-      <c r="E19" s="16" t="n">
+      <c r="E19" s="17" t="n">
         <v>0.05000000000000004</v>
       </c>
-      <c r="F19" s="20" t="inlineStr">
+      <c r="F19" s="21" t="inlineStr">
         <is>
           <t>yfinance</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>July 2026</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B22" s="22" t="inlineStr">
+      <c r="B22" s="23" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C22" s="22" t="inlineStr">
+      <c r="C22" s="23" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D22" s="22" t="inlineStr">
+      <c r="D22" s="23" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr">
+      <c r="E22" s="23" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F22" s="22" t="inlineStr">
+      <c r="F22" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3495,39 +3509,39 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="inlineStr">
+      <c r="A30" s="22" t="inlineStr">
         <is>
           <t>August 2026</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="22" t="inlineStr">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B31" s="22" t="inlineStr">
+      <c r="B31" s="23" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C31" s="22" t="inlineStr">
+      <c r="C31" s="23" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D31" s="22" t="inlineStr">
+      <c r="D31" s="23" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E31" s="22" t="inlineStr">
+      <c r="E31" s="23" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F31" s="22" t="inlineStr">
+      <c r="F31" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3558,39 +3572,39 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="21" t="inlineStr">
+      <c r="A34" s="22" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="22" t="inlineStr">
+      <c r="A35" s="23" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B35" s="22" t="inlineStr">
+      <c r="B35" s="23" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C35" s="22" t="inlineStr">
+      <c r="C35" s="23" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D35" s="22" t="inlineStr">
+      <c r="D35" s="23" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E35" s="22" t="inlineStr">
+      <c r="E35" s="23" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F35" s="22" t="inlineStr">
+      <c r="F35" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3669,39 +3683,39 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="21" t="inlineStr">
+      <c r="A40" s="22" t="inlineStr">
         <is>
           <t>October 2026</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="22" t="inlineStr">
+      <c r="A41" s="23" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C41" s="22" t="inlineStr">
+      <c r="C41" s="23" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D41" s="22" t="inlineStr">
+      <c r="D41" s="23" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E41" s="22" t="inlineStr">
+      <c r="E41" s="23" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F41" s="22" t="inlineStr">
+      <c r="F41" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3804,39 +3818,39 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="21" t="inlineStr">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t>November 2026</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="22" t="inlineStr">
+      <c r="A48" s="23" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B48" s="22" t="inlineStr">
+      <c r="B48" s="23" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C48" s="22" t="inlineStr">
+      <c r="C48" s="23" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D48" s="22" t="inlineStr">
+      <c r="D48" s="23" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E48" s="22" t="inlineStr">
+      <c r="E48" s="23" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F48" s="22" t="inlineStr">
+      <c r="F48" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3987,39 +4001,39 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="21" t="inlineStr">
+      <c r="A56" s="22" t="inlineStr">
         <is>
           <t>December 2026</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="22" t="inlineStr">
+      <c r="A57" s="23" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B57" s="22" t="inlineStr">
+      <c r="B57" s="23" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C57" s="22" t="inlineStr">
+      <c r="C57" s="23" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D57" s="22" t="inlineStr">
+      <c r="D57" s="23" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E57" s="22" t="inlineStr">
+      <c r="E57" s="23" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F57" s="22" t="inlineStr">
+      <c r="F57" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -4122,39 +4136,39 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="21" t="inlineStr">
+      <c r="A63" s="22" t="inlineStr">
         <is>
           <t>January 2027</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="22" t="inlineStr">
+      <c r="A64" s="23" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B64" s="22" t="inlineStr">
+      <c r="B64" s="23" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C64" s="22" t="inlineStr">
+      <c r="C64" s="23" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D64" s="22" t="inlineStr">
+      <c r="D64" s="23" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E64" s="22" t="inlineStr">
+      <c r="E64" s="23" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F64" s="22" t="inlineStr">
+      <c r="F64" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -4233,39 +4247,39 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="21" t="inlineStr">
+      <c r="A69" s="22" t="inlineStr">
         <is>
           <t>February 2027</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="22" t="inlineStr">
+      <c r="A70" s="23" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B70" s="22" t="inlineStr">
+      <c r="B70" s="23" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C70" s="22" t="inlineStr">
+      <c r="C70" s="23" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D70" s="22" t="inlineStr">
+      <c r="D70" s="23" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E70" s="22" t="inlineStr">
+      <c r="E70" s="23" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F70" s="22" t="inlineStr">
+      <c r="F70" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -4370,20 +4384,20 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B75" s="10" t="n">
-        <v>46433</v>
+        <v>46432</v>
       </c>
       <c r="C75" s="10" t="n">
-        <v>46425</v>
+        <v>46481</v>
       </c>
       <c r="D75" s="7" t="n">
-        <v>1.883</v>
+        <v>0.41</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>0.01019313304721025</v>
+        <v>0.02499999999999988</v>
       </c>
       <c r="F75" s="12" t="inlineStr">
         <is>
@@ -4394,20 +4408,20 @@
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B76" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="C76" s="10" t="n">
-        <v>46383</v>
+        <v>46425</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>7.45</v>
+        <v>1.883</v>
       </c>
       <c r="E76" s="8" t="n">
-        <v>4.96</v>
+        <v>0.01019313304721025</v>
       </c>
       <c r="F76" s="12" t="inlineStr">
         <is>
@@ -4418,20 +4432,20 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>DVN</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="B77" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="C77" s="10" t="n">
-        <v>46276</v>
+        <v>46383</v>
       </c>
       <c r="D77" s="7" t="n">
-        <v>0.24</v>
+        <v>7.45</v>
       </c>
       <c r="E77" s="8" t="n">
-        <v>0.09090909090909087</v>
+        <v>4.96</v>
       </c>
       <c r="F77" s="12" t="inlineStr">
         <is>
@@ -4442,20 +4456,20 @@
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>DVN</t>
         </is>
       </c>
       <c r="B78" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="C78" s="10" t="n">
-        <v>46177</v>
+        <v>46276</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1.423</v>
+        <v>0.24</v>
       </c>
       <c r="E78" s="8" t="n">
-        <v>0.05018450184501849</v>
+        <v>0.09090909090909087</v>
       </c>
       <c r="F78" s="12" t="inlineStr">
         <is>
@@ -4466,20 +4480,20 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>PFG</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B79" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="C79" s="10" t="n">
-        <v>46270</v>
+        <v>46177</v>
       </c>
       <c r="D79" s="7" t="n">
-        <v>0.8</v>
+        <v>1.423</v>
       </c>
       <c r="E79" s="8" t="n">
-        <v>0.01265822784810128</v>
+        <v>0.05018450184501849</v>
       </c>
       <c r="F79" s="12" t="inlineStr">
         <is>
@@ -4490,20 +4504,20 @@
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>UL</t>
+          <t>PFG</t>
         </is>
       </c>
       <c r="B80" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="C80" s="10" t="n">
-        <v>46243</v>
+        <v>46270</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>0.555</v>
+        <v>0.8</v>
       </c>
       <c r="E80" s="8" t="n">
-        <v>0.005735494868956323</v>
+        <v>0.01265822784810128</v>
       </c>
       <c r="F80" s="12" t="inlineStr">
         <is>
@@ -4514,20 +4528,20 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>ALSN</t>
+          <t>UL</t>
         </is>
       </c>
       <c r="B81" s="10" t="n">
-        <v>46440</v>
+        <v>46433</v>
       </c>
       <c r="C81" s="10" t="n">
-        <v>46450</v>
+        <v>46243</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>0.29</v>
+        <v>0.555</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>0.07407407407407393</v>
+        <v>0.005735494868956323</v>
       </c>
       <c r="F81" s="12" t="inlineStr">
         <is>
@@ -4538,111 +4552,111 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
+          <t>ALSN</t>
+        </is>
+      </c>
+      <c r="B82" s="10" t="n">
+        <v>46440</v>
+      </c>
+      <c r="C82" s="10" t="n">
+        <v>46450</v>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="E82" s="8" t="n">
+        <v>0.07407407407407393</v>
+      </c>
+      <c r="F82" s="12" t="inlineStr">
+        <is>
+          <t>Notion + yfinance</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
           <t>HD</t>
         </is>
       </c>
-      <c r="B82" s="10" t="n">
+      <c r="B83" s="10" t="n">
         <v>46441</v>
       </c>
-      <c r="C82" s="10" t="n">
+      <c r="C83" s="10" t="n">
         <v>46456</v>
       </c>
-      <c r="D82" s="7" t="n">
+      <c r="D83" s="7" t="n">
         <v>2.33</v>
       </c>
-      <c r="E82" s="8" t="n">
+      <c r="E83" s="8" t="n">
         <v>0.01304347826086967</v>
       </c>
-      <c r="F82" s="12" t="inlineStr">
-        <is>
-          <t>Notion + yfinance</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="21" t="inlineStr">
-        <is>
-          <t>March 2027</t>
+      <c r="F83" s="12" t="inlineStr">
+        <is>
+          <t>Notion + yfinance</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="22" t="inlineStr">
         <is>
+          <t>March 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="23" t="inlineStr">
+        <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B85" s="22" t="inlineStr">
+      <c r="B86" s="23" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C85" s="22" t="inlineStr">
+      <c r="C86" s="23" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D85" s="22" t="inlineStr">
+      <c r="D86" s="23" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E85" s="22" t="inlineStr">
+      <c r="E86" s="23" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F85" s="22" t="inlineStr">
+      <c r="F86" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="5" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
         <is>
           <t>GD</t>
         </is>
       </c>
-      <c r="B86" s="10" t="n">
+      <c r="B87" s="10" t="n">
         <v>46451</v>
       </c>
-      <c r="C86" s="10" t="n">
+      <c r="C87" s="10" t="n">
         <v>46487</v>
       </c>
-      <c r="D86" s="7" t="n">
+      <c r="D87" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="E86" s="8" t="n">
+      <c r="E87" s="8" t="n">
         <v>0.05633802816901413</v>
       </c>
-      <c r="F86" s="12" t="inlineStr">
-        <is>
-          <t>Notion + yfinance</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="13" t="inlineStr">
-        <is>
-          <t>CSCO</t>
-        </is>
-      </c>
-      <c r="B87" s="18" t="n">
-        <v>46460</v>
-      </c>
-      <c r="C87" s="18" t="n">
-        <v>46481</v>
-      </c>
-      <c r="D87" s="15" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="E87" s="16" t="n">
-        <v>0.02499999999999988</v>
-      </c>
-      <c r="F87" s="20" t="inlineStr">
-        <is>
-          <t>yfinance</t>
+      <c r="F87" s="12" t="inlineStr">
+        <is>
+          <t>Notion + yfinance</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4747,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete Holdings Dividend Summary - 03/23/2026</t>
+          <t>Complete Holdings Dividend Summary - 03/30/2026</t>
         </is>
       </c>
     </row>
@@ -4833,11 +4847,11 @@
       <c r="F5" s="7" t="n">
         <v>0.29</v>
       </c>
-      <c r="G5" s="23" t="n">
+      <c r="G5" s="24" t="n">
         <v>1.16</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.01011774953826027</v>
+        <v>0.01014074662286406</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>46090</v>
@@ -4886,11 +4900,11 @@
       <c r="F6" s="7" t="n">
         <v>2.52</v>
       </c>
-      <c r="G6" s="23" t="n">
+      <c r="G6" s="24" t="n">
         <v>10.08</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.02869097539422992</v>
+        <v>0.02867628152814483</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>46066</v>
@@ -4939,11 +4953,11 @@
       <c r="F7" s="7" t="n">
         <v>1.883</v>
       </c>
-      <c r="G7" s="23" t="n">
+      <c r="G7" s="24" t="n">
         <v>3.766</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.002723282372501188</v>
+        <v>0.00296196100543417</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>46063</v>
@@ -4992,11 +5006,11 @@
       <c r="F8" s="7" t="n">
         <v>0.703</v>
       </c>
-      <c r="G8" s="23" t="n">
+      <c r="G8" s="24" t="n">
         <v>2.812</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.04124678949944683</v>
+        <v>0.040594776039757</v>
       </c>
       <c r="I8" s="10" t="n">
         <v>46070</v>
@@ -5045,11 +5059,11 @@
       <c r="F9" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="23" t="n">
+      <c r="G9" s="24" t="n">
         <v>4</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.03003454137242492</v>
+        <v>0.02967138990015516</v>
       </c>
       <c r="I9" s="10" t="n">
         <v>46080</v>
@@ -5098,11 +5112,11 @@
       <c r="F10" s="7" t="n">
         <v>1.24</v>
       </c>
-      <c r="G10" s="23" t="n">
+      <c r="G10" s="24" t="n">
         <v>4.96</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.04611808330319646</v>
+        <v>0.04900701556039189</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>46050</v>
@@ -5151,11 +5165,11 @@
       <c r="F11" s="7" t="n">
         <v>7.45</v>
       </c>
-      <c r="G11" s="23" t="n">
+      <c r="G11" s="24" t="n">
         <v>29.8</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.09735221224892325</v>
+        <v>0.1007675883168235</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>46091</v>
@@ -5204,11 +5218,11 @@
       <c r="F12" s="7" t="n">
         <v>0.23</v>
       </c>
-      <c r="G12" s="23" t="n">
+      <c r="G12" s="24" t="n">
         <v>0.92</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.02188391959954028</v>
+        <v>0.0214252452124615</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>46072</v>
@@ -5257,11 +5271,11 @@
       <c r="F13" s="7" t="n">
         <v>0.6</v>
       </c>
-      <c r="G13" s="23" t="n">
+      <c r="G13" s="24" t="n">
         <v>2.4</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0.007356208990148843</v>
+        <v>0.007635530491459991</v>
       </c>
       <c r="I13" s="10" t="n">
         <v>46066</v>
@@ -5282,55 +5296,55 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>CSCO</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>QDVD/DAC</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Jan/Apr/Jul/Oct</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="F14" s="15" t="n">
+      <c r="F14" s="7" t="n">
         <v>0.41</v>
       </c>
       <c r="G14" s="24" t="n">
         <v>1.64</v>
       </c>
-      <c r="H14" s="17" t="n">
-        <v>0.02079898581784063</v>
-      </c>
-      <c r="I14" s="18" t="n">
+      <c r="H14" s="9" t="n">
+        <v>0.02077527171622906</v>
+      </c>
+      <c r="I14" s="10" t="n">
         <v>46024</v>
       </c>
-      <c r="J14" s="16" t="n">
+      <c r="J14" s="8" t="n">
         <v>0.02499999999999988</v>
       </c>
-      <c r="K14" s="18" t="n">
-        <v>46460</v>
-      </c>
-      <c r="L14" s="18" t="n">
+      <c r="K14" s="10" t="n">
+        <v>46432</v>
+      </c>
+      <c r="L14" s="10" t="n">
         <v>46481</v>
       </c>
-      <c r="M14" s="20" t="inlineStr">
-        <is>
-          <t>yfinance</t>
+      <c r="M14" s="12" t="inlineStr">
+        <is>
+          <t>Notion + yfinance</t>
         </is>
       </c>
     </row>
@@ -5363,11 +5377,11 @@
       <c r="F15" s="7" t="n">
         <v>1.78</v>
       </c>
-      <c r="G15" s="23" t="n">
+      <c r="G15" s="24" t="n">
         <v>7.12</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.03538327635252886</v>
+        <v>0.03326092504050905</v>
       </c>
       <c r="I15" s="10" t="n">
         <v>46070</v>
@@ -5416,11 +5430,11 @@
       <c r="F16" s="7" t="n">
         <v>0.8</v>
       </c>
-      <c r="G16" s="23" t="n">
+      <c r="G16" s="24" t="n">
         <v>3.2</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.01629162014983631</v>
+        <v>0.01634988749254875</v>
       </c>
       <c r="I16" s="10" t="n">
         <v>46035</v>
@@ -5469,11 +5483,11 @@
       <c r="F17" s="7" t="n">
         <v>0.24</v>
       </c>
-      <c r="G17" s="23" t="n">
+      <c r="G17" s="24" t="n">
         <v>0.96</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.02006479204737895</v>
+        <v>0.01829616881390908</v>
       </c>
       <c r="I17" s="10" t="n">
         <v>46094</v>
@@ -5522,11 +5536,11 @@
       <c r="F18" s="7" t="n">
         <v>0.84</v>
       </c>
-      <c r="G18" s="23" t="n">
+      <c r="G18" s="24" t="n">
         <v>3.36</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.04986272751327035</v>
+        <v>0.04632565912794535</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>46094</v>
@@ -5575,11 +5589,11 @@
       <c r="F19" s="7" t="n">
         <v>0.64</v>
       </c>
-      <c r="G19" s="23" t="n">
+      <c r="G19" s="24" t="n">
         <v>2.56</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.02537542692959548</v>
+        <v>0.02327378459090542</v>
       </c>
       <c r="I19" s="10" t="n">
         <v>46062</v>
@@ -5628,11 +5642,11 @@
       <c r="F20" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="G20" s="23" t="n">
+      <c r="G20" s="24" t="n">
         <v>6</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.0174218562737619</v>
+        <v>0.01724782270450997</v>
       </c>
       <c r="I20" s="10" t="n">
         <v>46038</v>
@@ -5681,11 +5695,11 @@
       <c r="F21" s="7" t="n">
         <v>2.33</v>
       </c>
-      <c r="G21" s="23" t="n">
+      <c r="G21" s="24" t="n">
         <v>9.32</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.02796825186337326</v>
+        <v>0.02851809941441286</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>46093</v>
@@ -5734,11 +5748,11 @@
       <c r="F22" s="7" t="n">
         <v>1.38</v>
       </c>
-      <c r="G22" s="23" t="n">
+      <c r="G22" s="24" t="n">
         <v>5.52</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>0.01366336633663366</v>
+        <v>0.0146463000754747</v>
       </c>
       <c r="I22" s="10" t="n">
         <v>46080</v>
@@ -5787,11 +5801,11 @@
       <c r="F23" s="7" t="n">
         <v>0.293</v>
       </c>
-      <c r="G23" s="23" t="n">
+      <c r="G23" s="24" t="n">
         <v>1.172</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.05265049361856506</v>
+        <v>0.05067012721677747</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>46034</v>
@@ -5840,11 +5854,11 @@
       <c r="F24" s="7" t="n">
         <v>0.82</v>
       </c>
-      <c r="G24" s="23" t="n">
+      <c r="G24" s="24" t="n">
         <v>3.28</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>0.02994613381315931</v>
+        <v>0.02918668873610638</v>
       </c>
       <c r="I24" s="10" t="n">
         <v>46024</v>
@@ -5893,11 +5907,11 @@
       <c r="F25" s="7" t="n">
         <v>0.61</v>
       </c>
-      <c r="G25" s="23" t="n">
+      <c r="G25" s="24" t="n">
         <v>2.44</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.01475211662660081</v>
+        <v>0.01577348219982237</v>
       </c>
       <c r="I25" s="10" t="n">
         <v>46086</v>
@@ -5946,11 +5960,11 @@
       <c r="F26" s="7" t="n">
         <v>1.3</v>
       </c>
-      <c r="G26" s="23" t="n">
+      <c r="G26" s="24" t="n">
         <v>5.2</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>0.02203016500553975</v>
+        <v>0.02150270835143434</v>
       </c>
       <c r="I26" s="10" t="n">
         <v>46077</v>
@@ -5999,11 +6013,11 @@
       <c r="F27" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="G27" s="23" t="n">
+      <c r="G27" s="24" t="n">
         <v>6</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.02058107236004315</v>
+        <v>0.02104414080461985</v>
       </c>
       <c r="I27" s="10" t="n">
         <v>46028</v>
@@ -6052,11 +6066,11 @@
       <c r="F28" s="7" t="n">
         <v>0.976</v>
       </c>
-      <c r="G28" s="23" t="n">
+      <c r="G28" s="24" t="n">
         <v>1.952</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0.02049343832020997</v>
+        <v>0.02049244854572341</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>45853</v>
@@ -6105,11 +6119,11 @@
       <c r="F29" s="7" t="n">
         <v>0.79</v>
       </c>
-      <c r="G29" s="23" t="n">
+      <c r="G29" s="24" t="n">
         <v>3.16</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.01230577473752138</v>
+        <v>0.01275659546945501</v>
       </c>
       <c r="I29" s="10" t="n">
         <v>46022</v>
@@ -6158,14 +6172,14 @@
       <c r="F30" s="7" t="n">
         <v>0.71</v>
       </c>
-      <c r="G30" s="23" t="n">
+      <c r="G30" s="24" t="n">
         <v>2.84</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.03268124223397447</v>
+        <v>0.03263617685080991</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>46017</v>
+        <v>46108</v>
       </c>
       <c r="J30" s="8" t="n">
         <v>0.0142857142857143</v>
@@ -6211,11 +6225,11 @@
       <c r="F31" s="7" t="n">
         <v>0.48</v>
       </c>
-      <c r="G31" s="23" t="n">
+      <c r="G31" s="24" t="n">
         <v>1.92</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0.0359617910086034</v>
+        <v>0.0361990943977892</v>
       </c>
       <c r="I31" s="10" t="n">
         <v>46020</v>
@@ -6264,11 +6278,11 @@
       <c r="F32" s="7" t="n">
         <v>0.91</v>
       </c>
-      <c r="G32" s="23" t="n">
+      <c r="G32" s="24" t="n">
         <v>3.64</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.009441793172158741</v>
+        <v>0.01011349878049246</v>
       </c>
       <c r="I32" s="10" t="n">
         <v>46072</v>
@@ -6317,11 +6331,11 @@
       <c r="F33" s="7" t="n">
         <v>0.87</v>
       </c>
-      <c r="G33" s="23" t="n">
+      <c r="G33" s="24" t="n">
         <v>3.48</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0.04068272109836166</v>
+        <v>0.03850409499617897</v>
       </c>
       <c r="I33" s="10" t="n">
         <v>46036</v>
@@ -6370,11 +6384,11 @@
       <c r="F34" s="7" t="n">
         <v>0.41</v>
       </c>
-      <c r="G34" s="23" t="n">
+      <c r="G34" s="24" t="n">
         <v>1.64</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0.03073463233210399</v>
+        <v>0.03174603183979984</v>
       </c>
       <c r="I34" s="10" t="n">
         <v>46083</v>
@@ -6423,11 +6437,11 @@
       <c r="F35" s="7" t="n">
         <v>0.584</v>
       </c>
-      <c r="G35" s="23" t="n">
+      <c r="G35" s="24" t="n">
         <v>1.168</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0.03161028351510873</v>
+        <v>0.03309719381407237</v>
       </c>
       <c r="I35" s="10" t="n">
         <v>45887</v>
@@ -6476,11 +6490,11 @@
       <c r="F36" s="7" t="n">
         <v>0.27</v>
       </c>
-      <c r="G36" s="23" t="n">
+      <c r="G36" s="24" t="n">
         <v>3.24</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0.05314088789783094</v>
+        <v>0.05277732582200233</v>
       </c>
       <c r="I36" s="10" t="n">
         <v>46080</v>
@@ -6529,11 +6543,11 @@
       <c r="F37" s="7" t="n">
         <v>1.08</v>
       </c>
-      <c r="G37" s="23" t="n">
+      <c r="G37" s="24" t="n">
         <v>4.32</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.04596967353172818</v>
+        <v>0.04682926829268293</v>
       </c>
       <c r="I37" s="10" t="n">
         <v>46050</v>
@@ -6582,11 +6596,11 @@
       <c r="F38" s="7" t="n">
         <v>1.423</v>
       </c>
-      <c r="G38" s="23" t="n">
+      <c r="G38" s="24" t="n">
         <v>5.692</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0.03783686339934728</v>
+        <v>0.03653519090405939</v>
       </c>
       <c r="I38" s="10" t="n">
         <v>46087</v>
@@ -6635,11 +6649,11 @@
       <c r="F39" s="7" t="n">
         <v>0.43</v>
       </c>
-      <c r="G39" s="23" t="n">
+      <c r="G39" s="24" t="n">
         <v>1.72</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.06394052135283915</v>
+        <v>0.06281177656172118</v>
       </c>
       <c r="I39" s="10" t="n">
         <v>46045</v>
@@ -6688,11 +6702,11 @@
       <c r="F40" s="7" t="n">
         <v>0.8</v>
       </c>
-      <c r="G40" s="23" t="n">
+      <c r="G40" s="24" t="n">
         <v>3.2</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.03720497524150213</v>
+        <v>0.03650051405080914</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>46092</v>
@@ -6741,11 +6755,11 @@
       <c r="F41" s="7" t="n">
         <v>1.057</v>
       </c>
-      <c r="G41" s="23" t="n">
+      <c r="G41" s="24" t="n">
         <v>4.228</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0.0291535954348521</v>
+        <v>0.02939990314843966</v>
       </c>
       <c r="I41" s="10" t="n">
         <v>46045</v>
@@ -6766,53 +6780,53 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="A42" s="14" t="inlineStr">
         <is>
           <t>POR</t>
         </is>
       </c>
-      <c r="B42" s="14" t="inlineStr">
+      <c r="B42" s="15" t="inlineStr">
         <is>
           <t>QDVD/DAC/SMID</t>
         </is>
       </c>
-      <c r="C42" s="14" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="D42" s="14" t="inlineStr">
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
         <is>
           <t>Mar/Jun/Sep/Dec</t>
         </is>
       </c>
-      <c r="E42" s="14" t="inlineStr">
+      <c r="E42" s="15" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="F42" s="15" t="n">
+      <c r="F42" s="16" t="n">
         <v>0.525</v>
       </c>
-      <c r="G42" s="24" t="n">
+      <c r="G42" s="25" t="n">
         <v>2.1</v>
       </c>
-      <c r="H42" s="17" t="n">
-        <v>0.04154713772034981</v>
-      </c>
-      <c r="I42" s="18" t="n">
-        <v>46013</v>
-      </c>
-      <c r="J42" s="16" t="n">
+      <c r="H42" s="18" t="n">
+        <v>0.0402723172224527</v>
+      </c>
+      <c r="I42" s="19" t="n">
+        <v>46104</v>
+      </c>
+      <c r="J42" s="17" t="n">
         <v>0.05000000000000004</v>
       </c>
-      <c r="K42" s="18" t="n">
+      <c r="K42" s="19" t="n">
         <v>46176</v>
       </c>
-      <c r="L42" s="18" t="n">
+      <c r="L42" s="19" t="n">
         <v>46197</v>
       </c>
-      <c r="M42" s="20" t="inlineStr">
+      <c r="M42" s="21" t="inlineStr">
         <is>
           <t>yfinance</t>
         </is>
@@ -6847,11 +6861,11 @@
       <c r="F43" s="7" t="n">
         <v>1.27</v>
       </c>
-      <c r="G43" s="23" t="n">
+      <c r="G43" s="24" t="n">
         <v>5.08</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0.02895742012250174</v>
+        <v>0.02688399565783459</v>
       </c>
       <c r="I43" s="10" t="n">
         <v>46076</v>
@@ -6900,11 +6914,11 @@
       <c r="F44" s="7" t="n">
         <v>0.93</v>
       </c>
-      <c r="G44" s="23" t="n">
+      <c r="G44" s="24" t="n">
         <v>3.72</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.01846291281599689</v>
+        <v>0.01864755074222239</v>
       </c>
       <c r="I44" s="10" t="n">
         <v>46070</v>
@@ -6953,11 +6967,11 @@
       <c r="F45" s="7" t="n">
         <v>0.93</v>
       </c>
-      <c r="G45" s="23" t="n">
+      <c r="G45" s="24" t="n">
         <v>3.72</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>0.01846291281599689</v>
+        <v>0.01864755074222239</v>
       </c>
       <c r="I45" s="10" t="n">
         <v>46070</v>
@@ -7006,11 +7020,11 @@
       <c r="F46" s="7" t="n">
         <v>2.44</v>
       </c>
-      <c r="G46" s="23" t="n">
+      <c r="G46" s="24" t="n">
         <v>9.76</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.0268223978014428</v>
+        <v>0.02719988759972165</v>
       </c>
       <c r="I46" s="10" t="n">
         <v>46077</v>
@@ -7059,11 +7073,11 @@
       <c r="F47" s="7" t="n">
         <v>0.83</v>
       </c>
-      <c r="G47" s="23" t="n">
+      <c r="G47" s="24" t="n">
         <v>3.32</v>
       </c>
       <c r="H47" s="9" t="n">
-        <v>0.04739810245968331</v>
+        <v>0.04879482591603472</v>
       </c>
       <c r="I47" s="10" t="n">
         <v>46091</v>
@@ -7112,11 +7126,11 @@
       <c r="F48" s="7" t="n">
         <v>1.3</v>
       </c>
-      <c r="G48" s="23" t="n">
+      <c r="G48" s="24" t="n">
         <v>5.2</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>0.05940820373037564</v>
+        <v>0.0581557898200166</v>
       </c>
       <c r="I48" s="10" t="n">
         <v>46097</v>
@@ -7165,11 +7179,11 @@
       <c r="F49" s="7" t="n">
         <v>0.994</v>
       </c>
-      <c r="G49" s="23" t="n">
+      <c r="G49" s="24" t="n">
         <v>3.976</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.04551803170526622</v>
+        <v>0.0429535990399483</v>
       </c>
       <c r="I49" s="10" t="n">
         <v>45930</v>
@@ -7218,11 +7232,11 @@
       <c r="F50" s="7" t="n">
         <v>1.42</v>
       </c>
-      <c r="G50" s="23" t="n">
+      <c r="G50" s="24" t="n">
         <v>5.68</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.0297506811988012</v>
+        <v>0.02987833617940912</v>
       </c>
       <c r="I50" s="10" t="n">
         <v>46052</v>
@@ -7271,11 +7285,11 @@
       <c r="F51" s="7" t="n">
         <v>0.555</v>
       </c>
-      <c r="G51" s="23" t="n">
+      <c r="G51" s="24" t="n">
         <v>2.22</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.03599513623773182</v>
+        <v>0.03716103009083437</v>
       </c>
       <c r="I51" s="10" t="n">
         <v>46080</v>
@@ -7324,11 +7338,11 @@
       <c r="F52" s="7" t="n">
         <v>1.38</v>
       </c>
-      <c r="G52" s="23" t="n">
+      <c r="G52" s="24" t="n">
         <v>5.52</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.02307065393635178</v>
+        <v>0.02292834890965732</v>
       </c>
       <c r="I52" s="10" t="n">
         <v>46080</v>
@@ -7377,11 +7391,11 @@
       <c r="F53" s="7" t="n">
         <v>1.64</v>
       </c>
-      <c r="G53" s="23" t="n">
+      <c r="G53" s="24" t="n">
         <v>6.56</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>0.06706880854454768</v>
+        <v>0.06847598946793178</v>
       </c>
       <c r="I53" s="10" t="n">
         <v>46070</v>
@@ -7430,11 +7444,11 @@
       <c r="F54" s="7" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="G54" s="23" t="n">
+      <c r="G54" s="24" t="n">
         <v>2.76</v>
       </c>
       <c r="H54" s="9" t="n">
-        <v>0.0552</v>
+        <v>0.05448429504518887</v>
       </c>
       <c r="I54" s="10" t="n">
         <v>46034</v>
@@ -7483,11 +7497,11 @@
       <c r="F55" s="7" t="n">
         <v>1.03</v>
       </c>
-      <c r="G55" s="23" t="n">
+      <c r="G55" s="24" t="n">
         <v>4.12</v>
       </c>
       <c r="H55" s="9" t="n">
-        <v>0.02607182508545984</v>
+        <v>0.02356574933849925</v>
       </c>
       <c r="I55" s="10" t="n">
         <v>46065</v>
@@ -7510,252 +7524,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
-    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
-    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
-                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
-                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{161435CF-554B-4E9C-8EF7-D306330B17B9}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94120F72-60DA-490F-BAAC-86AA11994D08}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8340C35D-F94E-472C-A02F-046046F1B44A}"/>
 </file>
</xml_diff>

<commit_message>
Update dividend calendar 2026-04-06
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -561,7 +561,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estimated Dividend Calendar: Anticipated Announcements - 03/30/2026</t>
+          <t>Estimated Dividend Calendar: Anticipated Announcements - 04/06/2026</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         <v>46122</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>46132</v>
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="L6" s="9" t="n">
-        <v>0.02939990314843966</v>
+        <v>0.02946546684884909</v>
       </c>
     </row>
     <row r="7">
@@ -711,8 +711,8 @@
       <c r="H7" s="10" t="n">
         <v>46127</v>
       </c>
-      <c r="I7" s="13" t="n">
-        <v>16</v>
+      <c r="I7" s="11" t="n">
+        <v>9</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>46503</v>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.02049244854572341</v>
+        <v>0.0195944584037564</v>
       </c>
     </row>
     <row r="8">
@@ -757,8 +757,8 @@
       <c r="H8" s="10" t="n">
         <v>46128</v>
       </c>
-      <c r="I8" s="13" t="n">
-        <v>17</v>
+      <c r="I8" s="11" t="n">
+        <v>10</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>46165</v>
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.02150270835143434</v>
+        <v>0.02139433526031882</v>
       </c>
     </row>
     <row r="9">
@@ -804,7 +804,7 @@
         <v>46134</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>46161</v>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>0.02688399565783459</v>
+        <v>0.02905015235229855</v>
       </c>
     </row>
     <row r="10">
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>0.994</v>
+        <v>0.974</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>0.831</v>
@@ -850,7 +850,7 @@
         <v>46140</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>46190</v>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.0429535990399483</v>
+        <v>0.04255365613034411</v>
       </c>
     </row>
     <row r="11">
@@ -896,7 +896,7 @@
         <v>46143</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46152</v>
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.04682926829268293</v>
+        <v>0.04695652173913044</v>
       </c>
     </row>
     <row r="12">
@@ -942,7 +942,7 @@
         <v>46162</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>46198</v>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0.03263617685080991</v>
+        <v>0.03260661162396298</v>
       </c>
     </row>
     <row r="13">
@@ -988,7 +988,7 @@
         <v>46176</v>
       </c>
       <c r="I13" s="20" t="n">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="J13" s="19" t="n">
         <v>46197</v>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="L13" s="18" t="n">
-        <v>0.0402723172224527</v>
+        <v>0.03943291630609523</v>
       </c>
     </row>
     <row r="14">
@@ -1034,7 +1034,7 @@
         <v>46218</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>46248</v>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.01864755074222239</v>
+        <v>0.0182053974002074</v>
       </c>
     </row>
     <row r="15">
@@ -1080,7 +1080,7 @@
         <v>46218</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>46248</v>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>0.01864755074222239</v>
+        <v>0.0182053974002074</v>
       </c>
     </row>
     <row r="16">
@@ -1126,7 +1126,7 @@
         <v>46220</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>46264</v>
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="L16" s="9" t="n">
-        <v>0.02292834890965732</v>
+        <v>0.02260395961839812</v>
       </c>
     </row>
     <row r="17">
@@ -1172,7 +1172,7 @@
         <v>46227</v>
       </c>
       <c r="I17" s="13" t="n">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>46267</v>
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.04879482591603472</v>
+        <v>0.04888823179157632</v>
       </c>
     </row>
     <row r="18">
@@ -1218,7 +1218,7 @@
         <v>46232</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>46264</v>
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.02967138990015516</v>
+        <v>0.02880910342347681</v>
       </c>
     </row>
     <row r="19">
@@ -1264,7 +1264,7 @@
         <v>46232</v>
       </c>
       <c r="I19" s="13" t="n">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>46246</v>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0.04900701556039189</v>
+        <v>0.04837608562423524</v>
       </c>
     </row>
     <row r="20">
@@ -1310,7 +1310,7 @@
         <v>46263</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>46297</v>
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0.02918668873610638</v>
+        <v>0.02911802652356768</v>
       </c>
     </row>
     <row r="21">
@@ -1356,7 +1356,7 @@
         <v>46267</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46303</v>
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.05448429504518887</v>
+        <v>0.05561152409027773</v>
       </c>
     </row>
     <row r="22">
@@ -1402,7 +1402,7 @@
         <v>46278</v>
       </c>
       <c r="I22" s="13" t="n">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="J22" s="10" t="n">
         <v>46344</v>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="L22" s="9" t="n">
-        <v>0.01011349878049246</v>
+        <v>0.009770500924087532</v>
       </c>
     </row>
     <row r="23">
@@ -1448,7 +1448,7 @@
         <v>46285</v>
       </c>
       <c r="I23" s="13" t="n">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>46325</v>
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0.02987833617940912</v>
+        <v>0.02878279634676914</v>
       </c>
     </row>
     <row r="24">
@@ -1494,7 +1494,7 @@
         <v>46305</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="J24" s="10" t="n">
         <v>46339</v>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="L24" s="9" t="n">
-        <v>0.03850409499617897</v>
+        <v>0.038431804337001</v>
       </c>
     </row>
     <row r="25">
@@ -1540,7 +1540,7 @@
         <v>46311</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>46386</v>
@@ -1551,7 +1551,7 @@
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>0.01275659546945501</v>
+        <v>0.01301965272377644</v>
       </c>
     </row>
     <row r="26">
@@ -1586,7 +1586,7 @@
         <v>46317</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>46351</v>
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0.0146463000754747</v>
+        <v>0.01372656238853958</v>
       </c>
     </row>
     <row r="27">
@@ -1632,7 +1632,7 @@
         <v>46322</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>46338</v>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="L27" s="9" t="n">
-        <v>0.02327378459090542</v>
+        <v>0.02220680106790347</v>
       </c>
     </row>
     <row r="28">
@@ -1678,7 +1678,7 @@
         <v>46329</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>46338</v>
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="L28" s="9" t="n">
-        <v>0.007635530491459991</v>
+        <v>0.007531774818673483</v>
       </c>
     </row>
     <row r="29">
@@ -1724,7 +1724,7 @@
         <v>46332</v>
       </c>
       <c r="I29" s="13" t="n">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>46346</v>
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>0.02719988759972165</v>
+        <v>0.02673633489571878</v>
       </c>
     </row>
     <row r="30">
@@ -1770,7 +1770,7 @@
         <v>46341</v>
       </c>
       <c r="I30" s="13" t="n">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="J30" s="10" t="n">
         <v>46339</v>
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="L30" s="9" t="n">
-        <v>0.02356574933849925</v>
+        <v>0.02562587564240667</v>
       </c>
     </row>
     <row r="31">
@@ -1816,7 +1816,7 @@
         <v>46344</v>
       </c>
       <c r="I31" s="13" t="n">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>46385</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="n">
-        <v>0.0361990943977892</v>
+        <v>0.03831570498132009</v>
       </c>
     </row>
     <row r="32">
@@ -1862,7 +1862,7 @@
         <v>46347</v>
       </c>
       <c r="I32" s="13" t="n">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>46358</v>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="L32" s="9" t="n">
-        <v>0.03174603183979984</v>
+        <v>0.03746858539749241</v>
       </c>
     </row>
     <row r="33">
@@ -1908,7 +1908,7 @@
         <v>46352</v>
       </c>
       <c r="I33" s="13" t="n">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>46400</v>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>0.05067012721677747</v>
+        <v>0.05307971032833607</v>
       </c>
     </row>
     <row r="34">
@@ -1954,7 +1954,7 @@
         <v>46360</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>46371</v>
@@ -1965,7 +1965,7 @@
         </is>
       </c>
       <c r="L34" s="9" t="n">
-        <v>0.04632565912794535</v>
+        <v>0.04515521885010952</v>
       </c>
     </row>
     <row r="35">
@@ -2000,7 +2000,7 @@
         <v>46366</v>
       </c>
       <c r="I35" s="13" t="n">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>46432</v>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0.02867628152814483</v>
+        <v>0.02915401301518438</v>
       </c>
     </row>
     <row r="36">
@@ -2046,7 +2046,7 @@
         <v>46370</v>
       </c>
       <c r="I36" s="13" t="n">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>46413</v>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="L36" s="9" t="n">
-        <v>0.06281177656172118</v>
+        <v>0.06112295797109072</v>
       </c>
     </row>
     <row r="37">
@@ -2092,7 +2092,7 @@
         <v>46371</v>
       </c>
       <c r="I37" s="13" t="n">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>46344</v>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>0.0214252452124615</v>
+        <v>0.02106227091511688</v>
       </c>
     </row>
     <row r="38">
@@ -2138,7 +2138,7 @@
         <v>46411</v>
       </c>
       <c r="I38" s="13" t="n">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>46435</v>
@@ -2149,7 +2149,7 @@
         </is>
       </c>
       <c r="L38" s="9" t="n">
-        <v>0.040594776039757</v>
+        <v>0.03977650487500992</v>
       </c>
     </row>
     <row r="39">
@@ -2184,7 +2184,7 @@
         <v>46416</v>
       </c>
       <c r="I39" s="13" t="n">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>46483</v>
@@ -2195,7 +2195,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.01634988749254875</v>
+        <v>0.01618941586923297</v>
       </c>
     </row>
     <row r="40">
@@ -2230,7 +2230,7 @@
         <v>46417</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="J40" s="10" t="n">
         <v>46433</v>
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.03326092504050905</v>
+        <v>0.03602783048703352</v>
       </c>
     </row>
     <row r="41">
@@ -2261,22 +2261,22 @@
         </is>
       </c>
       <c r="D41" s="7" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="E41" s="7" t="n">
         <v>0.584</v>
       </c>
-      <c r="E41" s="7" t="n">
-        <v>0.513</v>
-      </c>
       <c r="F41" s="8" t="n">
-        <v>1.142300194931774</v>
+        <v>1.183219178082192</v>
       </c>
       <c r="G41" s="9" t="n">
         <v>0.12</v>
       </c>
       <c r="H41" s="10" t="n">
-        <v>46419</v>
+        <v>46422</v>
       </c>
       <c r="I41" s="13" t="n">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>46472</v>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>0.03309719381407237</v>
+        <v>0.06854838569090677</v>
       </c>
     </row>
     <row r="42">
@@ -2322,7 +2322,7 @@
         <v>46423</v>
       </c>
       <c r="I42" s="13" t="n">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="J42" s="10" t="n">
         <v>46435</v>
@@ -2333,7 +2333,7 @@
         </is>
       </c>
       <c r="L42" s="9" t="n">
-        <v>0.06847598946793178</v>
+        <v>0.06725790489254314</v>
       </c>
     </row>
     <row r="43">
@@ -2368,7 +2368,7 @@
         <v>46428</v>
       </c>
       <c r="I43" s="13" t="n">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>46452</v>
@@ -2379,7 +2379,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>0.01577348219982237</v>
+        <v>0.01528008289635777</v>
       </c>
     </row>
     <row r="44">
@@ -2414,7 +2414,7 @@
         <v>46428</v>
       </c>
       <c r="I44" s="13" t="n">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="J44" s="10" t="n">
         <v>46460</v>
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="L44" s="9" t="n">
-        <v>0.0581557898200166</v>
+        <v>0.05781632042302506</v>
       </c>
     </row>
     <row r="45">
@@ -2445,25 +2445,25 @@
         </is>
       </c>
       <c r="D45" s="7" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E45" s="7" t="n">
         <v>0.41</v>
       </c>
-      <c r="E45" s="7" t="n">
-        <v>0.4</v>
-      </c>
       <c r="F45" s="8" t="n">
-        <v>0.02499999999999988</v>
+        <v>0.02439024390243905</v>
       </c>
       <c r="G45" s="9" t="n">
         <v>0.04</v>
       </c>
       <c r="H45" s="10" t="n">
-        <v>46432</v>
+        <v>46431</v>
       </c>
       <c r="I45" s="13" t="n">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="J45" s="10" t="n">
-        <v>46481</v>
+        <v>46480</v>
       </c>
       <c r="K45" s="12" t="inlineStr">
         <is>
@@ -2471,7 +2471,7 @@
         </is>
       </c>
       <c r="L45" s="9" t="n">
-        <v>0.02077527171622906</v>
+        <v>0.02118403623397195</v>
       </c>
     </row>
     <row r="46">
@@ -2506,7 +2506,7 @@
         <v>46433</v>
       </c>
       <c r="I46" s="13" t="n">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="J46" s="10" t="n">
         <v>46425</v>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="L46" s="9" t="n">
-        <v>0.00296196100543417</v>
+        <v>0.002892672996696654</v>
       </c>
     </row>
     <row r="47">
@@ -2552,7 +2552,7 @@
         <v>46433</v>
       </c>
       <c r="I47" s="13" t="n">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="J47" s="10" t="n">
         <v>46383</v>
@@ -2563,7 +2563,7 @@
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>0.1007675883168235</v>
+        <v>0.09680353545512323</v>
       </c>
     </row>
     <row r="48">
@@ -2598,7 +2598,7 @@
         <v>46433</v>
       </c>
       <c r="I48" s="13" t="n">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="J48" s="10" t="n">
         <v>46276</v>
@@ -2609,7 +2609,7 @@
         </is>
       </c>
       <c r="L48" s="9" t="n">
-        <v>0.01829616881390908</v>
+        <v>0.01938806446195164</v>
       </c>
     </row>
     <row r="49">
@@ -2644,7 +2644,7 @@
         <v>46433</v>
       </c>
       <c r="I49" s="13" t="n">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>46177</v>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>0.03653519090405939</v>
+        <v>0.03651761197349492</v>
       </c>
     </row>
     <row r="50">
@@ -2690,7 +2690,7 @@
         <v>46433</v>
       </c>
       <c r="I50" s="13" t="n">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="J50" s="10" t="n">
         <v>46270</v>
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="L50" s="9" t="n">
-        <v>0.03650051405080914</v>
+        <v>0.03542370102874154</v>
       </c>
     </row>
     <row r="51">
@@ -2736,7 +2736,7 @@
         <v>46433</v>
       </c>
       <c r="I51" s="13" t="n">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="J51" s="10" t="n">
         <v>46243</v>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>0.03716103009083437</v>
+        <v>0.03963578051289666</v>
       </c>
     </row>
     <row r="52">
@@ -2782,7 +2782,7 @@
         <v>46440</v>
       </c>
       <c r="I52" s="13" t="n">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="J52" s="10" t="n">
         <v>46450</v>
@@ -2793,7 +2793,7 @@
         </is>
       </c>
       <c r="L52" s="9" t="n">
-        <v>0.01014074662286406</v>
+        <v>0.009962640308522799</v>
       </c>
     </row>
     <row r="53">
@@ -2828,7 +2828,7 @@
         <v>46441</v>
       </c>
       <c r="I53" s="13" t="n">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="J53" s="10" t="n">
         <v>46456</v>
@@ -2839,7 +2839,7 @@
         </is>
       </c>
       <c r="L53" s="9" t="n">
-        <v>0.02851809941441286</v>
+        <v>0.02894409937888199</v>
       </c>
     </row>
     <row r="54">
@@ -2874,7 +2874,7 @@
         <v>46451</v>
       </c>
       <c r="I54" s="13" t="n">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="J54" s="10" t="n">
         <v>46487</v>
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="L54" s="9" t="n">
-        <v>0.01724782270450997</v>
+        <v>0.0172314755590317</v>
       </c>
     </row>
     <row r="55">
@@ -2920,7 +2920,7 @@
         <v>46461</v>
       </c>
       <c r="I55" s="13" t="n">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="J55" s="10" t="n">
         <v>46300</v>
@@ -2931,7 +2931,7 @@
         </is>
       </c>
       <c r="L55" s="9" t="n">
-        <v>0.02104414080461985</v>
+        <v>0.02029289318332066</v>
       </c>
     </row>
     <row r="56">
@@ -2951,13 +2951,13 @@
         </is>
       </c>
       <c r="D56" s="7" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="E56" s="7" t="n">
         <v>0.27</v>
       </c>
-      <c r="E56" s="7" t="n">
-        <v>0.269</v>
-      </c>
       <c r="F56" s="8" t="n">
-        <v>0.003717472118959111</v>
+        <v>0.003703703703703707</v>
       </c>
       <c r="G56" s="9" t="n">
         <v>0.02</v>
@@ -2966,7 +2966,7 @@
         <v>46461</v>
       </c>
       <c r="I56" s="13" t="n">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="J56" s="10" t="n">
         <v>46196</v>
@@ -2977,7 +2977,7 @@
         </is>
       </c>
       <c r="L56" s="9" t="n">
-        <v>0.05277732582200233</v>
+        <v>0.05231660244502703</v>
       </c>
     </row>
   </sheetData>
@@ -3012,7 +3012,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Expected Increase Announcements by Month - 03/30/2026</t>
+          <t>Expected Increase Announcements by Month - 04/06/2026</t>
         </is>
       </c>
     </row>
@@ -3164,7 +3164,7 @@
         <v>46190</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>0.994</v>
+        <v>0.974</v>
       </c>
       <c r="E10" s="8" t="n">
         <v>0.2021660649819495</v>
@@ -4292,16 +4292,16 @@
         </is>
       </c>
       <c r="B71" s="10" t="n">
-        <v>46419</v>
+        <v>46422</v>
       </c>
       <c r="C71" s="10" t="n">
         <v>46472</v>
       </c>
       <c r="D71" s="7" t="n">
-        <v>0.584</v>
+        <v>1.275</v>
       </c>
       <c r="E71" s="8" t="n">
-        <v>1.142300194931774</v>
+        <v>1.183219178082192</v>
       </c>
       <c r="F71" s="12" t="inlineStr">
         <is>
@@ -4388,16 +4388,16 @@
         </is>
       </c>
       <c r="B75" s="10" t="n">
-        <v>46432</v>
+        <v>46431</v>
       </c>
       <c r="C75" s="10" t="n">
-        <v>46481</v>
+        <v>46480</v>
       </c>
       <c r="D75" s="7" t="n">
-        <v>0.41</v>
+        <v>0.42</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>0.02499999999999988</v>
+        <v>0.02439024390243905</v>
       </c>
       <c r="F75" s="12" t="inlineStr">
         <is>
@@ -4697,10 +4697,10 @@
         <v>46196</v>
       </c>
       <c r="D89" s="7" t="n">
-        <v>0.27</v>
+        <v>0.271</v>
       </c>
       <c r="E89" s="8" t="n">
-        <v>0.003717472118959111</v>
+        <v>0.003703703703703707</v>
       </c>
       <c r="F89" s="12" t="inlineStr">
         <is>
@@ -4747,7 +4747,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete Holdings Dividend Summary - 03/30/2026</t>
+          <t>Complete Holdings Dividend Summary - 04/06/2026</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
         <v>1.16</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.01014074662286406</v>
+        <v>0.009962640308522799</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>46090</v>
@@ -4904,7 +4904,7 @@
         <v>10.08</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.02867628152814483</v>
+        <v>0.02915401301518438</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>46066</v>
@@ -4957,7 +4957,7 @@
         <v>3.766</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.00296196100543417</v>
+        <v>0.002892672996696654</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>46063</v>
@@ -5010,7 +5010,7 @@
         <v>2.812</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.040594776039757</v>
+        <v>0.03977650487500992</v>
       </c>
       <c r="I8" s="10" t="n">
         <v>46070</v>
@@ -5063,7 +5063,7 @@
         <v>4</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.02967138990015516</v>
+        <v>0.02880910342347681</v>
       </c>
       <c r="I9" s="10" t="n">
         <v>46080</v>
@@ -5116,7 +5116,7 @@
         <v>4.96</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.04900701556039189</v>
+        <v>0.04837608562423524</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>46050</v>
@@ -5169,7 +5169,7 @@
         <v>29.8</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.1007675883168235</v>
+        <v>0.09680353545512323</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>46091</v>
@@ -5222,7 +5222,7 @@
         <v>0.92</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.0214252452124615</v>
+        <v>0.02106227091511688</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>46072</v>
@@ -5275,7 +5275,7 @@
         <v>2.4</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0.007635530491459991</v>
+        <v>0.007531774818673483</v>
       </c>
       <c r="I13" s="10" t="n">
         <v>46066</v>
@@ -5322,25 +5322,25 @@
         </is>
       </c>
       <c r="F14" s="7" t="n">
-        <v>0.41</v>
+        <v>0.42</v>
       </c>
       <c r="G14" s="24" t="n">
-        <v>1.64</v>
+        <v>1.68</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0.02077527171622906</v>
+        <v>0.02118403623397195</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>46024</v>
+        <v>46114</v>
       </c>
       <c r="J14" s="8" t="n">
-        <v>0.02499999999999988</v>
+        <v>0.02439024390243905</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>46432</v>
+        <v>46431</v>
       </c>
       <c r="L14" s="10" t="n">
-        <v>46481</v>
+        <v>46480</v>
       </c>
       <c r="M14" s="12" t="inlineStr">
         <is>
@@ -5381,7 +5381,7 @@
         <v>7.12</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.03326092504050905</v>
+        <v>0.03602783048703352</v>
       </c>
       <c r="I15" s="10" t="n">
         <v>46070</v>
@@ -5434,7 +5434,7 @@
         <v>3.2</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.01634988749254875</v>
+        <v>0.01618941586923297</v>
       </c>
       <c r="I16" s="10" t="n">
         <v>46035</v>
@@ -5487,7 +5487,7 @@
         <v>0.96</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.01829616881390908</v>
+        <v>0.01938806446195164</v>
       </c>
       <c r="I17" s="10" t="n">
         <v>46094</v>
@@ -5540,7 +5540,7 @@
         <v>3.36</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.04632565912794535</v>
+        <v>0.04515521885010952</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>46094</v>
@@ -5593,7 +5593,7 @@
         <v>2.56</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.02327378459090542</v>
+        <v>0.02220680106790347</v>
       </c>
       <c r="I19" s="10" t="n">
         <v>46062</v>
@@ -5646,7 +5646,7 @@
         <v>6</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.01724782270450997</v>
+        <v>0.0172314755590317</v>
       </c>
       <c r="I20" s="10" t="n">
         <v>46038</v>
@@ -5699,7 +5699,7 @@
         <v>9.32</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.02851809941441286</v>
+        <v>0.02894409937888199</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>46093</v>
@@ -5752,7 +5752,7 @@
         <v>5.52</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>0.0146463000754747</v>
+        <v>0.01372656238853958</v>
       </c>
       <c r="I22" s="10" t="n">
         <v>46080</v>
@@ -5805,7 +5805,7 @@
         <v>1.172</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.05067012721677747</v>
+        <v>0.05307971032833607</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>46034</v>
@@ -5858,10 +5858,10 @@
         <v>3.28</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>0.02918668873610638</v>
+        <v>0.02911802652356768</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>46024</v>
+        <v>46113</v>
       </c>
       <c r="J24" s="8" t="n">
         <v>0.02499999999999988</v>
@@ -5911,7 +5911,7 @@
         <v>2.44</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.01577348219982237</v>
+        <v>0.01528008289635777</v>
       </c>
       <c r="I25" s="10" t="n">
         <v>46086</v>
@@ -5964,7 +5964,7 @@
         <v>5.2</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>0.02150270835143434</v>
+        <v>0.02139433526031882</v>
       </c>
       <c r="I26" s="10" t="n">
         <v>46077</v>
@@ -6017,7 +6017,7 @@
         <v>6</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.02104414080461985</v>
+        <v>0.02029289318332066</v>
       </c>
       <c r="I27" s="10" t="n">
         <v>46028</v>
@@ -6070,7 +6070,7 @@
         <v>1.952</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0.02049244854572341</v>
+        <v>0.0195944584037564</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>45853</v>
@@ -6123,10 +6123,10 @@
         <v>3.16</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.01275659546945501</v>
+        <v>0.01301965272377644</v>
       </c>
       <c r="I29" s="10" t="n">
-        <v>46022</v>
+        <v>46112</v>
       </c>
       <c r="J29" s="8" t="n">
         <v>0.05333333333333338</v>
@@ -6176,7 +6176,7 @@
         <v>2.84</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.03263617685080991</v>
+        <v>0.03260661162396298</v>
       </c>
       <c r="I30" s="10" t="n">
         <v>46108</v>
@@ -6229,7 +6229,7 @@
         <v>1.92</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0.0361990943977892</v>
+        <v>0.03831570498132009</v>
       </c>
       <c r="I31" s="10" t="n">
         <v>46020</v>
@@ -6282,7 +6282,7 @@
         <v>3.64</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.01011349878049246</v>
+        <v>0.009770500924087532</v>
       </c>
       <c r="I32" s="10" t="n">
         <v>46072</v>
@@ -6335,7 +6335,7 @@
         <v>3.48</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0.03850409499617897</v>
+        <v>0.038431804337001</v>
       </c>
       <c r="I33" s="10" t="n">
         <v>46036</v>
@@ -6388,7 +6388,7 @@
         <v>1.64</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0.03174603183979984</v>
+        <v>0.03746858539749241</v>
       </c>
       <c r="I34" s="10" t="n">
         <v>46083</v>
@@ -6435,22 +6435,22 @@
         </is>
       </c>
       <c r="F35" s="7" t="n">
-        <v>0.584</v>
+        <v>1.275</v>
       </c>
       <c r="G35" s="24" t="n">
-        <v>1.168</v>
+        <v>2.55</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0.03309719381407237</v>
+        <v>0.06854838569090677</v>
       </c>
       <c r="I35" s="10" t="n">
-        <v>45887</v>
+        <v>46111</v>
       </c>
       <c r="J35" s="8" t="n">
-        <v>1.142300194931774</v>
+        <v>1.183219178082192</v>
       </c>
       <c r="K35" s="10" t="n">
-        <v>46419</v>
+        <v>46422</v>
       </c>
       <c r="L35" s="10" t="n">
         <v>46472</v>
@@ -6488,19 +6488,19 @@
         </is>
       </c>
       <c r="F36" s="7" t="n">
-        <v>0.27</v>
+        <v>0.271</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>3.24</v>
+        <v>3.252</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0.05277732582200233</v>
+        <v>0.05231660244502703</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>46080</v>
+        <v>46112</v>
       </c>
       <c r="J36" s="8" t="n">
-        <v>0.003717472118959111</v>
+        <v>0.003703703703703707</v>
       </c>
       <c r="K36" s="10" t="n">
         <v>46461</v>
@@ -6547,7 +6547,7 @@
         <v>4.32</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.04682926829268293</v>
+        <v>0.04695652173913044</v>
       </c>
       <c r="I37" s="10" t="n">
         <v>46050</v>
@@ -6600,7 +6600,7 @@
         <v>5.692</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0.03653519090405939</v>
+        <v>0.03651761197349492</v>
       </c>
       <c r="I38" s="10" t="n">
         <v>46087</v>
@@ -6653,7 +6653,7 @@
         <v>1.72</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.06281177656172118</v>
+        <v>0.06112295797109072</v>
       </c>
       <c r="I39" s="10" t="n">
         <v>46045</v>
@@ -6706,7 +6706,7 @@
         <v>3.2</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.03650051405080914</v>
+        <v>0.03542370102874154</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>46092</v>
@@ -6759,7 +6759,7 @@
         <v>4.228</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0.02939990314843966</v>
+        <v>0.02946546684884909</v>
       </c>
       <c r="I41" s="10" t="n">
         <v>46045</v>
@@ -6812,7 +6812,7 @@
         <v>2.1</v>
       </c>
       <c r="H42" s="18" t="n">
-        <v>0.0402723172224527</v>
+        <v>0.03943291630609523</v>
       </c>
       <c r="I42" s="19" t="n">
         <v>46104</v>
@@ -6865,7 +6865,7 @@
         <v>5.08</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0.02688399565783459</v>
+        <v>0.02905015235229855</v>
       </c>
       <c r="I43" s="10" t="n">
         <v>46076</v>
@@ -6918,7 +6918,7 @@
         <v>3.72</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.01864755074222239</v>
+        <v>0.0182053974002074</v>
       </c>
       <c r="I44" s="10" t="n">
         <v>46070</v>
@@ -6971,7 +6971,7 @@
         <v>3.72</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>0.01864755074222239</v>
+        <v>0.0182053974002074</v>
       </c>
       <c r="I45" s="10" t="n">
         <v>46070</v>
@@ -7024,7 +7024,7 @@
         <v>9.76</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.02719988759972165</v>
+        <v>0.02673633489571878</v>
       </c>
       <c r="I46" s="10" t="n">
         <v>46077</v>
@@ -7077,7 +7077,7 @@
         <v>3.32</v>
       </c>
       <c r="H47" s="9" t="n">
-        <v>0.04879482591603472</v>
+        <v>0.04888823179157632</v>
       </c>
       <c r="I47" s="10" t="n">
         <v>46091</v>
@@ -7130,7 +7130,7 @@
         <v>5.2</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>0.0581557898200166</v>
+        <v>0.05781632042302506</v>
       </c>
       <c r="I48" s="10" t="n">
         <v>46097</v>
@@ -7177,16 +7177,16 @@
         </is>
       </c>
       <c r="F49" s="7" t="n">
-        <v>0.994</v>
+        <v>0.974</v>
       </c>
       <c r="G49" s="24" t="n">
-        <v>3.976</v>
+        <v>3.896</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.0429535990399483</v>
+        <v>0.04255365613034411</v>
       </c>
       <c r="I49" s="10" t="n">
-        <v>45930</v>
+        <v>46112</v>
       </c>
       <c r="J49" s="8" t="n">
         <v>0.2021660649819495</v>
@@ -7236,7 +7236,7 @@
         <v>5.68</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.02987833617940912</v>
+        <v>0.02878279634676914</v>
       </c>
       <c r="I50" s="10" t="n">
         <v>46052</v>
@@ -7289,7 +7289,7 @@
         <v>2.22</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.03716103009083437</v>
+        <v>0.03963578051289666</v>
       </c>
       <c r="I51" s="10" t="n">
         <v>46080</v>
@@ -7342,7 +7342,7 @@
         <v>5.52</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.02292834890965732</v>
+        <v>0.02260395961839812</v>
       </c>
       <c r="I52" s="10" t="n">
         <v>46080</v>
@@ -7395,7 +7395,7 @@
         <v>6.56</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>0.06847598946793178</v>
+        <v>0.06725790489254314</v>
       </c>
       <c r="I53" s="10" t="n">
         <v>46070</v>
@@ -7448,7 +7448,7 @@
         <v>2.76</v>
       </c>
       <c r="H54" s="9" t="n">
-        <v>0.05448429504518887</v>
+        <v>0.05561152409027773</v>
       </c>
       <c r="I54" s="10" t="n">
         <v>46034</v>
@@ -7501,7 +7501,7 @@
         <v>4.12</v>
       </c>
       <c r="H55" s="9" t="n">
-        <v>0.02356574933849925</v>
+        <v>0.02562587564240667</v>
       </c>
       <c r="I55" s="10" t="n">
         <v>46065</v>

</xml_diff>

<commit_message>
Update Fish CCC to March, update dividend calendar
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -7524,4 +7524,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD01F46B-E70E-4E75-9A21-05C9862856AE}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{844DA483-6868-46EE-8DEC-2DB25D264EF2}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6A27D70-83F6-4C97-9F74-EA5E31419677}"/>
 </file>
</xml_diff>

<commit_message>
Clean up canary file; sync latest dividend calendar
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -7577,4 +7577,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A9EE666-59A1-445B-A6BB-685A9ABB2D2B}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5669A616-8E12-4102-B2C2-12C542DC3108}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72DFD854-7B62-4A32-ACE5-0295C9E9EA2A}"/>
 </file>
</xml_diff>

<commit_message>
Update dividend calendar 2026-06-01
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -550,7 +550,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estimated Dividend Calendar: Anticipated Announcements - 05/25/2026</t>
+          <t>Estimated Dividend Calendar: Anticipated Announcements - 06/01/2026</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
         <v>46162</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-5</v>
+        <v>-12</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>46563</v>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="L6" s="9" t="n">
-        <v>0.03613231622307302</v>
+        <v>0.03798822791396991</v>
       </c>
     </row>
     <row r="7">
@@ -701,7 +701,7 @@
         <v>46218</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>46248</v>
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.01737992953039871</v>
+        <v>0.01859581611162467</v>
       </c>
     </row>
     <row r="8">
@@ -747,7 +747,7 @@
         <v>46220</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>46264</v>
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.02076124529346597</v>
+        <v>0.02116402056970356</v>
       </c>
     </row>
     <row r="9">
@@ -793,7 +793,7 @@
         <v>46227</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>46267</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>0.04342139732871405</v>
+        <v>0.04297178239972002</v>
       </c>
     </row>
     <row r="10">
@@ -824,13 +824,13 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="E10" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="7" t="n">
-        <v>0.95</v>
-      </c>
       <c r="F10" s="8" t="n">
-        <v>0.05263157894736847</v>
+        <v>0.03000000000000003</v>
       </c>
       <c r="G10" s="9" t="n">
         <v>0.06</v>
@@ -839,7 +839,7 @@
         <v>46232</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>46264</v>
@@ -850,7 +850,7 @@
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.02869852102073829</v>
+        <v>0.03043622674109861</v>
       </c>
     </row>
     <row r="11">
@@ -885,7 +885,7 @@
         <v>46232</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46246</v>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.05215014160624624</v>
+        <v>0.05544997394320728</v>
       </c>
     </row>
     <row r="12">
@@ -931,7 +931,7 @@
         <v>46263</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>46297</v>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0.03202812110838314</v>
+        <v>0.03260437425199132</v>
       </c>
     </row>
     <row r="13">
@@ -977,7 +977,7 @@
         <v>46278</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>46344</v>
@@ -988,7 +988,7 @@
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>0.008696275261740157</v>
+        <v>0.007827956989247311</v>
       </c>
     </row>
     <row r="14">
@@ -1023,7 +1023,7 @@
         <v>46280</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>46303</v>
@@ -1034,7 +1034,7 @@
         </is>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.05857290774302305</v>
+        <v>0.05932132175180416</v>
       </c>
     </row>
     <row r="15">
@@ -1069,7 +1069,7 @@
         <v>46285</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>46325</v>
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>0.01836939347681198</v>
+        <v>0.01952493873877673</v>
       </c>
     </row>
     <row r="16">
@@ -1115,7 +1115,7 @@
         <v>46305</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>46339</v>
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="L16" s="9" t="n">
-        <v>0.03267605633802817</v>
+        <v>0.03207668972737766</v>
       </c>
     </row>
     <row r="17">
@@ -1161,7 +1161,7 @@
         <v>46311</v>
       </c>
       <c r="I17" s="13" t="n">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>46386</v>
@@ -1172,7 +1172,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.011995596886681</v>
+        <v>0.01247717304408395</v>
       </c>
     </row>
     <row r="18">
@@ -1207,7 +1207,7 @@
         <v>46317</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>46351</v>
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.01721610552954179</v>
+        <v>0.01850982488567165</v>
       </c>
     </row>
     <row r="19">
@@ -1253,7 +1253,7 @@
         <v>46322</v>
       </c>
       <c r="I19" s="13" t="n">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>46338</v>
@@ -1264,7 +1264,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0.02277580040255237</v>
+        <v>0.023931943262468</v>
       </c>
     </row>
     <row r="20">
@@ -1299,7 +1299,7 @@
         <v>46329</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>46338</v>
@@ -1310,7 +1310,7 @@
         </is>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0.008730129744386562</v>
+        <v>0.008972130483968787</v>
       </c>
     </row>
     <row r="21">
@@ -1345,7 +1345,7 @@
         <v>46332</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46346</v>
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.02661939223366119</v>
+        <v>0.02652642468034239</v>
       </c>
     </row>
     <row r="22">
@@ -1391,7 +1391,7 @@
         <v>46341</v>
       </c>
       <c r="I22" s="13" t="n">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="J22" s="10" t="n">
         <v>46339</v>
@@ -1402,7 +1402,7 @@
         </is>
       </c>
       <c r="L22" s="9" t="n">
-        <v>0.02659437160273528</v>
+        <v>0.0276510067114094</v>
       </c>
     </row>
     <row r="23">
@@ -1437,7 +1437,7 @@
         <v>46344</v>
       </c>
       <c r="I23" s="13" t="n">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>46385</v>
@@ -1448,7 +1448,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0.04016736465785078</v>
+        <v>0.0406177275525001</v>
       </c>
     </row>
     <row r="24">
@@ -1483,7 +1483,7 @@
         <v>46347</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="J24" s="10" t="n">
         <v>46358</v>
@@ -1494,7 +1494,7 @@
         </is>
       </c>
       <c r="L24" s="9" t="n">
-        <v>0.03671367958864462</v>
+        <v>0.03578441925543904</v>
       </c>
     </row>
     <row r="25">
@@ -1529,7 +1529,7 @@
         <v>46352</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>46400</v>
@@ -1540,7 +1540,7 @@
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>0.05517890831588747</v>
+        <v>0.0502572905376204</v>
       </c>
     </row>
     <row r="26">
@@ -1575,7 +1575,7 @@
         <v>46360</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>46371</v>
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0.04533189254576684</v>
+        <v>0.04449447165672079</v>
       </c>
     </row>
     <row r="27">
@@ -1621,7 +1621,7 @@
         <v>46366</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>46432</v>
@@ -1632,7 +1632,7 @@
         </is>
       </c>
       <c r="L27" s="9" t="n">
-        <v>0.02970822388048694</v>
+        <v>0.0304605330321046</v>
       </c>
     </row>
     <row r="28">
@@ -1667,7 +1667,7 @@
         <v>46370</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>46413</v>
@@ -1678,7 +1678,7 @@
         </is>
       </c>
       <c r="L28" s="9" t="n">
-        <v>0.06640926738737934</v>
+        <v>0.06686882792307368</v>
       </c>
     </row>
     <row r="29">
@@ -1713,7 +1713,7 @@
         <v>46371</v>
       </c>
       <c r="I29" s="13" t="n">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>46344</v>
@@ -1724,7 +1724,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>0.02148026991987978</v>
+        <v>0.02198064771382014</v>
       </c>
     </row>
     <row r="30">
@@ -1759,7 +1759,7 @@
         <v>46402</v>
       </c>
       <c r="I30" s="13" t="n">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="J30" s="10" t="n">
         <v>46483</v>
@@ -1770,7 +1770,7 @@
         </is>
       </c>
       <c r="L30" s="9" t="n">
-        <v>0.01762204744474112</v>
+        <v>0.01754699192598384</v>
       </c>
     </row>
     <row r="31">
@@ -1805,7 +1805,7 @@
         <v>46411</v>
       </c>
       <c r="I31" s="13" t="n">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>46435</v>
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="n">
-        <v>0.03785166193761971</v>
+        <v>0.03916980030838525</v>
       </c>
     </row>
     <row r="32">
@@ -1851,7 +1851,7 @@
         <v>46417</v>
       </c>
       <c r="I32" s="13" t="n">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>46433</v>
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="L32" s="9" t="n">
-        <v>0.0371937537084845</v>
+        <v>0.0382940836807255</v>
       </c>
     </row>
     <row r="33">
@@ -1897,7 +1897,7 @@
         <v>46422</v>
       </c>
       <c r="I33" s="13" t="n">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>46472</v>
@@ -1908,7 +1908,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>0.05671708300547242</v>
+        <v>0.05704697889209416</v>
       </c>
     </row>
     <row r="34">
@@ -1943,7 +1943,7 @@
         <v>46428</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>46452</v>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="L34" s="9" t="n">
-        <v>0.01740495012131711</v>
+        <v>0.01771324863883848</v>
       </c>
     </row>
     <row r="35">
@@ -1989,7 +1989,7 @@
         <v>46428</v>
       </c>
       <c r="I35" s="13" t="n">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>46460</v>
@@ -2000,7 +2000,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0.05029499981330527</v>
+        <v>0.04959215180541567</v>
       </c>
     </row>
     <row r="36">
@@ -2035,7 +2035,7 @@
         <v>46431</v>
       </c>
       <c r="I36" s="13" t="n">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>46480</v>
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="L36" s="9" t="n">
-        <v>0.01395232911639436</v>
+        <v>0.01410579363160145</v>
       </c>
     </row>
     <row r="37">
@@ -2081,7 +2081,7 @@
         <v>46433</v>
       </c>
       <c r="I37" s="13" t="n">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>46425</v>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>0.007782472784615239</v>
+        <v>0.007991648467354199</v>
       </c>
     </row>
     <row r="38">
@@ -2127,7 +2127,7 @@
         <v>46433</v>
       </c>
       <c r="I38" s="13" t="n">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>46383</v>
@@ -2138,7 +2138,7 @@
         </is>
       </c>
       <c r="L38" s="9" t="n">
-        <v>0.102324619290005</v>
+        <v>0.1111069719600328</v>
       </c>
     </row>
     <row r="39">
@@ -2173,7 +2173,7 @@
         <v>46433</v>
       </c>
       <c r="I39" s="13" t="n">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>46276</v>
@@ -2184,7 +2184,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.02033036796236036</v>
+        <v>0.02049420985253447</v>
       </c>
     </row>
     <row r="40">
@@ -2219,7 +2219,7 @@
         <v>46433</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="J40" s="10" t="n">
         <v>46270</v>
@@ -2230,7 +2230,7 @@
         </is>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.03081367402039418</v>
+        <v>0.03104686144828515</v>
       </c>
     </row>
     <row r="41">
@@ -2265,7 +2265,7 @@
         <v>46433</v>
       </c>
       <c r="I41" s="13" t="n">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>46243</v>
@@ -2276,7 +2276,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>0.03801220676551045</v>
+        <v>0.03906109920010292</v>
       </c>
     </row>
     <row r="42">
@@ -2311,7 +2311,7 @@
         <v>46440</v>
       </c>
       <c r="I42" s="13" t="n">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="J42" s="10" t="n">
         <v>46450</v>
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="L42" s="9" t="n">
-        <v>0.01055793183764243</v>
+        <v>0.01035205922842178</v>
       </c>
     </row>
     <row r="43">
@@ -2357,7 +2357,7 @@
         <v>46441</v>
       </c>
       <c r="I43" s="13" t="n">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>46456</v>
@@ -2368,7 +2368,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>0.02976969937062066</v>
+        <v>0.0298545717812205</v>
       </c>
     </row>
     <row r="44">
@@ -2403,7 +2403,7 @@
         <v>46452</v>
       </c>
       <c r="I44" s="13" t="n">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="J44" s="10" t="n">
         <v>46487</v>
@@ -2414,7 +2414,7 @@
         </is>
       </c>
       <c r="L44" s="9" t="n">
-        <v>0.01854822166962447</v>
+        <v>0.01863408644778464</v>
       </c>
     </row>
     <row r="45">
@@ -2449,7 +2449,7 @@
         <v>46461</v>
       </c>
       <c r="I45" s="13" t="n">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="J45" s="10" t="n">
         <v>46300</v>
@@ -2460,7 +2460,7 @@
         </is>
       </c>
       <c r="L45" s="9" t="n">
-        <v>0.01958352341659811</v>
+        <v>0.02003974557693619</v>
       </c>
     </row>
     <row r="46">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Dec</t>
         </is>
       </c>
       <c r="D46" s="7" t="n">
@@ -2495,10 +2495,10 @@
         <v>46461</v>
       </c>
       <c r="I46" s="13" t="n">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="J46" s="10" t="n">
-        <v>46196</v>
+        <v>46386</v>
       </c>
       <c r="K46" s="12" t="inlineStr">
         <is>
@@ -2506,7 +2506,7 @@
         </is>
       </c>
       <c r="L46" s="9" t="n">
-        <v>0.05243469809734441</v>
+        <v>0.05379652537562463</v>
       </c>
     </row>
     <row r="47">
@@ -2541,7 +2541,7 @@
         <v>46488</v>
       </c>
       <c r="I47" s="13" t="n">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="J47" s="10" t="n">
         <v>46498</v>
@@ -2552,7 +2552,7 @@
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>0.03015785050105535</v>
+        <v>0.03095728656212699</v>
       </c>
     </row>
     <row r="48">
@@ -2587,7 +2587,7 @@
         <v>46492</v>
       </c>
       <c r="I48" s="13" t="n">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="J48" s="10" t="n">
         <v>46501</v>
@@ -2598,7 +2598,7 @@
         </is>
       </c>
       <c r="L48" s="9" t="n">
-        <v>0.0202817422379329</v>
+        <v>0.0204872076875597</v>
       </c>
     </row>
     <row r="49">
@@ -2633,7 +2633,7 @@
         <v>46492</v>
       </c>
       <c r="I49" s="13" t="n">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>46197</v>
@@ -2644,7 +2644,7 @@
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>0.04215174654483525</v>
+        <v>0.04247572933518482</v>
       </c>
     </row>
     <row r="50">
@@ -2679,7 +2679,7 @@
         <v>46492</v>
       </c>
       <c r="I50" s="13" t="n">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="J50" s="10" t="n">
         <v>46376</v>
@@ -2690,7 +2690,7 @@
         </is>
       </c>
       <c r="L50" s="9" t="n">
-        <v>0.04253275180021647</v>
+        <v>0.04387881472944864</v>
       </c>
     </row>
     <row r="51">
@@ -2710,13 +2710,13 @@
         </is>
       </c>
       <c r="D51" s="7" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="E51" s="7" t="n">
         <v>1.3</v>
       </c>
-      <c r="E51" s="7" t="n">
-        <v>1.24</v>
-      </c>
       <c r="F51" s="8" t="n">
-        <v>0.04838709677419359</v>
+        <v>0.0307692307692308</v>
       </c>
       <c r="G51" s="9" t="n">
         <v>0.06</v>
@@ -2725,10 +2725,10 @@
         <v>46493</v>
       </c>
       <c r="I51" s="13" t="n">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="J51" s="10" t="n">
-        <v>46530</v>
+        <v>46531</v>
       </c>
       <c r="K51" s="12" t="inlineStr">
         <is>
@@ -2736,7 +2736,7 @@
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>0.02218998071717222</v>
+        <v>0.02409367805377783</v>
       </c>
     </row>
     <row r="52">
@@ -2771,7 +2771,7 @@
         <v>46499</v>
       </c>
       <c r="I52" s="13" t="n">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="J52" s="10" t="n">
         <v>46526</v>
@@ -2782,7 +2782,7 @@
         </is>
       </c>
       <c r="L52" s="9" t="n">
-        <v>0.02858911548315806</v>
+        <v>0.02828271494384326</v>
       </c>
     </row>
     <row r="53">
@@ -2817,7 +2817,7 @@
         <v>46508</v>
       </c>
       <c r="I53" s="13" t="n">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="J53" s="10" t="n">
         <v>46518</v>
@@ -2828,7 +2828,7 @@
         </is>
       </c>
       <c r="L53" s="9" t="n">
-        <v>0.04907216494845361</v>
+        <v>0.0472577605327386</v>
       </c>
     </row>
     <row r="54">
@@ -2863,7 +2863,7 @@
         <v>46517</v>
       </c>
       <c r="I54" s="13" t="n">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="J54" s="10" t="n">
         <v>46542</v>
@@ -2874,7 +2874,7 @@
         </is>
       </c>
       <c r="L54" s="9" t="n">
-        <v>0.03780301337001037</v>
+        <v>0.03954705853105136</v>
       </c>
     </row>
   </sheetData>
@@ -2909,7 +2909,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Expected Increase Announcements by Month - 05/25/2026</t>
+          <t>Expected Increase Announcements by Month - 06/01/2026</t>
         </is>
       </c>
     </row>
@@ -3100,10 +3100,10 @@
         <v>46264</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>1</v>
+        <v>1.03</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>0.05263157894736847</v>
+        <v>0.03000000000000003</v>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
         <v>46461</v>
       </c>
       <c r="C73" s="10" t="n">
-        <v>46196</v>
+        <v>46386</v>
       </c>
       <c r="D73" s="7" t="n">
         <v>0.271</v>
@@ -4432,13 +4432,13 @@
         <v>46493</v>
       </c>
       <c r="C81" s="10" t="n">
-        <v>46530</v>
+        <v>46531</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>1.3</v>
+        <v>1.34</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>0.04838709677419359</v>
+        <v>0.0307692307692308</v>
       </c>
       <c r="F81" s="12" t="inlineStr">
         <is>
@@ -4596,7 +4596,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete Holdings Dividend Summary - 05/25/2026</t>
+          <t>Complete Holdings Dividend Summary - 06/01/2026</t>
         </is>
       </c>
     </row>
@@ -4700,7 +4700,7 @@
         <v>1.16</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.01055793183764243</v>
+        <v>0.01035205922842178</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>46160</v>
@@ -4753,7 +4753,7 @@
         <v>10.08</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.02970822388048694</v>
+        <v>0.0304605330321046</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>46157</v>
@@ -4806,7 +4806,7 @@
         <v>12.708</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.007782472784615239</v>
+        <v>0.007991648467354199</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>46139</v>
@@ -4859,7 +4859,7 @@
         <v>2.812</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.03785166193761971</v>
+        <v>0.03916980030838525</v>
       </c>
       <c r="I8" s="10" t="n">
         <v>46157</v>
@@ -4906,19 +4906,19 @@
         </is>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1</v>
+        <v>1.03</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>4</v>
+        <v>4.12</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.02869852102073829</v>
+        <v>0.03043622674109861</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>46080</v>
+        <v>46171</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>0.05263157894736847</v>
+        <v>0.03000000000000003</v>
       </c>
       <c r="K9" s="10" t="n">
         <v>46232</v>
@@ -4965,7 +4965,7 @@
         <v>4.96</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.05215014160624624</v>
+        <v>0.05544997394320728</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>46134</v>
@@ -5018,7 +5018,7 @@
         <v>29.8</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.102324619290005</v>
+        <v>0.1111069719600328</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>46091</v>
@@ -5071,7 +5071,7 @@
         <v>0.92</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.02148026991987978</v>
+        <v>0.02198064771382014</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>46163</v>
@@ -5124,7 +5124,7 @@
         <v>2.4</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0.008730129744386562</v>
+        <v>0.008972130483968787</v>
       </c>
       <c r="I13" s="10" t="n">
         <v>46157</v>
@@ -5177,7 +5177,7 @@
         <v>1.68</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0.01395232911639436</v>
+        <v>0.01410579363160145</v>
       </c>
       <c r="I14" s="10" t="n">
         <v>46114</v>
@@ -5230,7 +5230,7 @@
         <v>7.12</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.0371937537084845</v>
+        <v>0.0382940836807255</v>
       </c>
       <c r="I15" s="10" t="n">
         <v>46161</v>
@@ -5283,7 +5283,7 @@
         <v>3.44</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.01762204744474112</v>
+        <v>0.01754699192598384</v>
       </c>
       <c r="I16" s="10" t="n">
         <v>46118</v>
@@ -5336,7 +5336,7 @@
         <v>0.96</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.02033036796236036</v>
+        <v>0.02049420985253447</v>
       </c>
       <c r="I17" s="10" t="n">
         <v>46094</v>
@@ -5389,7 +5389,7 @@
         <v>3.36</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.04533189254576684</v>
+        <v>0.04449447165672079</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>46094</v>
@@ -5442,7 +5442,7 @@
         <v>2.56</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.02277580040255237</v>
+        <v>0.023931943262468</v>
       </c>
       <c r="I19" s="10" t="n">
         <v>46143</v>
@@ -5495,7 +5495,7 @@
         <v>6.36</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.01854822166962447</v>
+        <v>0.01863408644778464</v>
       </c>
       <c r="I20" s="10" t="n">
         <v>46122</v>
@@ -5533,7 +5533,7 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Mar/Jun/Aug/Nov</t>
+          <t>Mar/Aug/Sep/Nov</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -5548,7 +5548,7 @@
         <v>9.32</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.02976969937062066</v>
+        <v>0.0298545717812205</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>46093</v>
@@ -5601,10 +5601,10 @@
         <v>5.52</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>0.01721610552954179</v>
+        <v>0.01850982488567165</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>46080</v>
+        <v>46171</v>
       </c>
       <c r="J22" s="8" t="n">
         <v>0.02222222222222208</v>
@@ -5654,7 +5654,7 @@
         <v>1.172</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.05517890831588747</v>
+        <v>0.0502572905376204</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>46125</v>
@@ -5707,7 +5707,7 @@
         <v>3.28</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>0.03202812110838314</v>
+        <v>0.03260437425199132</v>
       </c>
       <c r="I24" s="10" t="n">
         <v>46113</v>
@@ -5760,7 +5760,7 @@
         <v>2.44</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.01740495012131711</v>
+        <v>0.01771324863883848</v>
       </c>
       <c r="I25" s="10" t="n">
         <v>46086</v>
@@ -5807,25 +5807,25 @@
         </is>
       </c>
       <c r="F26" s="7" t="n">
-        <v>1.3</v>
+        <v>1.34</v>
       </c>
       <c r="G26" s="16" t="n">
-        <v>5.2</v>
+        <v>5.36</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>0.02218998071717222</v>
+        <v>0.02409367805377783</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>46077</v>
+        <v>46168</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>0.04838709677419359</v>
+        <v>0.0307692307692308</v>
       </c>
       <c r="K26" s="10" t="n">
         <v>46493</v>
       </c>
       <c r="L26" s="10" t="n">
-        <v>46530</v>
+        <v>46531</v>
       </c>
       <c r="M26" s="12" t="inlineStr">
         <is>
@@ -5866,7 +5866,7 @@
         <v>6</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.01958352341659811</v>
+        <v>0.02003974557693619</v>
       </c>
       <c r="I27" s="10" t="n">
         <v>46118</v>
@@ -5919,7 +5919,7 @@
         <v>2.174</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0.0202817422379329</v>
+        <v>0.0204872076875597</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>46132</v>
@@ -5972,7 +5972,7 @@
         <v>3.16</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.011995596886681</v>
+        <v>0.01247717304408395</v>
       </c>
       <c r="I29" s="10" t="n">
         <v>46112</v>
@@ -6025,7 +6025,7 @@
         <v>2.84</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.03613231622307302</v>
+        <v>0.03798822791396991</v>
       </c>
       <c r="I30" s="10" t="n">
         <v>46108</v>
@@ -6078,7 +6078,7 @@
         <v>1.92</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0.04016736465785078</v>
+        <v>0.0406177275525001</v>
       </c>
       <c r="I31" s="10" t="n">
         <v>46132</v>
@@ -6131,7 +6131,7 @@
         <v>3.64</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.008696275261740157</v>
+        <v>0.007827956989247311</v>
       </c>
       <c r="I32" s="10" t="n">
         <v>46163</v>
@@ -6184,7 +6184,7 @@
         <v>3.48</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0.03267605633802817</v>
+        <v>0.03207668972737766</v>
       </c>
       <c r="I33" s="10" t="n">
         <v>46120</v>
@@ -6237,7 +6237,7 @@
         <v>1.64</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0.03671367958864462</v>
+        <v>0.03578441925543904</v>
       </c>
       <c r="I34" s="10" t="n">
         <v>46083</v>
@@ -6290,7 +6290,7 @@
         <v>2.55</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0.05671708300547242</v>
+        <v>0.05704697889209416</v>
       </c>
       <c r="I35" s="10" t="n">
         <v>46111</v>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Dec</t>
         </is>
       </c>
       <c r="F36" s="7" t="n">
@@ -6343,10 +6343,10 @@
         <v>3.252</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0.05243469809734441</v>
+        <v>0.05379652537562463</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>46142</v>
+        <v>46171</v>
       </c>
       <c r="J36" s="8" t="n">
         <v>0.003703703703703707</v>
@@ -6355,7 +6355,7 @@
         <v>46461</v>
       </c>
       <c r="L36" s="10" t="n">
-        <v>46196</v>
+        <v>46386</v>
       </c>
       <c r="M36" s="12" t="inlineStr">
         <is>
@@ -6396,7 +6396,7 @@
         <v>4.76</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.04907216494845361</v>
+        <v>0.0472577605327386</v>
       </c>
       <c r="I37" s="10" t="n">
         <v>46155</v>
@@ -6449,7 +6449,7 @@
         <v>5.692</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0.03780301337001037</v>
+        <v>0.03954705853105136</v>
       </c>
       <c r="I38" s="10" t="n">
         <v>46087</v>
@@ -6502,7 +6502,7 @@
         <v>1.72</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.06640926738737934</v>
+        <v>0.06686882792307368</v>
       </c>
       <c r="I39" s="10" t="n">
         <v>46150</v>
@@ -6555,7 +6555,7 @@
         <v>3.2</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.03081367402039418</v>
+        <v>0.03104686144828515</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>46092</v>
@@ -6608,7 +6608,7 @@
         <v>4.356</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0.03015785050105535</v>
+        <v>0.03095728656212699</v>
       </c>
       <c r="I41" s="10" t="n">
         <v>46136</v>
@@ -6661,7 +6661,7 @@
         <v>2.1</v>
       </c>
       <c r="H42" s="9" t="n">
-        <v>0.04215174654483525</v>
+        <v>0.04247572933518482</v>
       </c>
       <c r="I42" s="10" t="n">
         <v>46104</v>
@@ -6714,7 +6714,7 @@
         <v>5.08</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0.02858911548315806</v>
+        <v>0.02828271494384326</v>
       </c>
       <c r="I43" s="10" t="n">
         <v>46160</v>
@@ -6767,7 +6767,7 @@
         <v>3.72</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.01737992953039871</v>
+        <v>0.01859581611162467</v>
       </c>
       <c r="I44" s="10" t="n">
         <v>46161</v>
@@ -6820,7 +6820,7 @@
         <v>9.76</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>0.02661939223366119</v>
+        <v>0.02652642468034239</v>
       </c>
       <c r="I45" s="10" t="n">
         <v>46162</v>
@@ -6873,7 +6873,7 @@
         <v>3.32</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.04342139732871405</v>
+        <v>0.04297178239972002</v>
       </c>
       <c r="I46" s="10" t="n">
         <v>46091</v>
@@ -6926,7 +6926,7 @@
         <v>5.2</v>
       </c>
       <c r="H47" s="9" t="n">
-        <v>0.05029499981330527</v>
+        <v>0.04959215180541567</v>
       </c>
       <c r="I47" s="10" t="n">
         <v>46097</v>
@@ -6979,7 +6979,7 @@
         <v>3.896</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>0.04253275180021647</v>
+        <v>0.04387881472944864</v>
       </c>
       <c r="I48" s="10" t="n">
         <v>46112</v>
@@ -7032,7 +7032,7 @@
         <v>5.68</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.01836939347681198</v>
+        <v>0.01952493873877673</v>
       </c>
       <c r="I49" s="10" t="n">
         <v>46147</v>
@@ -7085,7 +7085,7 @@
         <v>2.18</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.03801220676551045</v>
+        <v>0.03906109920010292</v>
       </c>
       <c r="I50" s="10" t="n">
         <v>46157</v>
@@ -7138,10 +7138,10 @@
         <v>5.52</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.02076124529346597</v>
+        <v>0.02116402056970356</v>
       </c>
       <c r="I51" s="10" t="n">
-        <v>46080</v>
+        <v>46171</v>
       </c>
       <c r="J51" s="8" t="n">
         <v>0.02985074626865658</v>
@@ -7191,7 +7191,7 @@
         <v>2.832</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.05857290774302305</v>
+        <v>0.05932132175180416</v>
       </c>
       <c r="I52" s="10" t="n">
         <v>46122</v>
@@ -7244,7 +7244,7 @@
         <v>4.12</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>0.02659437160273528</v>
+        <v>0.0276510067114094</v>
       </c>
       <c r="I53" s="10" t="n">
         <v>46157</v>

</xml_diff>

<commit_message>
Update dividend calendar 2026-06-29
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -561,7 +561,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estimated Dividend Calendar: Anticipated Announcements - 06/22/2026</t>
+          <t>Estimated Dividend Calendar: Anticipated Announcements - 06/29/2026</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         <v>46048</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-147</v>
+        <v>-154</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>46413</v>
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="L6" s="9" t="n">
-        <v>0.06873126977897696</v>
+        <v>0.07063654920140841</v>
       </c>
     </row>
     <row r="7">
@@ -712,7 +712,7 @@
         <v>46218</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>46248</v>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.01763534633993057</v>
+        <v>0.01731722625385386</v>
       </c>
     </row>
     <row r="8">
@@ -758,7 +758,7 @@
         <v>46220</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>46264</v>
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.02124752098652373</v>
+        <v>0.02030046090334901</v>
       </c>
     </row>
     <row r="9">
@@ -804,7 +804,7 @@
         <v>46227</v>
       </c>
       <c r="I9" s="20" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="J9" s="19" t="n">
         <v>46248</v>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="L9" s="18" t="n">
-        <v>0.02617162186093445</v>
+        <v>0.02451063829787234</v>
       </c>
     </row>
     <row r="10">
@@ -850,7 +850,7 @@
         <v>46227</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>46267</v>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.03782398111404369</v>
+        <v>0.0366304399155838</v>
       </c>
     </row>
     <row r="11">
@@ -896,7 +896,7 @@
         <v>46232</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46264</v>
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.02793220338983051</v>
+        <v>0.02656522082200493</v>
       </c>
     </row>
     <row r="12">
@@ -942,7 +942,7 @@
         <v>46232</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>46246</v>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0.05257857686051969</v>
+        <v>0.05151908513516609</v>
       </c>
     </row>
     <row r="13">
@@ -988,7 +988,7 @@
         <v>46263</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>46297</v>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>0.03371537109041089</v>
+        <v>0.03387554973798062</v>
       </c>
     </row>
     <row r="14">
@@ -1034,7 +1034,7 @@
         <v>46278</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>46344</v>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.009569377867591678</v>
+        <v>0.009613226387814601</v>
       </c>
     </row>
     <row r="15">
@@ -1080,7 +1080,7 @@
         <v>46280</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>46303</v>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>0.06219391697573379</v>
+        <v>0.06477481020832258</v>
       </c>
     </row>
     <row r="16">
@@ -1126,7 +1126,7 @@
         <v>46285</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>46325</v>
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="L16" s="9" t="n">
-        <v>0.01719830968486408</v>
+        <v>0.02014684548490726</v>
       </c>
     </row>
     <row r="17">
@@ -1172,7 +1172,7 @@
         <v>46305</v>
       </c>
       <c r="I17" s="13" t="n">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>46339</v>
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.02962206248349254</v>
+        <v>0.02976903297327682</v>
       </c>
     </row>
     <row r="18">
@@ -1218,7 +1218,7 @@
         <v>46311</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>46386</v>
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.01150366739745763</v>
+        <v>0.01183177102782167</v>
       </c>
     </row>
     <row r="19">
@@ -1264,7 +1264,7 @@
         <v>46317</v>
       </c>
       <c r="I19" s="13" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>46351</v>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0.01983043645094449</v>
+        <v>0.01960505770657732</v>
       </c>
     </row>
     <row r="20">
@@ -1310,7 +1310,7 @@
         <v>46322</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>46338</v>
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0.02287552422685487</v>
+        <v>0.02201724414764789</v>
       </c>
     </row>
     <row r="21">
@@ -1356,7 +1356,7 @@
         <v>46329</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46338</v>
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.008822718698096135</v>
+        <v>0.008374625278987521</v>
       </c>
     </row>
     <row r="22">
@@ -1402,7 +1402,7 @@
         <v>46332</v>
       </c>
       <c r="I22" s="13" t="n">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="J22" s="10" t="n">
         <v>46346</v>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="L22" s="9" t="n">
-        <v>0.02508836232408511</v>
+        <v>0.02468136743815182</v>
       </c>
     </row>
     <row r="23">
@@ -1448,7 +1448,7 @@
         <v>46341</v>
       </c>
       <c r="I23" s="13" t="n">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>46339</v>
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0.02998108030051665</v>
+        <v>0.03029189152561084</v>
       </c>
     </row>
     <row r="24">
@@ -1494,7 +1494,7 @@
         <v>46344</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="J24" s="10" t="n">
         <v>46385</v>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="L24" s="9" t="n">
-        <v>0.04147764013882235</v>
+        <v>0.03701918322307009</v>
       </c>
     </row>
     <row r="25">
@@ -1540,7 +1540,7 @@
         <v>46347</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>46358</v>
@@ -1551,7 +1551,7 @@
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>0.03697024295390339</v>
+        <v>0.04014196593747481</v>
       </c>
     </row>
     <row r="26">
@@ -1586,7 +1586,7 @@
         <v>46352</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>46400</v>
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0.04857024619816713</v>
+        <v>0.04419306107730098</v>
       </c>
     </row>
     <row r="27">
@@ -1632,7 +1632,7 @@
         <v>46360</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>46371</v>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="L27" s="9" t="n">
-        <v>0.0464088388009079</v>
+        <v>0.04904393366268946</v>
       </c>
     </row>
     <row r="28">
@@ -1678,7 +1678,7 @@
         <v>46366</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>46432</v>
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="L28" s="9" t="n">
-        <v>0.02948144216909636</v>
+        <v>0.02792475819572862</v>
       </c>
     </row>
     <row r="29">
@@ -1724,7 +1724,7 @@
         <v>46371</v>
       </c>
       <c r="I29" s="13" t="n">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>46344</v>
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>0.02141776186201622</v>
+        <v>0.02038103705005755</v>
       </c>
     </row>
     <row r="30">
@@ -1770,7 +1770,7 @@
         <v>46402</v>
       </c>
       <c r="I30" s="13" t="n">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="J30" s="10" t="n">
         <v>46483</v>
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="L30" s="9" t="n">
-        <v>0.01775667204802915</v>
+        <v>0.01647272886959504</v>
       </c>
     </row>
     <row r="31">
@@ -1816,7 +1816,7 @@
         <v>46411</v>
       </c>
       <c r="I31" s="13" t="n">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>46435</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="n">
-        <v>0.03865823594422466</v>
+        <v>0.0373687707641196</v>
       </c>
     </row>
     <row r="32">
@@ -1862,7 +1862,7 @@
         <v>46417</v>
       </c>
       <c r="I32" s="13" t="n">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>46433</v>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="L32" s="9" t="n">
-        <v>0.04095955775758391</v>
+        <v>0.04189467565667787</v>
       </c>
     </row>
     <row r="33">
@@ -1908,7 +1908,7 @@
         <v>46422</v>
       </c>
       <c r="I33" s="13" t="n">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>46472</v>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>0.05626667250263881</v>
+        <v>0.05293751498715974</v>
       </c>
     </row>
     <row r="34">
@@ -1954,7 +1954,7 @@
         <v>46428</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>46452</v>
@@ -1965,7 +1965,7 @@
         </is>
       </c>
       <c r="L34" s="9" t="n">
-        <v>0.01969330080670224</v>
+        <v>0.01789381042152013</v>
       </c>
     </row>
     <row r="35">
@@ -2000,7 +2000,7 @@
         <v>46428</v>
       </c>
       <c r="I35" s="13" t="n">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>46460</v>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0.0476364952871926</v>
+        <v>0.04650330901620179</v>
       </c>
     </row>
     <row r="36">
@@ -2046,7 +2046,7 @@
         <v>46431</v>
       </c>
       <c r="I36" s="13" t="n">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>46480</v>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="L36" s="9" t="n">
-        <v>0.01383741001009712</v>
+        <v>0.01444043366754725</v>
       </c>
     </row>
     <row r="37">
@@ -2092,7 +2092,7 @@
         <v>46432</v>
       </c>
       <c r="I37" s="13" t="n">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>46455</v>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>0.03346026542424558</v>
+        <v>0.03219606041300103</v>
       </c>
     </row>
     <row r="38">
@@ -2138,7 +2138,7 @@
         <v>46433</v>
       </c>
       <c r="I38" s="13" t="n">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>46425</v>
@@ -2149,7 +2149,7 @@
         </is>
       </c>
       <c r="L38" s="9" t="n">
-        <v>0.006605229735607282</v>
+        <v>0.007051303507108543</v>
       </c>
     </row>
     <row r="39">
@@ -2184,7 +2184,7 @@
         <v>46433</v>
       </c>
       <c r="I39" s="13" t="n">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>46383</v>
@@ -2195,7 +2195,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.02108763565929368</v>
+        <v>0.02338576410879153</v>
       </c>
     </row>
     <row r="40">
@@ -2230,7 +2230,7 @@
         <v>46433</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="J40" s="10" t="n">
         <v>46368</v>
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.0301460204333374</v>
+        <v>0.0299976577203504</v>
       </c>
     </row>
     <row r="41">
@@ -2276,7 +2276,7 @@
         <v>46433</v>
       </c>
       <c r="I41" s="13" t="n">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>46270</v>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>0.02958686615498475</v>
+        <v>0.03064847788156331</v>
       </c>
     </row>
     <row r="42">
@@ -2322,7 +2322,7 @@
         <v>46433</v>
       </c>
       <c r="I42" s="13" t="n">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="J42" s="10" t="n">
         <v>46243</v>
@@ -2333,7 +2333,7 @@
         </is>
       </c>
       <c r="L42" s="9" t="n">
-        <v>0.03775872481084097</v>
+        <v>0.03599735717577861</v>
       </c>
     </row>
     <row r="43">
@@ -2368,7 +2368,7 @@
         <v>46440</v>
       </c>
       <c r="I43" s="13" t="n">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>46450</v>
@@ -2379,7 +2379,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>0.009718498609821541</v>
+        <v>0.009721756645716097</v>
       </c>
     </row>
     <row r="44">
@@ -2414,7 +2414,7 @@
         <v>46441</v>
       </c>
       <c r="I44" s="13" t="n">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="J44" s="10" t="n">
         <v>46456</v>
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="L44" s="9" t="n">
-        <v>0.02825055708305586</v>
+        <v>0.02690880658391252</v>
       </c>
     </row>
     <row r="45">
@@ -2460,7 +2460,7 @@
         <v>46452</v>
       </c>
       <c r="I45" s="13" t="n">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="J45" s="10" t="n">
         <v>46487</v>
@@ -2471,7 +2471,7 @@
         </is>
       </c>
       <c r="L45" s="9" t="n">
-        <v>0.0184674343897353</v>
+        <v>0.01815975412709446</v>
       </c>
     </row>
     <row r="46">
@@ -2506,7 +2506,7 @@
         <v>46461</v>
       </c>
       <c r="I46" s="13" t="n">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="J46" s="10" t="n">
         <v>46300</v>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="L46" s="9" t="n">
-        <v>0.0183281663555542</v>
+        <v>0.01821161948526943</v>
       </c>
     </row>
     <row r="47">
@@ -2552,7 +2552,7 @@
         <v>46461</v>
       </c>
       <c r="I47" s="13" t="n">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="J47" s="10" t="n">
         <v>46386</v>
@@ -2563,7 +2563,7 @@
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>0.0538588927206442</v>
+        <v>0.05195294805937987</v>
       </c>
     </row>
     <row r="48">
@@ -2598,7 +2598,7 @@
         <v>46488</v>
       </c>
       <c r="I48" s="13" t="n">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="J48" s="10" t="n">
         <v>46498</v>
@@ -2609,7 +2609,7 @@
         </is>
       </c>
       <c r="L48" s="9" t="n">
-        <v>0.02920745620106488</v>
+        <v>0.02944038795851004</v>
       </c>
     </row>
     <row r="49">
@@ -2644,7 +2644,7 @@
         <v>46492</v>
       </c>
       <c r="I49" s="13" t="n">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>46501</v>
@@ -2655,13 +2655,13 @@
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>0.0203615254130588</v>
+        <v>0.02013615591849956</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>POR</t>
+          <t>TTE</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
@@ -2671,43 +2671,43 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Dec</t>
         </is>
       </c>
       <c r="D50" s="7" t="n">
-        <v>0.525</v>
+        <v>0.974</v>
       </c>
       <c r="E50" s="7" t="n">
-        <v>0.5</v>
+        <v>0.994</v>
       </c>
       <c r="F50" s="8" t="n">
-        <v>0.05000000000000004</v>
+        <v>0.001006036217303824</v>
       </c>
       <c r="G50" s="9" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="H50" s="10" t="n">
         <v>46492</v>
       </c>
       <c r="I50" s="13" t="n">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="J50" s="10" t="n">
-        <v>46562</v>
+        <v>46376</v>
       </c>
       <c r="K50" s="12" t="inlineStr">
         <is>
-          <t>yfinance</t>
+          <t>Notion + yfinance</t>
         </is>
       </c>
       <c r="L50" s="9" t="n">
-        <v>0.04170390267283352</v>
+        <v>0.0498018641546523</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
@@ -2717,29 +2717,29 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Dec</t>
+          <t>May</t>
         </is>
       </c>
       <c r="D51" s="7" t="n">
-        <v>0.974</v>
+        <v>1.34</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>0.994</v>
+        <v>1.3</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>0.001006036217303824</v>
+        <v>0.0307692307692308</v>
       </c>
       <c r="G51" s="9" t="n">
         <v>0.06</v>
       </c>
       <c r="H51" s="10" t="n">
-        <v>46492</v>
+        <v>46493</v>
       </c>
       <c r="I51" s="13" t="n">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="J51" s="10" t="n">
-        <v>46376</v>
+        <v>46531</v>
       </c>
       <c r="K51" s="12" t="inlineStr">
         <is>
@@ -2747,13 +2747,13 @@
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>0.0483915028769668</v>
+        <v>0.02100025461704885</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>PSX</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -2767,25 +2767,25 @@
         </is>
       </c>
       <c r="D52" s="7" t="n">
-        <v>1.34</v>
+        <v>1.27</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="F52" s="8" t="n">
-        <v>0.0307692307692308</v>
+        <v>0.05833333333333339</v>
       </c>
       <c r="G52" s="9" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="H52" s="10" t="n">
-        <v>46493</v>
+        <v>46499</v>
       </c>
       <c r="I52" s="13" t="n">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J52" s="10" t="n">
-        <v>46531</v>
+        <v>46526</v>
       </c>
       <c r="K52" s="12" t="inlineStr">
         <is>
@@ -2793,13 +2793,13 @@
         </is>
       </c>
       <c r="L52" s="9" t="n">
-        <v>0.02339538683117294</v>
+        <v>0.02889236506851984</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>PSX</t>
+          <t>POR</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -2809,29 +2809,29 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
-        <v>1.27</v>
+        <v>0.551</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>1.2</v>
+        <v>0.525</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>0.05833333333333339</v>
+        <v>0.04952380952380957</v>
       </c>
       <c r="G53" s="9" t="n">
         <v>0.04</v>
       </c>
       <c r="H53" s="10" t="n">
-        <v>46499</v>
+        <v>46504</v>
       </c>
       <c r="I53" s="13" t="n">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="J53" s="10" t="n">
-        <v>46526</v>
+        <v>46562</v>
       </c>
       <c r="K53" s="12" t="inlineStr">
         <is>
@@ -2839,7 +2839,7 @@
         </is>
       </c>
       <c r="L53" s="9" t="n">
-        <v>0.03053068104233697</v>
+        <v>0.04219797088486882</v>
       </c>
     </row>
     <row r="54">
@@ -2874,7 +2874,7 @@
         <v>46508</v>
       </c>
       <c r="I54" s="13" t="n">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="J54" s="10" t="n">
         <v>46518</v>
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="L54" s="9" t="n">
-        <v>0.04844290552121706</v>
+        <v>0.04748129675810474</v>
       </c>
     </row>
     <row r="55">
@@ -2920,7 +2920,7 @@
         <v>46515</v>
       </c>
       <c r="I55" s="13" t="n">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="J55" s="10" t="n">
         <v>46542</v>
@@ -2931,7 +2931,7 @@
         </is>
       </c>
       <c r="L55" s="9" t="n">
-        <v>0.0417518885698331</v>
+        <v>0.042147228513663</v>
       </c>
     </row>
     <row r="56">
@@ -2951,22 +2951,22 @@
         </is>
       </c>
       <c r="D56" s="7" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="E56" s="7" t="n">
         <v>0.71</v>
       </c>
-      <c r="E56" s="7" t="n">
-        <v>0.7</v>
-      </c>
       <c r="F56" s="8" t="n">
-        <v>0.0142857142857143</v>
+        <v>0.01408450704225353</v>
       </c>
       <c r="G56" s="9" t="n">
         <v>0.08</v>
       </c>
       <c r="H56" s="10" t="n">
-        <v>46527</v>
+        <v>46532</v>
       </c>
       <c r="I56" s="13" t="n">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J56" s="10" t="n">
         <v>46563</v>
@@ -2977,7 +2977,7 @@
         </is>
       </c>
       <c r="L56" s="9" t="n">
-        <v>0.03593581136590545</v>
+        <v>0.03548983297408272</v>
       </c>
     </row>
   </sheetData>
@@ -3012,7 +3012,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Expected Increase Announcements by Month - 06/22/2026</t>
+          <t>Expected Increase Announcements by Month - 06/29/2026</t>
         </is>
       </c>
     </row>
@@ -4504,44 +4504,44 @@
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>POR</t>
+          <t>TTE</t>
         </is>
       </c>
       <c r="B80" s="10" t="n">
         <v>46492</v>
       </c>
       <c r="C80" s="10" t="n">
-        <v>46562</v>
+        <v>46376</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>0.525</v>
+        <v>0.974</v>
       </c>
       <c r="E80" s="8" t="n">
-        <v>0.05000000000000004</v>
+        <v>0.001006036217303824</v>
       </c>
       <c r="F80" s="12" t="inlineStr">
         <is>
-          <t>yfinance</t>
+          <t>Notion + yfinance</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="B81" s="10" t="n">
-        <v>46492</v>
+        <v>46493</v>
       </c>
       <c r="C81" s="10" t="n">
-        <v>46376</v>
+        <v>46531</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>0.974</v>
+        <v>1.34</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>0.001006036217303824</v>
+        <v>0.0307692307692308</v>
       </c>
       <c r="F81" s="12" t="inlineStr">
         <is>
@@ -4552,20 +4552,20 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>PSX</t>
         </is>
       </c>
       <c r="B82" s="10" t="n">
-        <v>46493</v>
+        <v>46499</v>
       </c>
       <c r="C82" s="10" t="n">
-        <v>46531</v>
+        <v>46526</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>1.34</v>
+        <v>1.27</v>
       </c>
       <c r="E82" s="8" t="n">
-        <v>0.0307692307692308</v>
+        <v>0.05833333333333339</v>
       </c>
       <c r="F82" s="12" t="inlineStr">
         <is>
@@ -4576,20 +4576,20 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>PSX</t>
+          <t>POR</t>
         </is>
       </c>
       <c r="B83" s="10" t="n">
-        <v>46499</v>
+        <v>46504</v>
       </c>
       <c r="C83" s="10" t="n">
-        <v>46526</v>
+        <v>46562</v>
       </c>
       <c r="D83" s="7" t="n">
-        <v>1.27</v>
+        <v>0.551</v>
       </c>
       <c r="E83" s="8" t="n">
-        <v>0.05833333333333339</v>
+        <v>0.04952380952380957</v>
       </c>
       <c r="F83" s="12" t="inlineStr">
         <is>
@@ -4691,16 +4691,16 @@
         </is>
       </c>
       <c r="B89" s="10" t="n">
-        <v>46527</v>
+        <v>46532</v>
       </c>
       <c r="C89" s="10" t="n">
         <v>46563</v>
       </c>
       <c r="D89" s="7" t="n">
-        <v>0.71</v>
+        <v>0.72</v>
       </c>
       <c r="E89" s="8" t="n">
-        <v>0.0142857142857143</v>
+        <v>0.01408450704225353</v>
       </c>
       <c r="F89" s="12" t="inlineStr">
         <is>
@@ -4747,7 +4747,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete Holdings Dividend Summary - 06/22/2026</t>
+          <t>Complete Holdings Dividend Summary - 06/29/2026</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
         <v>1.16</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.009718498609821541</v>
+        <v>0.009721756645716097</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>46160</v>
@@ -4904,7 +4904,7 @@
         <v>10.08</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.02948144216909636</v>
+        <v>0.02792475819572862</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>46157</v>
@@ -4957,7 +4957,7 @@
         <v>12.708</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.006605229735607282</v>
+        <v>0.007051303507108543</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>46139</v>
@@ -5010,7 +5010,7 @@
         <v>2.016</v>
       </c>
       <c r="H8" s="18" t="n">
-        <v>0.02617162186093445</v>
+        <v>0.02451063829787234</v>
       </c>
       <c r="I8" s="19" t="n">
         <v>46160</v>
@@ -5063,7 +5063,7 @@
         <v>2.812</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.03865823594422466</v>
+        <v>0.0373687707641196</v>
       </c>
       <c r="I9" s="10" t="n">
         <v>46157</v>
@@ -5116,7 +5116,7 @@
         <v>4.12</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.02793220338983051</v>
+        <v>0.02656522082200493</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>46171</v>
@@ -5169,7 +5169,7 @@
         <v>4.96</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.05257857686051969</v>
+        <v>0.05151908513516609</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>46134</v>
@@ -5222,7 +5222,7 @@
         <v>5.2</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.02108763565929368</v>
+        <v>0.02338576410879153</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>46182</v>
@@ -5275,7 +5275,7 @@
         <v>0.92</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0.02141776186201622</v>
+        <v>0.02038103705005755</v>
       </c>
       <c r="I13" s="10" t="n">
         <v>46163</v>
@@ -5328,7 +5328,7 @@
         <v>2.4</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0.008822718698096135</v>
+        <v>0.008374625278987521</v>
       </c>
       <c r="I14" s="10" t="n">
         <v>46157</v>
@@ -5381,7 +5381,7 @@
         <v>1.68</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.01383741001009712</v>
+        <v>0.01444043366754725</v>
       </c>
       <c r="I15" s="10" t="n">
         <v>46114</v>
@@ -5434,7 +5434,7 @@
         <v>7.12</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.04095955775758391</v>
+        <v>0.04189467565667787</v>
       </c>
       <c r="I16" s="10" t="n">
         <v>46161</v>
@@ -5487,7 +5487,7 @@
         <v>3.44</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.01775667204802915</v>
+        <v>0.01647272886959504</v>
       </c>
       <c r="I17" s="10" t="n">
         <v>46118</v>
@@ -5540,7 +5540,7 @@
         <v>1.28</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.0301460204333374</v>
+        <v>0.0299976577203504</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>46188</v>
@@ -5593,7 +5593,7 @@
         <v>3.36</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.0464088388009079</v>
+        <v>0.04904393366268946</v>
       </c>
       <c r="I19" s="10" t="n">
         <v>46188</v>
@@ -5646,7 +5646,7 @@
         <v>2.56</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.02287552422685487</v>
+        <v>0.02201724414764789</v>
       </c>
       <c r="I20" s="10" t="n">
         <v>46143</v>
@@ -5699,7 +5699,7 @@
         <v>6.36</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.0184674343897353</v>
+        <v>0.01815975412709446</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>46122</v>
@@ -5752,7 +5752,7 @@
         <v>9.32</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>0.02825055708305586</v>
+        <v>0.02690880658391252</v>
       </c>
       <c r="I22" s="10" t="n">
         <v>46177</v>
@@ -5805,7 +5805,7 @@
         <v>5.52</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.01983043645094449</v>
+        <v>0.01960505770657732</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>46171</v>
@@ -5858,7 +5858,7 @@
         <v>1.172</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>0.04857024619816713</v>
+        <v>0.04419306107730098</v>
       </c>
       <c r="I24" s="10" t="n">
         <v>46125</v>
@@ -5911,7 +5911,7 @@
         <v>3.28</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.03371537109041089</v>
+        <v>0.03387554973798062</v>
       </c>
       <c r="I25" s="10" t="n">
         <v>46113</v>
@@ -5964,7 +5964,7 @@
         <v>2.44</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>0.01969330080670224</v>
+        <v>0.01789381042152013</v>
       </c>
       <c r="I26" s="10" t="n">
         <v>46174</v>
@@ -6017,7 +6017,7 @@
         <v>5.36</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.02339538683117294</v>
+        <v>0.02100025461704885</v>
       </c>
       <c r="I27" s="10" t="n">
         <v>46168</v>
@@ -6070,7 +6070,7 @@
         <v>6</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0.0183281663555542</v>
+        <v>0.01821161948526943</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>46118</v>
@@ -6123,7 +6123,7 @@
         <v>2.174</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.0203615254130588</v>
+        <v>0.02013615591849956</v>
       </c>
       <c r="I29" s="10" t="n">
         <v>46132</v>
@@ -6176,7 +6176,7 @@
         <v>3.16</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.01150366739745763</v>
+        <v>0.01183177102782167</v>
       </c>
       <c r="I30" s="10" t="n">
         <v>46112</v>
@@ -6223,22 +6223,22 @@
         </is>
       </c>
       <c r="F31" s="7" t="n">
-        <v>0.71</v>
+        <v>0.72</v>
       </c>
       <c r="G31" s="24" t="n">
-        <v>2.84</v>
+        <v>2.88</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0.03593581136590545</v>
+        <v>0.03548983297408272</v>
       </c>
       <c r="I31" s="10" t="n">
-        <v>46108</v>
+        <v>46199</v>
       </c>
       <c r="J31" s="8" t="n">
-        <v>0.0142857142857143</v>
+        <v>0.01408450704225353</v>
       </c>
       <c r="K31" s="10" t="n">
-        <v>46527</v>
+        <v>46532</v>
       </c>
       <c r="L31" s="10" t="n">
         <v>46563</v>
@@ -6282,7 +6282,7 @@
         <v>1.92</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.04147764013882235</v>
+        <v>0.03701918322307009</v>
       </c>
       <c r="I32" s="10" t="n">
         <v>46132</v>
@@ -6335,7 +6335,7 @@
         <v>3.64</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0.009569377867591678</v>
+        <v>0.009613226387814601</v>
       </c>
       <c r="I33" s="10" t="n">
         <v>46163</v>
@@ -6388,7 +6388,7 @@
         <v>3.48</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0.02962206248349254</v>
+        <v>0.02976903297327682</v>
       </c>
       <c r="I34" s="10" t="n">
         <v>46120</v>
@@ -6441,7 +6441,7 @@
         <v>1.64</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0.03697024295390339</v>
+        <v>0.04014196593747481</v>
       </c>
       <c r="I35" s="10" t="n">
         <v>46174</v>
@@ -6494,7 +6494,7 @@
         <v>2.55</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0.05626667250263881</v>
+        <v>0.05293751498715974</v>
       </c>
       <c r="I36" s="10" t="n">
         <v>46111</v>
@@ -6547,7 +6547,7 @@
         <v>3.252</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.0538588927206442</v>
+        <v>0.05195294805937987</v>
       </c>
       <c r="I37" s="10" t="n">
         <v>46171</v>
@@ -6600,7 +6600,7 @@
         <v>4.76</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0.04844290552121706</v>
+        <v>0.04748129675810474</v>
       </c>
       <c r="I38" s="10" t="n">
         <v>46155</v>
@@ -6653,7 +6653,7 @@
         <v>2.68</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.03346026542424558</v>
+        <v>0.03219606041300103</v>
       </c>
       <c r="I39" s="10" t="n">
         <v>46182</v>
@@ -6706,7 +6706,7 @@
         <v>5.92</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.0417518885698331</v>
+        <v>0.042147228513663</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>46178</v>
@@ -6759,7 +6759,7 @@
         <v>1.72</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0.06873126977897696</v>
+        <v>0.07063654920140841</v>
       </c>
       <c r="I41" s="10" t="n">
         <v>46150</v>
@@ -6812,7 +6812,7 @@
         <v>3.28</v>
       </c>
       <c r="H42" s="9" t="n">
-        <v>0.02958686615498475</v>
+        <v>0.03064847788156331</v>
       </c>
       <c r="I42" s="10" t="n">
         <v>46174</v>
@@ -6865,7 +6865,7 @@
         <v>4.356</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0.02920745620106488</v>
+        <v>0.02944038795851004</v>
       </c>
       <c r="I43" s="10" t="n">
         <v>46136</v>
@@ -6912,29 +6912,29 @@
         </is>
       </c>
       <c r="F44" s="7" t="n">
-        <v>0.525</v>
+        <v>0.551</v>
       </c>
       <c r="G44" s="24" t="n">
-        <v>2.1</v>
+        <v>2.204</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.04170390267283352</v>
+        <v>0.04219797088486882</v>
       </c>
       <c r="I44" s="10" t="n">
-        <v>46104</v>
+        <v>46198</v>
       </c>
       <c r="J44" s="8" t="n">
-        <v>0.05000000000000004</v>
+        <v>0.04952380952380957</v>
       </c>
       <c r="K44" s="10" t="n">
-        <v>46492</v>
+        <v>46504</v>
       </c>
       <c r="L44" s="10" t="n">
         <v>46562</v>
       </c>
       <c r="M44" s="12" t="inlineStr">
         <is>
-          <t>yfinance</t>
+          <t>Notion + yfinance</t>
         </is>
       </c>
     </row>
@@ -6971,7 +6971,7 @@
         <v>5.08</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>0.03053068104233697</v>
+        <v>0.02889236506851984</v>
       </c>
       <c r="I45" s="10" t="n">
         <v>46160</v>
@@ -7024,7 +7024,7 @@
         <v>3.72</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.01763534633993057</v>
+        <v>0.01731722625385386</v>
       </c>
       <c r="I46" s="10" t="n">
         <v>46161</v>
@@ -7077,7 +7077,7 @@
         <v>9.76</v>
       </c>
       <c r="H47" s="9" t="n">
-        <v>0.02508836232408511</v>
+        <v>0.02468136743815182</v>
       </c>
       <c r="I47" s="10" t="n">
         <v>46162</v>
@@ -7130,7 +7130,7 @@
         <v>3.32</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>0.03782398111404369</v>
+        <v>0.0366304399155838</v>
       </c>
       <c r="I48" s="10" t="n">
         <v>46181</v>
@@ -7183,7 +7183,7 @@
         <v>5.2</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.0476364952871926</v>
+        <v>0.04650330901620179</v>
       </c>
       <c r="I49" s="10" t="n">
         <v>46188</v>
@@ -7236,7 +7236,7 @@
         <v>3.896</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.0483915028769668</v>
+        <v>0.0498018641546523</v>
       </c>
       <c r="I50" s="10" t="n">
         <v>46112</v>
@@ -7289,7 +7289,7 @@
         <v>5.68</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.01719830968486408</v>
+        <v>0.02014684548490726</v>
       </c>
       <c r="I51" s="10" t="n">
         <v>46147</v>
@@ -7342,7 +7342,7 @@
         <v>2.18</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.03775872481084097</v>
+        <v>0.03599735717577861</v>
       </c>
       <c r="I52" s="10" t="n">
         <v>46157</v>
@@ -7395,7 +7395,7 @@
         <v>5.52</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>0.02124752098652373</v>
+        <v>0.02030046090334901</v>
       </c>
       <c r="I53" s="10" t="n">
         <v>46171</v>
@@ -7448,7 +7448,7 @@
         <v>2.832</v>
       </c>
       <c r="H54" s="9" t="n">
-        <v>0.06219391697573379</v>
+        <v>0.06477481020832258</v>
       </c>
       <c r="I54" s="10" t="n">
         <v>46122</v>
@@ -7501,7 +7501,7 @@
         <v>4.12</v>
       </c>
       <c r="H55" s="9" t="n">
-        <v>0.02998108030051665</v>
+        <v>0.03029189152561084</v>
       </c>
       <c r="I55" s="10" t="n">
         <v>46157</v>

</xml_diff>

<commit_message>
Update dividend calendar 2026-07-13
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -145,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -172,11 +172,14 @@
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -575,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estimated Dividend Calendar: Anticipated Announcements - 07/06/2026</t>
+          <t>Estimated Dividend Calendar: Anticipated Announcements - 07/13/2026</t>
         </is>
       </c>
     </row>
@@ -680,7 +683,7 @@
         <v>46048</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-161</v>
+        <v>-168</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>46413</v>
@@ -691,7 +694,7 @@
         </is>
       </c>
       <c r="L6" s="9" t="n">
-        <v>0.07243629981928987</v>
+        <v>0.06981936204666597</v>
       </c>
     </row>
     <row r="7">
@@ -726,7 +729,7 @@
         <v>46218</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>46248</v>
@@ -737,7 +740,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.01674921160635266</v>
+        <v>0.01586015754252245</v>
       </c>
     </row>
     <row r="8">
@@ -772,7 +775,7 @@
         <v>46220</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>46264</v>
@@ -783,7 +786,7 @@
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.01950736818810225</v>
+        <v>0.0191056338898471</v>
       </c>
     </row>
     <row r="9">
@@ -818,7 +821,7 @@
         <v>46227</v>
       </c>
       <c r="I9" s="20" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="J9" s="19" t="n">
         <v>46248</v>
@@ -829,7 +832,7 @@
         </is>
       </c>
       <c r="L9" s="18" t="n">
-        <v>0.02398429590958984</v>
+        <v>0.02358722325034518</v>
       </c>
     </row>
     <row r="10">
@@ -863,8 +866,8 @@
       <c r="H10" s="10" t="n">
         <v>46227</v>
       </c>
-      <c r="I10" s="22" t="n">
-        <v>18</v>
+      <c r="I10" s="13" t="n">
+        <v>11</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>46267</v>
@@ -875,7 +878,7 @@
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.03601062976288923</v>
+        <v>0.03744008892858095</v>
       </c>
     </row>
     <row r="11">
@@ -910,7 +913,7 @@
         <v>46232</v>
       </c>
       <c r="I11" s="22" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46264</v>
@@ -921,7 +924,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.02647389558232932</v>
+        <v>0.02615374869501659</v>
       </c>
     </row>
     <row r="12">
@@ -956,7 +959,7 @@
         <v>46232</v>
       </c>
       <c r="I12" s="22" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>46246</v>
@@ -967,7 +970,7 @@
         </is>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0.05178804407181118</v>
+        <v>0.05128205063482052</v>
       </c>
     </row>
     <row r="13">
@@ -1002,7 +1005,7 @@
         <v>46263</v>
       </c>
       <c r="I13" s="22" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>46297</v>
@@ -1013,7 +1016,7 @@
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>0.03396144718830089</v>
+        <v>0.03269048716727996</v>
       </c>
     </row>
     <row r="14">
@@ -1048,7 +1051,7 @@
         <v>46278</v>
       </c>
       <c r="I14" s="22" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>46344</v>
@@ -1059,7 +1062,7 @@
         </is>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.009451599621287882</v>
+        <v>0.009398884557615285</v>
       </c>
     </row>
     <row r="15">
@@ -1094,7 +1097,7 @@
         <v>46280</v>
       </c>
       <c r="I15" s="22" t="n">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>46303</v>
@@ -1105,7 +1108,7 @@
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>0.06707721265084407</v>
+        <v>0.06631898910307311</v>
       </c>
     </row>
     <row r="16">
@@ -1140,7 +1143,7 @@
         <v>46285</v>
       </c>
       <c r="I16" s="22" t="n">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>46325</v>
@@ -1151,7 +1154,7 @@
         </is>
       </c>
       <c r="L16" s="9" t="n">
-        <v>0.01867254003883344</v>
+        <v>0.01881667089258208</v>
       </c>
     </row>
     <row r="17">
@@ -1186,7 +1189,7 @@
         <v>46305</v>
       </c>
       <c r="I17" s="22" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>46339</v>
@@ -1197,7 +1200,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.02871523995292049</v>
+        <v>0.02772466613344378</v>
       </c>
     </row>
     <row r="18">
@@ -1232,7 +1235,7 @@
         <v>46311</v>
       </c>
       <c r="I18" s="22" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>46386</v>
@@ -1243,7 +1246,7 @@
         </is>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.01222579016936565</v>
+        <v>0.01243017852579043</v>
       </c>
     </row>
     <row r="19">
@@ -1278,7 +1281,7 @@
         <v>46317</v>
       </c>
       <c r="I19" s="22" t="n">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>46351</v>
@@ -1289,7 +1292,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0.01891447392155589</v>
+        <v>0.01918932048156368</v>
       </c>
     </row>
     <row r="20">
@@ -1324,7 +1327,7 @@
         <v>46322</v>
       </c>
       <c r="I20" s="22" t="n">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>46338</v>
@@ -1335,7 +1338,7 @@
         </is>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0.0223122847115672</v>
+        <v>0.02204615862425437</v>
       </c>
     </row>
     <row r="21">
@@ -1370,7 +1373,7 @@
         <v>46329</v>
       </c>
       <c r="I21" s="22" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46338</v>
@@ -1381,7 +1384,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.008169517657604557</v>
+        <v>0.007805259164950651</v>
       </c>
     </row>
     <row r="22">
@@ -1416,7 +1419,7 @@
         <v>46332</v>
       </c>
       <c r="I22" s="22" t="n">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J22" s="10" t="n">
         <v>46346</v>
@@ -1427,7 +1430,7 @@
         </is>
       </c>
       <c r="L22" s="9" t="n">
-        <v>0.02366835262725075</v>
+        <v>0.02413332593824269</v>
       </c>
     </row>
     <row r="23">
@@ -1462,7 +1465,7 @@
         <v>46341</v>
       </c>
       <c r="I23" s="22" t="n">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>46339</v>
@@ -1473,7 +1476,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0.03013899116296197</v>
+        <v>0.02883740561914779</v>
       </c>
     </row>
     <row r="24">
@@ -1508,7 +1511,7 @@
         <v>46344</v>
       </c>
       <c r="I24" s="22" t="n">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="J24" s="10" t="n">
         <v>46385</v>
@@ -1519,7 +1522,7 @@
         </is>
       </c>
       <c r="L24" s="9" t="n">
-        <v>0.03727793340807439</v>
+        <v>0.03590798496665439</v>
       </c>
     </row>
     <row r="25">
@@ -1554,7 +1557,7 @@
         <v>46347</v>
       </c>
       <c r="I25" s="22" t="n">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>46358</v>
@@ -1565,7 +1568,7 @@
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>0.03838502185069386</v>
+        <v>0.03671778722453514</v>
       </c>
     </row>
     <row r="26">
@@ -1600,7 +1603,7 @@
         <v>46352</v>
       </c>
       <c r="I26" s="22" t="n">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>46400</v>
@@ -1611,7 +1614,7 @@
         </is>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0.04816108666911</v>
+        <v>0.0475552841643708</v>
       </c>
     </row>
     <row r="27">
@@ -1646,7 +1649,7 @@
         <v>46360</v>
       </c>
       <c r="I27" s="22" t="n">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>46371</v>
@@ -1657,7 +1660,7 @@
         </is>
       </c>
       <c r="L27" s="9" t="n">
-        <v>0.0491947269380616</v>
+        <v>0.04913358039101189</v>
       </c>
     </row>
     <row r="28">
@@ -1692,7 +1695,7 @@
         <v>46366</v>
       </c>
       <c r="I28" s="22" t="n">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>46432</v>
@@ -1703,7 +1706,7 @@
         </is>
       </c>
       <c r="L28" s="9" t="n">
-        <v>0.02790465823278872</v>
+        <v>0.02787263837801698</v>
       </c>
     </row>
     <row r="29">
@@ -1738,7 +1741,7 @@
         <v>46371</v>
       </c>
       <c r="I29" s="22" t="n">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>46344</v>
@@ -1749,7 +1752,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>0.02077922006309264</v>
+        <v>0.02089959087762214</v>
       </c>
     </row>
     <row r="30">
@@ -1783,8 +1786,8 @@
       <c r="H30" s="19" t="n">
         <v>46383</v>
       </c>
-      <c r="I30" s="20" t="n">
-        <v>174</v>
+      <c r="I30" s="23" t="n">
+        <v>167</v>
       </c>
       <c r="J30" s="19" t="n">
         <v>46404</v>
@@ -1795,7 +1798,7 @@
         </is>
       </c>
       <c r="L30" s="18" t="n">
-        <v>0.01574908177427583</v>
+        <v>0.01576907618770492</v>
       </c>
     </row>
     <row r="31">
@@ -1830,7 +1833,7 @@
         <v>46402</v>
       </c>
       <c r="I31" s="22" t="n">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>46483</v>
@@ -1841,7 +1844,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="n">
-        <v>0.01611920688332178</v>
+        <v>0.01638173203491813</v>
       </c>
     </row>
     <row r="32">
@@ -1876,7 +1879,7 @@
         <v>46411</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>46435</v>
@@ -1887,7 +1890,7 @@
         </is>
       </c>
       <c r="L32" s="9" t="n">
-        <v>0.03827152172028183</v>
+        <v>0.03690046496205276</v>
       </c>
     </row>
     <row r="33">
@@ -1922,7 +1925,7 @@
         <v>46417</v>
       </c>
       <c r="I33" s="22" t="n">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>46433</v>
@@ -1933,7 +1936,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>0.04217010278625639</v>
+        <v>0.03954566954044979</v>
       </c>
     </row>
     <row r="34">
@@ -1968,7 +1971,7 @@
         <v>46422</v>
       </c>
       <c r="I34" s="22" t="n">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>46472</v>
@@ -1979,7 +1982,7 @@
         </is>
       </c>
       <c r="L34" s="9" t="n">
-        <v>0.05230232682053303</v>
+        <v>0.05161421036343746</v>
       </c>
     </row>
     <row r="35">
@@ -2014,7 +2017,7 @@
         <v>46428</v>
       </c>
       <c r="I35" s="22" t="n">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>46452</v>
@@ -2025,7 +2028,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0.01677321770485241</v>
+        <v>0.01603364514018875</v>
       </c>
     </row>
     <row r="36">
@@ -2060,7 +2063,7 @@
         <v>46428</v>
       </c>
       <c r="I36" s="22" t="n">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>46460</v>
@@ -2071,7 +2074,7 @@
         </is>
       </c>
       <c r="L36" s="9" t="n">
-        <v>0.04387260015233685</v>
+        <v>0.04476198744909742</v>
       </c>
     </row>
     <row r="37">
@@ -2106,7 +2109,7 @@
         <v>46431</v>
       </c>
       <c r="I37" s="22" t="n">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>46480</v>
@@ -2117,7 +2120,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>0.01464499022474442</v>
+        <v>0.01424996859778785</v>
       </c>
     </row>
     <row r="38">
@@ -2152,7 +2155,7 @@
         <v>46432</v>
       </c>
       <c r="I38" s="22" t="n">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>46455</v>
@@ -2163,7 +2166,7 @@
         </is>
       </c>
       <c r="L38" s="9" t="n">
-        <v>0.03305581376353177</v>
+        <v>0.0330425677095552</v>
       </c>
     </row>
     <row r="39">
@@ -2198,7 +2201,7 @@
         <v>46433</v>
       </c>
       <c r="I39" s="22" t="n">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>46425</v>
@@ -2209,7 +2212,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.006916520750870562</v>
+        <v>0.007227558827049737</v>
       </c>
     </row>
     <row r="40">
@@ -2244,7 +2247,7 @@
         <v>46433</v>
       </c>
       <c r="I40" s="22" t="n">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="J40" s="10" t="n">
         <v>46383</v>
@@ -2255,7 +2258,7 @@
         </is>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.0222478932745187</v>
+        <v>0.02151071350144007</v>
       </c>
     </row>
     <row r="41">
@@ -2290,7 +2293,7 @@
         <v>46433</v>
       </c>
       <c r="I41" s="22" t="n">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>46368</v>
@@ -2301,7 +2304,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>0.03159713781868049</v>
+        <v>0.02956461610196163</v>
       </c>
     </row>
     <row r="42">
@@ -2321,13 +2324,13 @@
         </is>
       </c>
       <c r="D42" s="7" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="E42" s="7" t="n">
         <v>0.8</v>
       </c>
-      <c r="E42" s="7" t="n">
-        <v>0.79</v>
-      </c>
       <c r="F42" s="8" t="n">
-        <v>0.01265822784810128</v>
+        <v>0.02499999999999988</v>
       </c>
       <c r="G42" s="9" t="n">
         <v>0.04</v>
@@ -2336,7 +2339,7 @@
         <v>46433</v>
       </c>
       <c r="I42" s="22" t="n">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="J42" s="10" t="n">
         <v>46270</v>
@@ -2347,7 +2350,7 @@
         </is>
       </c>
       <c r="L42" s="9" t="n">
-        <v>0.02865842642888866</v>
+        <v>0.0289241618683001</v>
       </c>
     </row>
     <row r="43">
@@ -2382,7 +2385,7 @@
         <v>46433</v>
       </c>
       <c r="I43" s="22" t="n">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>46243</v>
@@ -2393,7 +2396,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>0.03565587212565616</v>
+        <v>0.03523517112712499</v>
       </c>
     </row>
     <row r="44">
@@ -2428,7 +2431,7 @@
         <v>46440</v>
       </c>
       <c r="I44" s="22" t="n">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="J44" s="10" t="n">
         <v>46450</v>
@@ -2439,7 +2442,7 @@
         </is>
       </c>
       <c r="L44" s="9" t="n">
-        <v>0.01012128081164349</v>
+        <v>0.009957936486157157</v>
       </c>
     </row>
     <row r="45">
@@ -2474,7 +2477,7 @@
         <v>46441</v>
       </c>
       <c r="I45" s="22" t="n">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="J45" s="10" t="n">
         <v>46456</v>
@@ -2485,7 +2488,7 @@
         </is>
       </c>
       <c r="L45" s="9" t="n">
-        <v>0.02669798647274613</v>
+        <v>0.02709302325581395</v>
       </c>
     </row>
     <row r="46">
@@ -2520,7 +2523,7 @@
         <v>46452</v>
       </c>
       <c r="I46" s="22" t="n">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="J46" s="10" t="n">
         <v>46487</v>
@@ -2531,7 +2534,7 @@
         </is>
       </c>
       <c r="L46" s="9" t="n">
-        <v>0.01706993074294785</v>
+        <v>0.01690972219968362</v>
       </c>
     </row>
     <row r="47">
@@ -2566,7 +2569,7 @@
         <v>46461</v>
       </c>
       <c r="I47" s="22" t="n">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="J47" s="10" t="n">
         <v>46300</v>
@@ -2577,7 +2580,7 @@
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>0.01781049606101486</v>
+        <v>0.01787310033310249</v>
       </c>
     </row>
     <row r="48">
@@ -2612,7 +2615,7 @@
         <v>46461</v>
       </c>
       <c r="I48" s="22" t="n">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="J48" s="10" t="n">
         <v>46386</v>
@@ -2623,7 +2626,7 @@
         </is>
       </c>
       <c r="L48" s="9" t="n">
-        <v>0.0514516241719684</v>
+        <v>0.05076490983355867</v>
       </c>
     </row>
     <row r="49">
@@ -2658,7 +2661,7 @@
         <v>46488</v>
       </c>
       <c r="I49" s="22" t="n">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>46498</v>
@@ -2669,7 +2672,7 @@
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>0.02947325724122701</v>
+        <v>0.0291079196636194</v>
       </c>
     </row>
     <row r="50">
@@ -2704,7 +2707,7 @@
         <v>46492</v>
       </c>
       <c r="I50" s="22" t="n">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="J50" s="10" t="n">
         <v>46501</v>
@@ -2715,7 +2718,7 @@
         </is>
       </c>
       <c r="L50" s="9" t="n">
-        <v>0.02022325581395349</v>
+        <v>0.02087073374830579</v>
       </c>
     </row>
     <row r="51">
@@ -2750,7 +2753,7 @@
         <v>46492</v>
       </c>
       <c r="I51" s="22" t="n">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="J51" s="10" t="n">
         <v>46376</v>
@@ -2761,7 +2764,7 @@
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>0.05102481603972341</v>
+        <v>0.04866350385719938</v>
       </c>
     </row>
     <row r="52">
@@ -2796,7 +2799,7 @@
         <v>46493</v>
       </c>
       <c r="I52" s="22" t="n">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="J52" s="10" t="n">
         <v>46531</v>
@@ -2807,7 +2810,7 @@
         </is>
       </c>
       <c r="L52" s="9" t="n">
-        <v>0.02086008852056917</v>
+        <v>0.02073100078539538</v>
       </c>
     </row>
     <row r="53">
@@ -2842,7 +2845,7 @@
         <v>46499</v>
       </c>
       <c r="I53" s="22" t="n">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="J53" s="10" t="n">
         <v>46526</v>
@@ -2853,7 +2856,7 @@
         </is>
       </c>
       <c r="L53" s="9" t="n">
-        <v>0.02839337221937417</v>
+        <v>0.02606063813098966</v>
       </c>
     </row>
     <row r="54">
@@ -2888,7 +2891,7 @@
         <v>46504</v>
       </c>
       <c r="I54" s="22" t="n">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="J54" s="10" t="n">
         <v>46562</v>
@@ -2899,7 +2902,7 @@
         </is>
       </c>
       <c r="L54" s="9" t="n">
-        <v>0.04190114189992526</v>
+        <v>0.04122323003291564</v>
       </c>
     </row>
     <row r="55">
@@ -2934,7 +2937,7 @@
         <v>46508</v>
       </c>
       <c r="I55" s="22" t="n">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="J55" s="10" t="n">
         <v>46518</v>
@@ -2945,7 +2948,7 @@
         </is>
       </c>
       <c r="L55" s="9" t="n">
-        <v>0.04495018793044805</v>
+        <v>0.04346634925710766</v>
       </c>
     </row>
     <row r="56">
@@ -2980,7 +2983,7 @@
         <v>46515</v>
       </c>
       <c r="I56" s="22" t="n">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="J56" s="10" t="n">
         <v>46542</v>
@@ -2991,7 +2994,7 @@
         </is>
       </c>
       <c r="L56" s="9" t="n">
-        <v>0.04171070461141636</v>
+        <v>0.04234620794541938</v>
       </c>
     </row>
     <row r="57">
@@ -3026,7 +3029,7 @@
         <v>46532</v>
       </c>
       <c r="I57" s="22" t="n">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="J57" s="10" t="n">
         <v>46563</v>
@@ -3037,7 +3040,7 @@
         </is>
       </c>
       <c r="L57" s="9" t="n">
-        <v>0.03518201781732959</v>
+        <v>0.03406872745296734</v>
       </c>
     </row>
   </sheetData>
@@ -3072,44 +3075,44 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Expected Increase Announcements by Month - 07/06/2026</t>
+          <t>Expected Increase Announcements by Month - 07/13/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>January 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D5" s="24" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E5" s="24" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F5" s="24" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3140,39 +3143,39 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>July 2026</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D9" s="25" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E9" s="24" t="inlineStr">
+      <c r="E9" s="25" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F9" s="24" t="inlineStr">
+      <c r="F9" s="25" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3323,39 +3326,39 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>August 2026</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B18" s="24" t="inlineStr">
+      <c r="B18" s="25" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C18" s="24" t="inlineStr">
+      <c r="C18" s="25" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D18" s="24" t="inlineStr">
+      <c r="D18" s="25" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E18" s="24" t="inlineStr">
+      <c r="E18" s="25" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F18" s="24" t="inlineStr">
+      <c r="F18" s="25" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3386,39 +3389,39 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="inlineStr">
+      <c r="A21" s="24" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B22" s="24" t="inlineStr">
+      <c r="B22" s="25" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C22" s="24" t="inlineStr">
+      <c r="C22" s="25" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D22" s="24" t="inlineStr">
+      <c r="D22" s="25" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E22" s="24" t="inlineStr">
+      <c r="E22" s="25" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F22" s="24" t="inlineStr">
+      <c r="F22" s="25" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3497,39 +3500,39 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="inlineStr">
+      <c r="A27" s="24" t="inlineStr">
         <is>
           <t>October 2026</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="24" t="inlineStr">
+      <c r="A28" s="25" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B28" s="24" t="inlineStr">
+      <c r="B28" s="25" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C28" s="24" t="inlineStr">
+      <c r="C28" s="25" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D28" s="24" t="inlineStr">
+      <c r="D28" s="25" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E28" s="24" t="inlineStr">
+      <c r="E28" s="25" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F28" s="24" t="inlineStr">
+      <c r="F28" s="25" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3632,39 +3635,39 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="23" t="inlineStr">
+      <c r="A34" s="24" t="inlineStr">
         <is>
           <t>November 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="24" t="inlineStr">
+      <c r="A35" s="25" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B35" s="24" t="inlineStr">
+      <c r="B35" s="25" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C35" s="24" t="inlineStr">
+      <c r="C35" s="25" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D35" s="24" t="inlineStr">
+      <c r="D35" s="25" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E35" s="24" t="inlineStr">
+      <c r="E35" s="25" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F35" s="24" t="inlineStr">
+      <c r="F35" s="25" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3815,39 +3818,39 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="23" t="inlineStr">
+      <c r="A43" s="24" t="inlineStr">
         <is>
           <t>December 2026</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="24" t="inlineStr">
+      <c r="A44" s="25" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B44" s="24" t="inlineStr">
+      <c r="B44" s="25" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C44" s="24" t="inlineStr">
+      <c r="C44" s="25" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D44" s="24" t="inlineStr">
+      <c r="D44" s="25" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E44" s="24" t="inlineStr">
+      <c r="E44" s="25" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F44" s="24" t="inlineStr">
+      <c r="F44" s="25" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3950,39 +3953,39 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="23" t="inlineStr">
+      <c r="A50" s="24" t="inlineStr">
         <is>
           <t>January 2027</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="24" t="inlineStr">
+      <c r="A51" s="25" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B51" s="24" t="inlineStr">
+      <c r="B51" s="25" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C51" s="24" t="inlineStr">
+      <c r="C51" s="25" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D51" s="24" t="inlineStr">
+      <c r="D51" s="25" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E51" s="24" t="inlineStr">
+      <c r="E51" s="25" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F51" s="24" t="inlineStr">
+      <c r="F51" s="25" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -4061,39 +4064,39 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="23" t="inlineStr">
+      <c r="A56" s="24" t="inlineStr">
         <is>
           <t>February 2027</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="24" t="inlineStr">
+      <c r="A57" s="25" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B57" s="24" t="inlineStr">
+      <c r="B57" s="25" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C57" s="24" t="inlineStr">
+      <c r="C57" s="25" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D57" s="24" t="inlineStr">
+      <c r="D57" s="25" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E57" s="24" t="inlineStr">
+      <c r="E57" s="25" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F57" s="24" t="inlineStr">
+      <c r="F57" s="25" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -4304,10 +4307,10 @@
         <v>46270</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="E66" s="8" t="n">
-        <v>0.01265822784810128</v>
+        <v>0.02499999999999988</v>
       </c>
       <c r="F66" s="12" t="inlineStr">
         <is>
@@ -4388,39 +4391,39 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="23" t="inlineStr">
+      <c r="A71" s="24" t="inlineStr">
         <is>
           <t>March 2027</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="24" t="inlineStr">
+      <c r="A72" s="25" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B72" s="24" t="inlineStr">
+      <c r="B72" s="25" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C72" s="24" t="inlineStr">
+      <c r="C72" s="25" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D72" s="24" t="inlineStr">
+      <c r="D72" s="25" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E72" s="24" t="inlineStr">
+      <c r="E72" s="25" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F72" s="24" t="inlineStr">
+      <c r="F72" s="25" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -4499,39 +4502,39 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="23" t="inlineStr">
+      <c r="A77" s="24" t="inlineStr">
         <is>
           <t>April 2027</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="24" t="inlineStr">
+      <c r="A78" s="25" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B78" s="24" t="inlineStr">
+      <c r="B78" s="25" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C78" s="24" t="inlineStr">
+      <c r="C78" s="25" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D78" s="24" t="inlineStr">
+      <c r="D78" s="25" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E78" s="24" t="inlineStr">
+      <c r="E78" s="25" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F78" s="24" t="inlineStr">
+      <c r="F78" s="25" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -4682,39 +4685,39 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="23" t="inlineStr">
+      <c r="A86" s="24" t="inlineStr">
         <is>
           <t>May 2027</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="24" t="inlineStr">
+      <c r="A87" s="25" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B87" s="24" t="inlineStr">
+      <c r="B87" s="25" t="inlineStr">
         <is>
           <t>Est. Announce</t>
         </is>
       </c>
-      <c r="C87" s="24" t="inlineStr">
+      <c r="C87" s="25" t="inlineStr">
         <is>
           <t>Est. Ex-Date</t>
         </is>
       </c>
-      <c r="D87" s="24" t="inlineStr">
+      <c r="D87" s="25" t="inlineStr">
         <is>
           <t>Last Amount</t>
         </is>
       </c>
-      <c r="E87" s="24" t="inlineStr">
+      <c r="E87" s="25" t="inlineStr">
         <is>
           <t>Last Change</t>
         </is>
       </c>
-      <c r="F87" s="24" t="inlineStr">
+      <c r="F87" s="25" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -4831,7 +4834,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete Holdings Dividend Summary - 07/06/2026</t>
+          <t>Complete Holdings Dividend Summary - 07/13/2026</t>
         </is>
       </c>
     </row>
@@ -4931,11 +4934,11 @@
       <c r="F5" s="7" t="n">
         <v>0.29</v>
       </c>
-      <c r="G5" s="25" t="n">
+      <c r="G5" s="26" t="n">
         <v>1.16</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.01012128081164349</v>
+        <v>0.009957936486157157</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>46160</v>
@@ -4984,11 +4987,11 @@
       <c r="F6" s="7" t="n">
         <v>2.52</v>
       </c>
-      <c r="G6" s="25" t="n">
+      <c r="G6" s="26" t="n">
         <v>10.08</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.02790465823278872</v>
+        <v>0.02787263837801698</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>46157</v>
@@ -5037,11 +5040,11 @@
       <c r="F7" s="7" t="n">
         <v>3.177</v>
       </c>
-      <c r="G7" s="25" t="n">
+      <c r="G7" s="26" t="n">
         <v>12.708</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.006916520750870562</v>
+        <v>0.007227558827049737</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>46139</v>
@@ -5090,11 +5093,11 @@
       <c r="F8" s="16" t="n">
         <v>0.504</v>
       </c>
-      <c r="G8" s="26" t="n">
+      <c r="G8" s="27" t="n">
         <v>2.016</v>
       </c>
       <c r="H8" s="18" t="n">
-        <v>0.02398429590958984</v>
+        <v>0.02358722325034518</v>
       </c>
       <c r="I8" s="19" t="n">
         <v>46160</v>
@@ -5143,11 +5146,11 @@
       <c r="F9" s="7" t="n">
         <v>0.703</v>
       </c>
-      <c r="G9" s="25" t="n">
+      <c r="G9" s="26" t="n">
         <v>2.812</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.03827152172028183</v>
+        <v>0.03690046496205276</v>
       </c>
       <c r="I9" s="10" t="n">
         <v>46157</v>
@@ -5196,11 +5199,11 @@
       <c r="F10" s="7" t="n">
         <v>1.03</v>
       </c>
-      <c r="G10" s="25" t="n">
+      <c r="G10" s="26" t="n">
         <v>4.12</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.02647389558232932</v>
+        <v>0.02615374869501659</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>46171</v>
@@ -5249,11 +5252,11 @@
       <c r="F11" s="7" t="n">
         <v>1.24</v>
       </c>
-      <c r="G11" s="25" t="n">
+      <c r="G11" s="26" t="n">
         <v>4.96</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.05178804407181118</v>
+        <v>0.05128205063482052</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>46134</v>
@@ -5302,11 +5305,11 @@
       <c r="F12" s="7" t="n">
         <v>1.3</v>
       </c>
-      <c r="G12" s="25" t="n">
+      <c r="G12" s="26" t="n">
         <v>5.2</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.0222478932745187</v>
+        <v>0.02151071350144007</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>46182</v>
@@ -5355,11 +5358,11 @@
       <c r="F13" s="7" t="n">
         <v>0.23</v>
       </c>
-      <c r="G13" s="25" t="n">
+      <c r="G13" s="26" t="n">
         <v>0.92</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0.02077922006309264</v>
+        <v>0.02089959087762214</v>
       </c>
       <c r="I13" s="10" t="n">
         <v>46163</v>
@@ -5408,11 +5411,11 @@
       <c r="F14" s="7" t="n">
         <v>0.6</v>
       </c>
-      <c r="G14" s="25" t="n">
+      <c r="G14" s="26" t="n">
         <v>2.4</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0.008169517657604557</v>
+        <v>0.007805259164950651</v>
       </c>
       <c r="I14" s="10" t="n">
         <v>46157</v>
@@ -5461,14 +5464,14 @@
       <c r="F15" s="7" t="n">
         <v>0.42</v>
       </c>
-      <c r="G15" s="25" t="n">
+      <c r="G15" s="26" t="n">
         <v>1.68</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.01464499022474442</v>
+        <v>0.01424996859778785</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>46114</v>
+        <v>46209</v>
       </c>
       <c r="J15" s="8" t="n">
         <v>0.02439024390243905</v>
@@ -5514,11 +5517,11 @@
       <c r="F16" s="7" t="n">
         <v>1.78</v>
       </c>
-      <c r="G16" s="25" t="n">
+      <c r="G16" s="26" t="n">
         <v>7.12</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.04217010278625639</v>
+        <v>0.03954566954044979</v>
       </c>
       <c r="I16" s="10" t="n">
         <v>46161</v>
@@ -5567,14 +5570,14 @@
       <c r="F17" s="7" t="n">
         <v>0.86</v>
       </c>
-      <c r="G17" s="25" t="n">
+      <c r="G17" s="26" t="n">
         <v>3.44</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.01611920688332178</v>
+        <v>0.01638173203491813</v>
       </c>
       <c r="I17" s="10" t="n">
-        <v>46118</v>
+        <v>46211</v>
       </c>
       <c r="J17" s="8" t="n">
         <v>0.07499999999999993</v>
@@ -5620,11 +5623,11 @@
       <c r="F18" s="7" t="n">
         <v>0.32</v>
       </c>
-      <c r="G18" s="25" t="n">
+      <c r="G18" s="26" t="n">
         <v>1.28</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.03159713781868049</v>
+        <v>0.02956461610196163</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>46188</v>
@@ -5673,11 +5676,11 @@
       <c r="F19" s="7" t="n">
         <v>0.84</v>
       </c>
-      <c r="G19" s="25" t="n">
+      <c r="G19" s="26" t="n">
         <v>3.36</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.0491947269380616</v>
+        <v>0.04913358039101189</v>
       </c>
       <c r="I19" s="10" t="n">
         <v>46188</v>
@@ -5726,11 +5729,11 @@
       <c r="F20" s="7" t="n">
         <v>0.64</v>
       </c>
-      <c r="G20" s="25" t="n">
+      <c r="G20" s="26" t="n">
         <v>2.56</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.0223122847115672</v>
+        <v>0.02204615862425437</v>
       </c>
       <c r="I20" s="10" t="n">
         <v>46143</v>
@@ -5779,11 +5782,11 @@
       <c r="F21" s="7" t="n">
         <v>1.59</v>
       </c>
-      <c r="G21" s="25" t="n">
+      <c r="G21" s="26" t="n">
         <v>6.36</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.01706993074294785</v>
+        <v>0.01690972219968362</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>46205</v>
@@ -5832,11 +5835,11 @@
       <c r="F22" s="16" t="n">
         <v>0.295</v>
       </c>
-      <c r="G22" s="26" t="n">
+      <c r="G22" s="27" t="n">
         <v>1.18</v>
       </c>
       <c r="H22" s="18" t="n">
-        <v>0.01574908177427583</v>
+        <v>0.01576907618770492</v>
       </c>
       <c r="I22" s="19" t="n">
         <v>46125</v>
@@ -5885,11 +5888,11 @@
       <c r="F23" s="7" t="n">
         <v>2.33</v>
       </c>
-      <c r="G23" s="25" t="n">
+      <c r="G23" s="26" t="n">
         <v>9.32</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.02669798647274613</v>
+        <v>0.02709302325581395</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>46177</v>
@@ -5938,11 +5941,11 @@
       <c r="F24" s="7" t="n">
         <v>1.38</v>
       </c>
-      <c r="G24" s="25" t="n">
+      <c r="G24" s="26" t="n">
         <v>5.52</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>0.01891447392155589</v>
+        <v>0.01918932048156368</v>
       </c>
       <c r="I24" s="10" t="n">
         <v>46171</v>
@@ -5991,11 +5994,11 @@
       <c r="F25" s="7" t="n">
         <v>0.293</v>
       </c>
-      <c r="G25" s="25" t="n">
+      <c r="G25" s="26" t="n">
         <v>1.172</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.04816108666911</v>
+        <v>0.0475552841643708</v>
       </c>
       <c r="I25" s="10" t="n">
         <v>46125</v>
@@ -6044,11 +6047,11 @@
       <c r="F26" s="7" t="n">
         <v>0.82</v>
       </c>
-      <c r="G26" s="25" t="n">
+      <c r="G26" s="26" t="n">
         <v>3.28</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>0.03396144718830089</v>
+        <v>0.03269048716727996</v>
       </c>
       <c r="I26" s="10" t="n">
         <v>46204</v>
@@ -6097,14 +6100,14 @@
       <c r="F27" s="7" t="n">
         <v>0.61</v>
       </c>
-      <c r="G27" s="25" t="n">
+      <c r="G27" s="26" t="n">
         <v>2.44</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.01677321770485241</v>
+        <v>0.01603364514018875</v>
       </c>
       <c r="I27" s="10" t="n">
-        <v>46086</v>
+        <v>46174</v>
       </c>
       <c r="J27" s="8" t="n">
         <v>0.05172413793103453</v>
@@ -6150,11 +6153,11 @@
       <c r="F28" s="7" t="n">
         <v>1.34</v>
       </c>
-      <c r="G28" s="25" t="n">
+      <c r="G28" s="26" t="n">
         <v>5.36</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0.02086008852056917</v>
+        <v>0.02073100078539538</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>46168</v>
@@ -6203,14 +6206,14 @@
       <c r="F29" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="G29" s="25" t="n">
+      <c r="G29" s="26" t="n">
         <v>6</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.01781049606101486</v>
+        <v>0.01787310033310249</v>
       </c>
       <c r="I29" s="10" t="n">
-        <v>46118</v>
+        <v>46209</v>
       </c>
       <c r="J29" s="8" t="n">
         <v>0.07142857142857149</v>
@@ -6256,11 +6259,11 @@
       <c r="F30" s="7" t="n">
         <v>1.087</v>
       </c>
-      <c r="G30" s="25" t="n">
+      <c r="G30" s="26" t="n">
         <v>2.174</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.02022325581395349</v>
+        <v>0.02087073374830579</v>
       </c>
       <c r="I30" s="10" t="n">
         <v>46132</v>
@@ -6309,11 +6312,11 @@
       <c r="F31" s="7" t="n">
         <v>0.79</v>
       </c>
-      <c r="G31" s="25" t="n">
+      <c r="G31" s="26" t="n">
         <v>3.16</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0.01222579016936565</v>
+        <v>0.01243017852579043</v>
       </c>
       <c r="I31" s="10" t="n">
         <v>46203</v>
@@ -6362,11 +6365,11 @@
       <c r="F32" s="7" t="n">
         <v>0.72</v>
       </c>
-      <c r="G32" s="25" t="n">
+      <c r="G32" s="26" t="n">
         <v>2.88</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.03518201781732959</v>
+        <v>0.03406872745296734</v>
       </c>
       <c r="I32" s="10" t="n">
         <v>46199</v>
@@ -6415,14 +6418,14 @@
       <c r="F33" s="7" t="n">
         <v>0.48</v>
       </c>
-      <c r="G33" s="25" t="n">
+      <c r="G33" s="26" t="n">
         <v>1.92</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0.03727793340807439</v>
+        <v>0.03590798496665439</v>
       </c>
       <c r="I33" s="10" t="n">
-        <v>46132</v>
+        <v>46209</v>
       </c>
       <c r="J33" s="8" t="n">
         <v>0.0666666666666666</v>
@@ -6468,11 +6471,11 @@
       <c r="F34" s="7" t="n">
         <v>0.91</v>
       </c>
-      <c r="G34" s="25" t="n">
+      <c r="G34" s="26" t="n">
         <v>3.64</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0.009451599621287882</v>
+        <v>0.009398884557615285</v>
       </c>
       <c r="I34" s="10" t="n">
         <v>46163</v>
@@ -6521,14 +6524,14 @@
       <c r="F35" s="7" t="n">
         <v>0.87</v>
       </c>
-      <c r="G35" s="25" t="n">
+      <c r="G35" s="26" t="n">
         <v>3.48</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0.02871523995292049</v>
+        <v>0.02772466613344378</v>
       </c>
       <c r="I35" s="10" t="n">
-        <v>46120</v>
+        <v>46211</v>
       </c>
       <c r="J35" s="8" t="n">
         <v>0.0235294117647059</v>
@@ -6574,14 +6577,14 @@
       <c r="F36" s="7" t="n">
         <v>0.41</v>
       </c>
-      <c r="G36" s="25" t="n">
+      <c r="G36" s="26" t="n">
         <v>1.64</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0.03838502185069386</v>
+        <v>0.03671778722453514</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>46083</v>
+        <v>46174</v>
       </c>
       <c r="J36" s="8" t="n">
         <v>0.02499999999999988</v>
@@ -6627,11 +6630,11 @@
       <c r="F37" s="7" t="n">
         <v>1.275</v>
       </c>
-      <c r="G37" s="25" t="n">
+      <c r="G37" s="26" t="n">
         <v>2.55</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.05230232682053303</v>
+        <v>0.05161421036343746</v>
       </c>
       <c r="I37" s="10" t="n">
         <v>46111</v>
@@ -6680,11 +6683,11 @@
       <c r="F38" s="7" t="n">
         <v>0.271</v>
       </c>
-      <c r="G38" s="25" t="n">
+      <c r="G38" s="26" t="n">
         <v>3.252</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0.0514516241719684</v>
+        <v>0.05076490983355867</v>
       </c>
       <c r="I38" s="10" t="n">
         <v>46203</v>
@@ -6733,11 +6736,11 @@
       <c r="F39" s="7" t="n">
         <v>1.19</v>
       </c>
-      <c r="G39" s="25" t="n">
+      <c r="G39" s="26" t="n">
         <v>4.76</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.04495018793044805</v>
+        <v>0.04346634925710766</v>
       </c>
       <c r="I39" s="10" t="n">
         <v>46155</v>
@@ -6786,11 +6789,11 @@
       <c r="F40" s="7" t="n">
         <v>0.67</v>
       </c>
-      <c r="G40" s="25" t="n">
+      <c r="G40" s="26" t="n">
         <v>2.68</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.03305581376353177</v>
+        <v>0.0330425677095552</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>46182</v>
@@ -6839,11 +6842,11 @@
       <c r="F41" s="7" t="n">
         <v>1.48</v>
       </c>
-      <c r="G41" s="25" t="n">
+      <c r="G41" s="26" t="n">
         <v>5.92</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0.04171070461141636</v>
+        <v>0.04234620794541938</v>
       </c>
       <c r="I41" s="10" t="n">
         <v>46178</v>
@@ -6892,11 +6895,11 @@
       <c r="F42" s="7" t="n">
         <v>0.43</v>
       </c>
-      <c r="G42" s="25" t="n">
+      <c r="G42" s="26" t="n">
         <v>1.72</v>
       </c>
       <c r="H42" s="9" t="n">
-        <v>0.07243629981928987</v>
+        <v>0.06981936204666597</v>
       </c>
       <c r="I42" s="10" t="n">
         <v>46150</v>
@@ -6943,19 +6946,19 @@
         </is>
       </c>
       <c r="F43" s="7" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G43" s="25" t="n">
-        <v>3.2</v>
+        <v>0.82</v>
+      </c>
+      <c r="G43" s="26" t="n">
+        <v>3.28</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0.02865842642888866</v>
+        <v>0.0289241618683001</v>
       </c>
       <c r="I43" s="10" t="n">
-        <v>46092</v>
+        <v>46174</v>
       </c>
       <c r="J43" s="8" t="n">
-        <v>0.01265822784810128</v>
+        <v>0.02499999999999988</v>
       </c>
       <c r="K43" s="10" t="n">
         <v>46433</v>
@@ -6998,11 +7001,11 @@
       <c r="F44" s="7" t="n">
         <v>1.089</v>
       </c>
-      <c r="G44" s="25" t="n">
+      <c r="G44" s="26" t="n">
         <v>4.356</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.02947325724122701</v>
+        <v>0.0291079196636194</v>
       </c>
       <c r="I44" s="10" t="n">
         <v>46136</v>
@@ -7051,11 +7054,11 @@
       <c r="F45" s="7" t="n">
         <v>0.551</v>
       </c>
-      <c r="G45" s="25" t="n">
+      <c r="G45" s="26" t="n">
         <v>2.204</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>0.04190114189992526</v>
+        <v>0.04122323003291564</v>
       </c>
       <c r="I45" s="10" t="n">
         <v>46198</v>
@@ -7104,11 +7107,11 @@
       <c r="F46" s="7" t="n">
         <v>1.27</v>
       </c>
-      <c r="G46" s="25" t="n">
+      <c r="G46" s="26" t="n">
         <v>5.08</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.02839337221937417</v>
+        <v>0.02606063813098966</v>
       </c>
       <c r="I46" s="10" t="n">
         <v>46160</v>
@@ -7157,11 +7160,11 @@
       <c r="F47" s="7" t="n">
         <v>0.93</v>
       </c>
-      <c r="G47" s="25" t="n">
+      <c r="G47" s="26" t="n">
         <v>3.72</v>
       </c>
       <c r="H47" s="9" t="n">
-        <v>0.01674921160635266</v>
+        <v>0.01586015754252245</v>
       </c>
       <c r="I47" s="10" t="n">
         <v>46161</v>
@@ -7210,11 +7213,11 @@
       <c r="F48" s="7" t="n">
         <v>2.44</v>
       </c>
-      <c r="G48" s="25" t="n">
+      <c r="G48" s="26" t="n">
         <v>9.76</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>0.02366835262725075</v>
+        <v>0.02413332593824269</v>
       </c>
       <c r="I48" s="10" t="n">
         <v>46162</v>
@@ -7263,11 +7266,11 @@
       <c r="F49" s="7" t="n">
         <v>0.83</v>
       </c>
-      <c r="G49" s="25" t="n">
+      <c r="G49" s="26" t="n">
         <v>3.32</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.03601062976288923</v>
+        <v>0.03744008892858095</v>
       </c>
       <c r="I49" s="10" t="n">
         <v>46181</v>
@@ -7316,11 +7319,11 @@
       <c r="F50" s="7" t="n">
         <v>1.3</v>
       </c>
-      <c r="G50" s="25" t="n">
+      <c r="G50" s="26" t="n">
         <v>5.2</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.04387260015233685</v>
+        <v>0.04476198744909742</v>
       </c>
       <c r="I50" s="10" t="n">
         <v>46188</v>
@@ -7369,11 +7372,11 @@
       <c r="F51" s="7" t="n">
         <v>0.974</v>
       </c>
-      <c r="G51" s="25" t="n">
+      <c r="G51" s="26" t="n">
         <v>3.896</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.05102481603972341</v>
+        <v>0.04866350385719938</v>
       </c>
       <c r="I51" s="10" t="n">
         <v>46112</v>
@@ -7422,11 +7425,11 @@
       <c r="F52" s="7" t="n">
         <v>1.42</v>
       </c>
-      <c r="G52" s="25" t="n">
+      <c r="G52" s="26" t="n">
         <v>5.68</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.01867254003883344</v>
+        <v>0.01881667089258208</v>
       </c>
       <c r="I52" s="10" t="n">
         <v>46147</v>
@@ -7475,11 +7478,11 @@
       <c r="F53" s="7" t="n">
         <v>0.545</v>
       </c>
-      <c r="G53" s="25" t="n">
+      <c r="G53" s="26" t="n">
         <v>2.18</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>0.03565587212565616</v>
+        <v>0.03523517112712499</v>
       </c>
       <c r="I53" s="10" t="n">
         <v>46157</v>
@@ -7528,11 +7531,11 @@
       <c r="F54" s="7" t="n">
         <v>1.38</v>
       </c>
-      <c r="G54" s="25" t="n">
+      <c r="G54" s="26" t="n">
         <v>5.52</v>
       </c>
       <c r="H54" s="9" t="n">
-        <v>0.01950736818810225</v>
+        <v>0.0191056338898471</v>
       </c>
       <c r="I54" s="10" t="n">
         <v>46171</v>
@@ -7581,14 +7584,14 @@
       <c r="F55" s="7" t="n">
         <v>0.708</v>
       </c>
-      <c r="G55" s="25" t="n">
+      <c r="G55" s="26" t="n">
         <v>2.832</v>
       </c>
       <c r="H55" s="9" t="n">
-        <v>0.06707721265084407</v>
+        <v>0.06631898910307311</v>
       </c>
       <c r="I55" s="10" t="n">
-        <v>46122</v>
+        <v>46213</v>
       </c>
       <c r="J55" s="8" t="n">
         <v>0.02608695652173916</v>
@@ -7634,11 +7637,11 @@
       <c r="F56" s="7" t="n">
         <v>1.03</v>
       </c>
-      <c r="G56" s="25" t="n">
+      <c r="G56" s="26" t="n">
         <v>4.12</v>
       </c>
       <c r="H56" s="9" t="n">
-        <v>0.03013899116296197</v>
+        <v>0.02883740561914779</v>
       </c>
       <c r="I56" s="10" t="n">
         <v>46157</v>

</xml_diff>

<commit_message>
Update dividend calendar 2026-08-10
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -561,7 +561,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estimated Dividend Calendar: Anticipated Announcements - 08/03/2026</t>
+          <t>Estimated Dividend Calendar: Anticipated Announcements - 08/10/2026</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         <v>46048</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-189</v>
+        <v>-196</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>46413</v>
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="L6" s="9" t="n">
-        <v>0.06860789872107974</v>
+        <v>0.06394052135283915</v>
       </c>
     </row>
     <row r="7">
@@ -712,7 +712,7 @@
         <v>46236</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-1</v>
+        <v>-8</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>46613</v>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.01558898681591544</v>
+        <v>0.0151124292354321</v>
       </c>
     </row>
     <row r="8">
@@ -758,7 +758,7 @@
         <v>46263</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>46297</v>
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.03246881913478192</v>
+        <v>0.03144171788339006</v>
       </c>
     </row>
     <row r="9">
@@ -804,7 +804,7 @@
         <v>46278</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>46344</v>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>0.007421150426047773</v>
+        <v>0.007172413793103448</v>
       </c>
     </row>
     <row r="10">
@@ -850,7 +850,7 @@
         <v>46280</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>46303</v>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.05979729652666019</v>
+        <v>0.06105422232354177</v>
       </c>
     </row>
     <row r="11">
@@ -896,7 +896,7 @@
         <v>46285</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46325</v>
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.0213317318299373</v>
+        <v>0.02001550505473602</v>
       </c>
     </row>
     <row r="12">
@@ -942,7 +942,7 @@
         <v>46305</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>46339</v>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0.02787791355406566</v>
+        <v>0.02837226394875147</v>
       </c>
     </row>
     <row r="13">
@@ -988,7 +988,7 @@
         <v>46311</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>46386</v>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>0.01183786607889024</v>
+        <v>0.01124795320189071</v>
       </c>
     </row>
     <row r="14">
@@ -1034,7 +1034,7 @@
         <v>46317</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>46351</v>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.01652496664709451</v>
+        <v>0.01697208266431864</v>
       </c>
     </row>
     <row r="15">
@@ -1080,7 +1080,7 @@
         <v>46322</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>46338</v>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>0.02364677581271972</v>
+        <v>0.02411681547998738</v>
       </c>
     </row>
     <row r="16">
@@ -1126,7 +1126,7 @@
         <v>46329</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>46338</v>
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="L16" s="9" t="n">
-        <v>0.007708366638676293</v>
+        <v>0.007434598707771089</v>
       </c>
     </row>
     <row r="17">
@@ -1172,7 +1172,7 @@
         <v>46332</v>
       </c>
       <c r="I17" s="13" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>46346</v>
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.02348807553888279</v>
+        <v>0.02341566388645527</v>
       </c>
     </row>
     <row r="18">
@@ -1218,7 +1218,7 @@
         <v>46341</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>46339</v>
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.02665286551427834</v>
+        <v>0.02609824759533807</v>
       </c>
     </row>
     <row r="19">
@@ -1264,7 +1264,7 @@
         <v>46344</v>
       </c>
       <c r="I19" s="13" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>46385</v>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0.03667621883406817</v>
+        <v>0.03608344358269835</v>
       </c>
     </row>
     <row r="20">
@@ -1310,7 +1310,7 @@
         <v>46347</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>46358</v>
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0.03870206489675516</v>
+        <v>0.03984935120019991</v>
       </c>
     </row>
     <row r="21">
@@ -1356,7 +1356,7 @@
         <v>46352</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46400</v>
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.04628752030512757</v>
+        <v>0.04698336397427078</v>
       </c>
     </row>
     <row r="22">
@@ -1402,7 +1402,7 @@
         <v>46360</v>
       </c>
       <c r="I22" s="13" t="n">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J22" s="10" t="n">
         <v>46371</v>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="L22" s="9" t="n">
-        <v>0.0469044447518852</v>
+        <v>0.04619826543263427</v>
       </c>
     </row>
     <row r="23">
@@ -1448,7 +1448,7 @@
         <v>46366</v>
       </c>
       <c r="I23" s="13" t="n">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>46432</v>
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0.02628216836253416</v>
+        <v>0.02469498794862927</v>
       </c>
     </row>
     <row r="24">
@@ -1494,7 +1494,7 @@
         <v>46371</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="J24" s="10" t="n">
         <v>46344</v>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="L24" s="9" t="n">
-        <v>0.0217365619235988</v>
+        <v>0.02281746049016211</v>
       </c>
     </row>
     <row r="25">
@@ -1540,7 +1540,7 @@
         <v>46383</v>
       </c>
       <c r="I25" s="20" t="n">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="J25" s="19" t="n">
         <v>46404</v>
@@ -1551,7 +1551,7 @@
         </is>
       </c>
       <c r="L25" s="18" t="n">
-        <v>0.01460124932688757</v>
+        <v>0.01421429872523905</v>
       </c>
     </row>
     <row r="26">
@@ -1586,7 +1586,7 @@
         <v>46402</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>46483</v>
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0.01483525930464986</v>
+        <v>0.01441199867951928</v>
       </c>
     </row>
     <row r="27">
@@ -1632,7 +1632,7 @@
         <v>46411</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>46435</v>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="L27" s="9" t="n">
-        <v>0.03922443721909909</v>
+        <v>0.03816244952391996</v>
       </c>
     </row>
     <row r="28">
@@ -1678,7 +1678,7 @@
         <v>46417</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>46433</v>
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="L28" s="9" t="n">
-        <v>0.03662834169923343</v>
+        <v>0.0370929935566493</v>
       </c>
     </row>
     <row r="29">
@@ -1724,7 +1724,7 @@
         <v>46422</v>
       </c>
       <c r="I29" s="13" t="n">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>46472</v>
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>0.05467410020090957</v>
+        <v>0.05449882346879326</v>
       </c>
     </row>
     <row r="30">
@@ -1770,7 +1770,7 @@
         <v>46428</v>
       </c>
       <c r="I30" s="13" t="n">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="J30" s="10" t="n">
         <v>46452</v>
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="L30" s="9" t="n">
-        <v>0.01546359150656252</v>
+        <v>0.01567518914683119</v>
       </c>
     </row>
     <row r="31">
@@ -1810,13 +1810,13 @@
         <v>0.02362204724409451</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="H31" s="10" t="n">
         <v>46428</v>
       </c>
       <c r="I31" s="13" t="n">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>46460</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="n">
-        <v>0.04623660844994903</v>
+        <v>0.04571428571428571</v>
       </c>
     </row>
     <row r="32">
@@ -1862,7 +1862,7 @@
         <v>46431</v>
       </c>
       <c r="I32" s="13" t="n">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>46480</v>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="L32" s="9" t="n">
-        <v>0.01464562822254793</v>
+        <v>0.01348531044555835</v>
       </c>
     </row>
     <row r="33">
@@ -1908,7 +1908,7 @@
         <v>46432</v>
       </c>
       <c r="I33" s="13" t="n">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>46455</v>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>0.03485498792136554</v>
+        <v>0.03592493371068497</v>
       </c>
     </row>
     <row r="34">
@@ -1954,7 +1954,7 @@
         <v>46433</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>46425</v>
@@ -1965,7 +1965,7 @@
         </is>
       </c>
       <c r="L34" s="9" t="n">
-        <v>0.005269790339653252</v>
+        <v>0.004852845587305765</v>
       </c>
     </row>
     <row r="35">
@@ -2000,7 +2000,7 @@
         <v>46433</v>
       </c>
       <c r="I35" s="13" t="n">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>46383</v>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0.01936685288640596</v>
+        <v>0.01958863922015894</v>
       </c>
     </row>
     <row r="36">
@@ -2046,7 +2046,7 @@
         <v>46433</v>
       </c>
       <c r="I36" s="13" t="n">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>46368</v>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="L36" s="9" t="n">
-        <v>0.02897238549475621</v>
+        <v>0.02870598779142888</v>
       </c>
     </row>
     <row r="37">
@@ -2092,7 +2092,7 @@
         <v>46433</v>
       </c>
       <c r="I37" s="13" t="n">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>46635</v>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>0.028464808682162</v>
+        <v>0.02885165211275545</v>
       </c>
     </row>
     <row r="38">
@@ -2123,7 +2123,7 @@
         </is>
       </c>
       <c r="D38" s="7" t="n">
-        <v>0.545</v>
+        <v>0.531</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>0.588964</v>
@@ -2132,13 +2132,13 @@
         <v>0.005735494868956323</v>
       </c>
       <c r="G38" s="9" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="H38" s="10" t="n">
         <v>46433</v>
       </c>
       <c r="I38" s="13" t="n">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>46608</v>
@@ -2149,7 +2149,7 @@
         </is>
       </c>
       <c r="L38" s="9" t="n">
-        <v>0.03400405520582705</v>
+        <v>0.03411226243990159</v>
       </c>
     </row>
     <row r="39">
@@ -2184,7 +2184,7 @@
         <v>46440</v>
       </c>
       <c r="I39" s="13" t="n">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>46450</v>
@@ -2195,7 +2195,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.009990526172614474</v>
+        <v>0.009624239863116651</v>
       </c>
     </row>
     <row r="40">
@@ -2230,7 +2230,7 @@
         <v>46441</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="J40" s="10" t="n">
         <v>46456</v>
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.02755765719575049</v>
+        <v>0.02673512917565468</v>
       </c>
     </row>
     <row r="41">
@@ -2276,7 +2276,7 @@
         <v>46452</v>
       </c>
       <c r="I41" s="13" t="n">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>46487</v>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>0.01652141216985137</v>
+        <v>0.01607603275490687</v>
       </c>
     </row>
     <row r="42">
@@ -2322,7 +2322,7 @@
         <v>46461</v>
       </c>
       <c r="I42" s="13" t="n">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="J42" s="10" t="n">
         <v>46300</v>
@@ -2333,7 +2333,7 @@
         </is>
       </c>
       <c r="L42" s="9" t="n">
-        <v>0.01696496669833159</v>
+        <v>0.0167126259346279</v>
       </c>
     </row>
     <row r="43">
@@ -2368,7 +2368,7 @@
         <v>46461</v>
       </c>
       <c r="I43" s="13" t="n">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>46386</v>
@@ -2379,7 +2379,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>0.05085222769668224</v>
+        <v>0.05274083697774267</v>
       </c>
     </row>
     <row r="44">
@@ -2414,7 +2414,7 @@
         <v>46488</v>
       </c>
       <c r="I44" s="13" t="n">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="J44" s="10" t="n">
         <v>46498</v>
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="L44" s="9" t="n">
-        <v>0.02980703447511133</v>
+        <v>0.03004552440590653</v>
       </c>
     </row>
     <row r="45">
@@ -2460,7 +2460,7 @@
         <v>46492</v>
       </c>
       <c r="I45" s="13" t="n">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="J45" s="10" t="n">
         <v>46501</v>
@@ -2471,7 +2471,7 @@
         </is>
       </c>
       <c r="L45" s="9" t="n">
-        <v>0.02094192059635391</v>
+        <v>0.02054606845136392</v>
       </c>
     </row>
     <row r="46">
@@ -2506,7 +2506,7 @@
         <v>46492</v>
       </c>
       <c r="I46" s="13" t="n">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="J46" s="10" t="n">
         <v>46376</v>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="L46" s="9" t="n">
-        <v>0.04458430971857457</v>
+        <v>0.04476107994622253</v>
       </c>
     </row>
     <row r="47">
@@ -2552,7 +2552,7 @@
         <v>46493</v>
       </c>
       <c r="I47" s="13" t="n">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="J47" s="10" t="n">
         <v>46531</v>
@@ -2563,7 +2563,7 @@
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>0.02130841688416513</v>
+        <v>0.02065192195241944</v>
       </c>
     </row>
     <row r="48">
@@ -2598,7 +2598,7 @@
         <v>46499</v>
       </c>
       <c r="I48" s="13" t="n">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="J48" s="10" t="n">
         <v>46526</v>
@@ -2609,7 +2609,7 @@
         </is>
       </c>
       <c r="L48" s="9" t="n">
-        <v>0.02441485952410356</v>
+        <v>0.02415137438644563</v>
       </c>
     </row>
     <row r="49">
@@ -2644,7 +2644,7 @@
         <v>46504</v>
       </c>
       <c r="I49" s="13" t="n">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>46562</v>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>0.04384324606982604</v>
+        <v>0.04572614035505651</v>
       </c>
     </row>
     <row r="50">
@@ -2690,7 +2690,7 @@
         <v>46508</v>
       </c>
       <c r="I50" s="13" t="n">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="J50" s="10" t="n">
         <v>46518</v>
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="L50" s="9" t="n">
-        <v>0.03992953641939923</v>
+        <v>0.03958749238662681</v>
       </c>
     </row>
     <row r="51">
@@ -2736,7 +2736,7 @@
         <v>46515</v>
       </c>
       <c r="I51" s="13" t="n">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="J51" s="10" t="n">
         <v>46542</v>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>0.04207533851033222</v>
+        <v>0.04294837557547061</v>
       </c>
     </row>
     <row r="52">
@@ -2782,7 +2782,7 @@
         <v>46532</v>
       </c>
       <c r="I52" s="13" t="n">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="J52" s="10" t="n">
         <v>46563</v>
@@ -2793,7 +2793,7 @@
         </is>
       </c>
       <c r="L52" s="9" t="n">
-        <v>0.03319884726224784</v>
+        <v>0.032745879476208</v>
       </c>
     </row>
     <row r="53">
@@ -2822,13 +2822,13 @@
         <v>0.02985074626865658</v>
       </c>
       <c r="G53" s="9" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="H53" s="10" t="n">
         <v>46585</v>
       </c>
       <c r="I53" s="13" t="n">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="J53" s="10" t="n">
         <v>46629</v>
@@ -2839,7 +2839,7 @@
         </is>
       </c>
       <c r="L53" s="9" t="n">
-        <v>0.01891155700127388</v>
+        <v>0.0187831764947777</v>
       </c>
     </row>
     <row r="54">
@@ -2874,7 +2874,7 @@
         <v>46592</v>
       </c>
       <c r="I54" s="13" t="n">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="J54" s="10" t="n">
         <v>46613</v>
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="L54" s="9" t="n">
-        <v>0.02334008683068017</v>
+        <v>0.02328078955576035</v>
       </c>
     </row>
     <row r="55">
@@ -2914,13 +2914,13 @@
         <v>0.01219512195121952</v>
       </c>
       <c r="G55" s="9" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="H55" s="10" t="n">
         <v>46592</v>
       </c>
       <c r="I55" s="13" t="n">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="J55" s="10" t="n">
         <v>46632</v>
@@ -2931,7 +2931,7 @@
         </is>
       </c>
       <c r="L55" s="9" t="n">
-        <v>0.03401290830079057</v>
+        <v>0.03264824388132927</v>
       </c>
     </row>
     <row r="56">
@@ -2966,7 +2966,7 @@
         <v>46597</v>
       </c>
       <c r="I56" s="13" t="n">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="J56" s="10" t="n">
         <v>46611</v>
@@ -2977,7 +2977,7 @@
         </is>
       </c>
       <c r="L56" s="9" t="n">
-        <v>0.05011619620918463</v>
+        <v>0.04685433564521427</v>
       </c>
     </row>
     <row r="57">
@@ -3012,7 +3012,7 @@
         <v>46598</v>
       </c>
       <c r="I57" s="13" t="n">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="J57" s="10" t="n">
         <v>46629</v>
@@ -3023,7 +3023,7 @@
         </is>
       </c>
       <c r="L57" s="9" t="n">
-        <v>0.02462347489632013</v>
+        <v>0.02498938631660392</v>
       </c>
     </row>
   </sheetData>
@@ -3058,7 +3058,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Expected Increase Announcements by Month - 08/03/2026</t>
+          <t>Expected Increase Announcements by Month - 08/10/2026</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4155,7 @@
         <v>46608</v>
       </c>
       <c r="D59" s="7" t="n">
-        <v>0.545</v>
+        <v>0.531</v>
       </c>
       <c r="E59" s="8" t="n">
         <v>0.005735494868956323</v>
@@ -4817,7 +4817,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete Holdings Dividend Summary - 08/03/2026</t>
+          <t>Complete Holdings Dividend Summary - 08/10/2026</t>
         </is>
       </c>
     </row>
@@ -4921,7 +4921,7 @@
         <v>1.16</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.009990526172614474</v>
+        <v>0.009624239863116651</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>46160</v>
@@ -4974,7 +4974,7 @@
         <v>10.08</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.02628216836253416</v>
+        <v>0.02469498794862927</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>46157</v>
@@ -5027,7 +5027,7 @@
         <v>8.552</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.005269790339653252</v>
+        <v>0.004852845587305765</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>46231</v>
@@ -5080,7 +5080,7 @@
         <v>2.016</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.02334008683068017</v>
+        <v>0.02328078955576035</v>
       </c>
       <c r="I8" s="10" t="n">
         <v>46160</v>
@@ -5133,7 +5133,7 @@
         <v>2.812</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.03922443721909909</v>
+        <v>0.03816244952391996</v>
       </c>
       <c r="I9" s="10" t="n">
         <v>46157</v>
@@ -5186,7 +5186,7 @@
         <v>4.12</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.02462347489632013</v>
+        <v>0.02498938631660392</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>46171</v>
@@ -5239,7 +5239,7 @@
         <v>4.96</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.05011619620918463</v>
+        <v>0.04685433564521427</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>46134</v>
@@ -5292,7 +5292,7 @@
         <v>5.2</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.01936685288640596</v>
+        <v>0.01958863922015894</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>46182</v>
@@ -5345,7 +5345,7 @@
         <v>0.92</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0.0217365619235988</v>
+        <v>0.02281746049016211</v>
       </c>
       <c r="I13" s="10" t="n">
         <v>46163</v>
@@ -5398,7 +5398,7 @@
         <v>2.4</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0.007708366638676293</v>
+        <v>0.007434598707771089</v>
       </c>
       <c r="I14" s="10" t="n">
         <v>46157</v>
@@ -5451,7 +5451,7 @@
         <v>1.68</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.01464562822254793</v>
+        <v>0.01348531044555835</v>
       </c>
       <c r="I15" s="10" t="n">
         <v>46209</v>
@@ -5504,7 +5504,7 @@
         <v>7.12</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.03662834169923343</v>
+        <v>0.0370929935566493</v>
       </c>
       <c r="I16" s="10" t="n">
         <v>46161</v>
@@ -5557,7 +5557,7 @@
         <v>3.44</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.01483525930464986</v>
+        <v>0.01441199867951928</v>
       </c>
       <c r="I17" s="10" t="n">
         <v>46211</v>
@@ -5610,7 +5610,7 @@
         <v>1.28</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.02897238549475621</v>
+        <v>0.02870598779142888</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>46188</v>
@@ -5663,7 +5663,7 @@
         <v>3.36</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.0469044447518852</v>
+        <v>0.04619826543263427</v>
       </c>
       <c r="I19" s="10" t="n">
         <v>46188</v>
@@ -5716,7 +5716,7 @@
         <v>2.56</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.02364677581271972</v>
+        <v>0.02411681547998738</v>
       </c>
       <c r="I20" s="10" t="n">
         <v>46143</v>
@@ -5769,7 +5769,7 @@
         <v>6.36</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.01652141216985137</v>
+        <v>0.01607603275490687</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>46205</v>
@@ -5822,7 +5822,7 @@
         <v>1.18</v>
       </c>
       <c r="H22" s="18" t="n">
-        <v>0.01460124932688757</v>
+        <v>0.01421429872523905</v>
       </c>
       <c r="I22" s="19" t="n">
         <v>46223</v>
@@ -5875,7 +5875,7 @@
         <v>9.32</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.02755765719575049</v>
+        <v>0.02673512917565468</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>46177</v>
@@ -5928,7 +5928,7 @@
         <v>5.52</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>0.01652496664709451</v>
+        <v>0.01697208266431864</v>
       </c>
       <c r="I24" s="10" t="n">
         <v>46171</v>
@@ -5981,7 +5981,7 @@
         <v>1.172</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.04628752030512757</v>
+        <v>0.04698336397427078</v>
       </c>
       <c r="I25" s="10" t="n">
         <v>46216</v>
@@ -6034,7 +6034,7 @@
         <v>3.28</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>0.03246881913478192</v>
+        <v>0.03144171788339006</v>
       </c>
       <c r="I26" s="10" t="n">
         <v>46204</v>
@@ -6087,7 +6087,7 @@
         <v>2.44</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.01546359150656252</v>
+        <v>0.01567518914683119</v>
       </c>
       <c r="I27" s="10" t="n">
         <v>46174</v>
@@ -6140,7 +6140,7 @@
         <v>5.36</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0.02130841688416513</v>
+        <v>0.02065192195241944</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>46168</v>
@@ -6193,7 +6193,7 @@
         <v>6</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.01696496669833159</v>
+        <v>0.0167126259346279</v>
       </c>
       <c r="I29" s="10" t="n">
         <v>46209</v>
@@ -6246,7 +6246,7 @@
         <v>2.25</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.02094192059635391</v>
+        <v>0.02054606845136392</v>
       </c>
       <c r="I30" s="10" t="n">
         <v>46216</v>
@@ -6299,7 +6299,7 @@
         <v>3.16</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0.01183786607889024</v>
+        <v>0.01124795320189071</v>
       </c>
       <c r="I31" s="10" t="n">
         <v>46203</v>
@@ -6352,7 +6352,7 @@
         <v>2.88</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.03319884726224784</v>
+        <v>0.032745879476208</v>
       </c>
       <c r="I32" s="10" t="n">
         <v>46199</v>
@@ -6405,7 +6405,7 @@
         <v>1.92</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0.03667621883406817</v>
+        <v>0.03608344358269835</v>
       </c>
       <c r="I33" s="10" t="n">
         <v>46209</v>
@@ -6458,7 +6458,7 @@
         <v>3.64</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0.007421150426047773</v>
+        <v>0.007172413793103448</v>
       </c>
       <c r="I34" s="10" t="n">
         <v>46163</v>
@@ -6511,7 +6511,7 @@
         <v>3.48</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0.02787791355406566</v>
+        <v>0.02837226394875147</v>
       </c>
       <c r="I35" s="10" t="n">
         <v>46211</v>
@@ -6564,7 +6564,7 @@
         <v>1.64</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0.03870206489675516</v>
+        <v>0.03984935120019991</v>
       </c>
       <c r="I36" s="10" t="n">
         <v>46174</v>
@@ -6617,7 +6617,7 @@
         <v>2.55</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.05467410020090957</v>
+        <v>0.05449882346879326</v>
       </c>
       <c r="I37" s="10" t="n">
         <v>46111</v>
@@ -6670,7 +6670,7 @@
         <v>3.252</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0.05085222769668224</v>
+        <v>0.05274083697774267</v>
       </c>
       <c r="I38" s="10" t="n">
         <v>46234</v>
@@ -6723,7 +6723,7 @@
         <v>4.76</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.03992953641939923</v>
+        <v>0.03958749238662681</v>
       </c>
       <c r="I39" s="10" t="n">
         <v>46231</v>
@@ -6776,7 +6776,7 @@
         <v>2.68</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.03485498792136554</v>
+        <v>0.03592493371068497</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>46182</v>
@@ -6829,7 +6829,7 @@
         <v>5.92</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0.04207533851033222</v>
+        <v>0.04294837557547061</v>
       </c>
       <c r="I41" s="10" t="n">
         <v>46178</v>
@@ -6882,7 +6882,7 @@
         <v>1.72</v>
       </c>
       <c r="H42" s="9" t="n">
-        <v>0.06860789872107974</v>
+        <v>0.06394052135283915</v>
       </c>
       <c r="I42" s="10" t="n">
         <v>46227</v>
@@ -6935,7 +6935,7 @@
         <v>3.28</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0.028464808682162</v>
+        <v>0.02885165211275545</v>
       </c>
       <c r="I43" s="10" t="n">
         <v>46174</v>
@@ -6988,7 +6988,7 @@
         <v>4.356</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.02980703447511133</v>
+        <v>0.03004552440590653</v>
       </c>
       <c r="I44" s="10" t="n">
         <v>46227</v>
@@ -7041,7 +7041,7 @@
         <v>2.204</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>0.04384324606982604</v>
+        <v>0.04572614035505651</v>
       </c>
       <c r="I45" s="10" t="n">
         <v>46198</v>
@@ -7094,7 +7094,7 @@
         <v>5.08</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.02441485952410356</v>
+        <v>0.02415137438644563</v>
       </c>
       <c r="I46" s="10" t="n">
         <v>46160</v>
@@ -7147,7 +7147,7 @@
         <v>3.72</v>
       </c>
       <c r="H47" s="9" t="n">
-        <v>0.01558898681591544</v>
+        <v>0.0151124292354321</v>
       </c>
       <c r="I47" s="10" t="n">
         <v>46161</v>
@@ -7200,7 +7200,7 @@
         <v>9.76</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>0.02348807553888279</v>
+        <v>0.02341566388645527</v>
       </c>
       <c r="I48" s="10" t="n">
         <v>46162</v>
@@ -7253,7 +7253,7 @@
         <v>3.32</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.03401290830079057</v>
+        <v>0.03264824388132927</v>
       </c>
       <c r="I49" s="10" t="n">
         <v>46181</v>
@@ -7306,7 +7306,7 @@
         <v>5.2</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.04623660844994903</v>
+        <v>0.04571428571428571</v>
       </c>
       <c r="I50" s="10" t="n">
         <v>46188</v>
@@ -7359,7 +7359,7 @@
         <v>3.896</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.04458430971857457</v>
+        <v>0.04476107994622253</v>
       </c>
       <c r="I51" s="10" t="n">
         <v>46112</v>
@@ -7412,7 +7412,7 @@
         <v>5.68</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.0213317318299373</v>
+        <v>0.02001550505473602</v>
       </c>
       <c r="I52" s="10" t="n">
         <v>46234</v>
@@ -7459,16 +7459,16 @@
         </is>
       </c>
       <c r="F53" s="7" t="n">
-        <v>0.545</v>
+        <v>0.531</v>
       </c>
       <c r="G53" s="24" t="n">
-        <v>2.18</v>
+        <v>2.124</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>0.03400405520582705</v>
+        <v>0.03411226243990159</v>
       </c>
       <c r="I53" s="10" t="n">
-        <v>46157</v>
+        <v>46241</v>
       </c>
       <c r="J53" s="8" t="n">
         <v>0.005735494868956323</v>
@@ -7518,7 +7518,7 @@
         <v>5.52</v>
       </c>
       <c r="H54" s="9" t="n">
-        <v>0.01891155700127388</v>
+        <v>0.0187831764947777</v>
       </c>
       <c r="I54" s="10" t="n">
         <v>46171</v>
@@ -7571,7 +7571,7 @@
         <v>2.832</v>
       </c>
       <c r="H55" s="9" t="n">
-        <v>0.05979729652666019</v>
+        <v>0.06105422232354177</v>
       </c>
       <c r="I55" s="10" t="n">
         <v>46213</v>
@@ -7624,7 +7624,7 @@
         <v>4.12</v>
       </c>
       <c r="H56" s="9" t="n">
-        <v>0.02665286551427834</v>
+        <v>0.02609824759533807</v>
       </c>
       <c r="I56" s="10" t="n">
         <v>46157</v>

</xml_diff>

<commit_message>
Update dividend calendar 2026-08-24
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estimated Dividend Calendar: Anticipated Announcements - 08/17/2026</t>
+          <t>Estimated Dividend Calendar: Anticipated Announcements - 08/24/2026</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
         <v>46048</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-203</v>
+        <v>-210</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>46413</v>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="L6" s="9" t="n">
-        <v>0.06420689396395274</v>
+        <v>0.06156357035591447</v>
       </c>
     </row>
     <row r="7">
@@ -726,7 +726,7 @@
         <v>46263</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>46297</v>
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.03160531931567462</v>
+        <v>0.03052582683254938</v>
       </c>
     </row>
     <row r="8">
@@ -772,7 +772,7 @@
         <v>46278</v>
       </c>
       <c r="I8" s="14" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>46344</v>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.007508715643487043</v>
+        <v>0.00746459939730233</v>
       </c>
     </row>
     <row r="9">
@@ -818,10 +818,10 @@
         <v>46280</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>46303</v>
+        <v>46668</v>
       </c>
       <c r="K9" s="12" t="inlineStr">
         <is>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>0.05849970615865919</v>
+        <v>0.05682182968157457</v>
       </c>
     </row>
     <row r="10">
@@ -864,7 +864,7 @@
         <v>46285</v>
       </c>
       <c r="I10" s="14" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>46325</v>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.0199848708660232</v>
+        <v>0.02203856655366886</v>
       </c>
     </row>
     <row r="11">
@@ -910,7 +910,7 @@
         <v>46305</v>
       </c>
       <c r="I11" s="14" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46339</v>
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.02817585571864528</v>
+        <v>0.02885811514786943</v>
       </c>
     </row>
     <row r="12">
@@ -956,7 +956,7 @@
         <v>46311</v>
       </c>
       <c r="I12" s="14" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>46386</v>
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0.0111426505629441</v>
+        <v>0.01113362059047492</v>
       </c>
     </row>
     <row r="13">
@@ -1002,7 +1002,7 @@
         <v>46317</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>46351</v>
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>0.01696165179016014</v>
+        <v>0.01876465903400463</v>
       </c>
     </row>
     <row r="14">
@@ -1048,7 +1048,7 @@
         <v>46322</v>
       </c>
       <c r="I14" s="14" t="n">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>46338</v>
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.02370150865075563</v>
+        <v>0.02439024411518612</v>
       </c>
     </row>
     <row r="15">
@@ -1094,7 +1094,7 @@
         <v>46329</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>46338</v>
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>0.007609022827010429</v>
+        <v>0.007486664208023313</v>
       </c>
     </row>
     <row r="16">
@@ -1140,7 +1140,7 @@
         <v>46332</v>
       </c>
       <c r="I16" s="14" t="n">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>46346</v>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="L16" s="9" t="n">
-        <v>0.02426351771286513</v>
+        <v>0.02453370826079572</v>
       </c>
     </row>
     <row r="17">
@@ -1186,7 +1186,7 @@
         <v>46341</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>46340</v>
@@ -1197,7 +1197,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.02567218110309963</v>
+        <v>0.02511582643638334</v>
       </c>
     </row>
     <row r="18">
@@ -1232,7 +1232,7 @@
         <v>46344</v>
       </c>
       <c r="I18" s="14" t="n">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>46385</v>
@@ -1243,7 +1243,7 @@
         </is>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.03505248647218896</v>
+        <v>0.03417038972317595</v>
       </c>
     </row>
     <row r="19">
@@ -1278,7 +1278,7 @@
         <v>46347</v>
       </c>
       <c r="I19" s="14" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>46358</v>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0.04146261970446818</v>
+        <v>0.03991199823387459</v>
       </c>
     </row>
     <row r="20">
@@ -1324,7 +1324,7 @@
         <v>46352</v>
       </c>
       <c r="I20" s="14" t="n">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>46400</v>
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0.04853002147050658</v>
+        <v>0.04855012550259507</v>
       </c>
     </row>
     <row r="21">
@@ -1370,7 +1370,7 @@
         <v>46360</v>
       </c>
       <c r="I21" s="14" t="n">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46371</v>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.04597386662229366</v>
+        <v>0.04544224897291059</v>
       </c>
     </row>
     <row r="22">
@@ -1416,7 +1416,7 @@
         <v>46366</v>
       </c>
       <c r="I22" s="14" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="J22" s="10" t="n">
         <v>46432</v>
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="L22" s="9" t="n">
-        <v>0.02422494557111912</v>
+        <v>0.02286760765227264</v>
       </c>
     </row>
     <row r="23">
@@ -1447,19 +1447,19 @@
         </is>
       </c>
       <c r="D23" s="7" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="E23" s="7" t="n">
         <v>0.23</v>
       </c>
-      <c r="E23" s="7" t="n">
-        <v>0.22</v>
-      </c>
       <c r="F23" s="8" t="n">
-        <v>0.0454545454545455</v>
+        <v>0.04347826086956513</v>
       </c>
       <c r="G23" s="9" t="n">
         <v>0.04</v>
       </c>
       <c r="H23" s="10" t="n">
-        <v>46373</v>
+        <v>46380</v>
       </c>
       <c r="I23" s="14" t="n">
         <v>122</v>
@@ -1473,7 +1473,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0.02266568111706065</v>
+        <v>0.02475502914436672</v>
       </c>
     </row>
     <row r="24">
@@ -1508,7 +1508,7 @@
         <v>46383</v>
       </c>
       <c r="I24" s="21" t="n">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="J24" s="20" t="n">
         <v>46404</v>
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="L24" s="19" t="n">
-        <v>0.01451950349133763</v>
+        <v>0.01450522461134869</v>
       </c>
     </row>
     <row r="25">
@@ -1554,7 +1554,7 @@
         <v>46402</v>
       </c>
       <c r="I25" s="14" t="n">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>46483</v>
@@ -1565,7 +1565,7 @@
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>0.01465139102332933</v>
+        <v>0.01403680539107752</v>
       </c>
     </row>
     <row r="26">
@@ -1600,7 +1600,7 @@
         <v>46411</v>
       </c>
       <c r="I26" s="14" t="n">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>46435</v>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0.03830540607167161</v>
+        <v>0.03921896959116871</v>
       </c>
     </row>
     <row r="27">
@@ -1646,7 +1646,7 @@
         <v>46417</v>
       </c>
       <c r="I27" s="14" t="n">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>46433</v>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="L27" s="9" t="n">
-        <v>0.03536482359929009</v>
+        <v>0.03486606809614539</v>
       </c>
     </row>
     <row r="28">
@@ -1677,7 +1677,7 @@
         </is>
       </c>
       <c r="D28" s="7" t="n">
-        <v>1.275</v>
+        <v>0.579</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>0.584</v>
@@ -1692,7 +1692,7 @@
         <v>46423</v>
       </c>
       <c r="I28" s="14" t="n">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>46473</v>
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="L28" s="9" t="n">
-        <v>0.05646589921647503</v>
+        <v>0.02462781771004423</v>
       </c>
     </row>
     <row r="29">
@@ -1738,7 +1738,7 @@
         <v>46428</v>
       </c>
       <c r="I29" s="14" t="n">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>46452</v>
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>0.01620777860226065</v>
+        <v>0.01436646286276235</v>
       </c>
     </row>
     <row r="30">
@@ -1784,7 +1784,7 @@
         <v>46428</v>
       </c>
       <c r="I30" s="14" t="n">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="J30" s="10" t="n">
         <v>46460</v>
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="L30" s="9" t="n">
-        <v>0.0471762310908162</v>
+        <v>0.04661168979740114</v>
       </c>
     </row>
     <row r="31">
@@ -1830,7 +1830,7 @@
         <v>46431</v>
       </c>
       <c r="I31" s="14" t="n">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>46480</v>
@@ -1841,7 +1841,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="n">
-        <v>0.01483181822008854</v>
+        <v>0.01533686311811834</v>
       </c>
     </row>
     <row r="32">
@@ -1876,7 +1876,7 @@
         <v>46432</v>
       </c>
       <c r="I32" s="14" t="n">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>46455</v>
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="L32" s="9" t="n">
-        <v>0.03547319512567042</v>
+        <v>0.03663203753211416</v>
       </c>
     </row>
     <row r="33">
@@ -1922,7 +1922,7 @@
         <v>46433</v>
       </c>
       <c r="I33" s="14" t="n">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>46425</v>
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>0.004565912598123347</v>
+        <v>0.004937215292389725</v>
       </c>
     </row>
     <row r="34">
@@ -1968,7 +1968,7 @@
         <v>46433</v>
       </c>
       <c r="I34" s="14" t="n">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>46383</v>
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="L34" s="9" t="n">
-        <v>0.01919782524635881</v>
+        <v>0.01873873873873874</v>
       </c>
     </row>
     <row r="35">
@@ -2014,7 +2014,7 @@
         <v>46433</v>
       </c>
       <c r="I35" s="14" t="n">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>46368</v>
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0.02756838233010548</v>
+        <v>0.02629956951214198</v>
       </c>
     </row>
     <row r="36">
@@ -2060,7 +2060,7 @@
         <v>46433</v>
       </c>
       <c r="I36" s="14" t="n">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>46635</v>
@@ -2071,7 +2071,7 @@
         </is>
       </c>
       <c r="L36" s="9" t="n">
-        <v>0.02844752743438886</v>
+        <v>0.02919292176686114</v>
       </c>
     </row>
     <row r="37">
@@ -2106,7 +2106,7 @@
         <v>46433</v>
       </c>
       <c r="I37" s="14" t="n">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>46608</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>0.03470021290261385</v>
+        <v>0.03261921323323592</v>
       </c>
     </row>
     <row r="38">
@@ -2152,7 +2152,7 @@
         <v>46440</v>
       </c>
       <c r="I38" s="14" t="n">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>46450</v>
@@ -2163,7 +2163,7 @@
         </is>
       </c>
       <c r="L38" s="9" t="n">
-        <v>0.009264435815684403</v>
+        <v>0.008765169347060732</v>
       </c>
     </row>
     <row r="39">
@@ -2198,7 +2198,7 @@
         <v>46441</v>
       </c>
       <c r="I39" s="14" t="n">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>46456</v>
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.02797286813397985</v>
+        <v>0.02728536827029688</v>
       </c>
     </row>
     <row r="40">
@@ -2244,7 +2244,7 @@
         <v>46452</v>
       </c>
       <c r="I40" s="14" t="n">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="J40" s="10" t="n">
         <v>46487</v>
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.01617867832665757</v>
+        <v>0.01650469054964427</v>
       </c>
     </row>
     <row r="41">
@@ -2290,7 +2290,7 @@
         <v>46461</v>
       </c>
       <c r="I41" s="14" t="n">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>46300</v>
@@ -2301,7 +2301,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>0.01644962302947224</v>
+        <v>0.01681119631420541</v>
       </c>
     </row>
     <row r="42">
@@ -2336,7 +2336,7 @@
         <v>46461</v>
       </c>
       <c r="I42" s="14" t="n">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="J42" s="10" t="n">
         <v>46386</v>
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="L42" s="9" t="n">
-        <v>0.05213627254509019</v>
+        <v>0.05137432770585006</v>
       </c>
     </row>
     <row r="43">
@@ -2382,7 +2382,7 @@
         <v>46488</v>
       </c>
       <c r="I43" s="14" t="n">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>46498</v>
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>0.03035751504105644</v>
+        <v>0.02976222999340377</v>
       </c>
     </row>
     <row r="44">
@@ -2428,7 +2428,7 @@
         <v>46492</v>
       </c>
       <c r="I44" s="14" t="n">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="J44" s="10" t="n">
         <v>46501</v>
@@ -2439,7 +2439,7 @@
         </is>
       </c>
       <c r="L44" s="9" t="n">
-        <v>0.02073541568246589</v>
+        <v>0.01991679185347889</v>
       </c>
     </row>
     <row r="45">
@@ -2474,7 +2474,7 @@
         <v>46492</v>
       </c>
       <c r="I45" s="14" t="n">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="J45" s="10" t="n">
         <v>46376</v>
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="L45" s="9" t="n">
-        <v>0.04405993627978225</v>
+        <v>0.04394062597018357</v>
       </c>
     </row>
     <row r="46">
@@ -2520,7 +2520,7 @@
         <v>46493</v>
       </c>
       <c r="I46" s="14" t="n">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="J46" s="10" t="n">
         <v>46531</v>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="L46" s="9" t="n">
-        <v>0.02049948359267303</v>
+        <v>0.01976911409091994</v>
       </c>
     </row>
     <row r="47">
@@ -2566,7 +2566,7 @@
         <v>46499</v>
       </c>
       <c r="I47" s="14" t="n">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="J47" s="10" t="n">
         <v>46526</v>
@@ -2577,7 +2577,7 @@
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>0.02132393103767646</v>
+        <v>0.02090879099284308</v>
       </c>
     </row>
     <row r="48">
@@ -2612,7 +2612,7 @@
         <v>46504</v>
       </c>
       <c r="I48" s="14" t="n">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="J48" s="10" t="n">
         <v>46562</v>
@@ -2623,7 +2623,7 @@
         </is>
       </c>
       <c r="L48" s="9" t="n">
-        <v>0.04340291557664582</v>
+        <v>0.04455225279189258</v>
       </c>
     </row>
     <row r="49">
@@ -2658,7 +2658,7 @@
         <v>46508</v>
       </c>
       <c r="I49" s="14" t="n">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>46518</v>
@@ -2669,7 +2669,7 @@
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>0.0397644202597149</v>
+        <v>0.03756016628985256</v>
       </c>
     </row>
     <row r="50">
@@ -2704,7 +2704,7 @@
         <v>46515</v>
       </c>
       <c r="I50" s="14" t="n">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="J50" s="10" t="n">
         <v>46542</v>
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="L50" s="9" t="n">
-        <v>0.04272208766034556</v>
+        <v>0.04064538447016642</v>
       </c>
     </row>
     <row r="51">
@@ -2750,7 +2750,7 @@
         <v>46532</v>
       </c>
       <c r="I51" s="14" t="n">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="J51" s="10" t="n">
         <v>46563</v>
@@ -2761,13 +2761,13 @@
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>0.03158933923266214</v>
+        <v>0.03071017314446581</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>RGA</t>
+          <t>UNP</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -2781,25 +2781,25 @@
         </is>
       </c>
       <c r="D52" s="7" t="n">
-        <v>0.93</v>
+        <v>1.38</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>0.89</v>
+        <v>1.34</v>
       </c>
       <c r="F52" s="8" t="n">
-        <v>0.04494382022471914</v>
+        <v>0.02985074626865658</v>
       </c>
       <c r="G52" s="9" t="n">
         <v>0.06</v>
       </c>
       <c r="H52" s="10" t="n">
-        <v>46583</v>
+        <v>46585</v>
       </c>
       <c r="I52" s="14" t="n">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="J52" s="10" t="n">
-        <v>46613</v>
+        <v>46629</v>
       </c>
       <c r="K52" s="12" t="inlineStr">
         <is>
@@ -2807,13 +2807,13 @@
         </is>
       </c>
       <c r="L52" s="9" t="n">
-        <v>0.01490384578939962</v>
+        <v>0.01778722342210357</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>UNP</t>
+          <t>SWK</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -2823,29 +2823,29 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Aug</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
-        <v>1.38</v>
+        <v>0.83</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>1.34</v>
+        <v>0.82</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>0.02985074626865658</v>
+        <v>0.01219512195121952</v>
       </c>
       <c r="G53" s="9" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="H53" s="10" t="n">
-        <v>46585</v>
+        <v>46592</v>
       </c>
       <c r="I53" s="14" t="n">
         <v>334</v>
       </c>
       <c r="J53" s="10" t="n">
-        <v>46629</v>
+        <v>46632</v>
       </c>
       <c r="K53" s="12" t="inlineStr">
         <is>
@@ -2853,13 +2853,13 @@
         </is>
       </c>
       <c r="L53" s="9" t="n">
-        <v>0.01846030433687031</v>
+        <v>0.03298231550978693</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>AWR</t>
+          <t>RGA</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -2873,39 +2873,39 @@
         </is>
       </c>
       <c r="D54" s="7" t="n">
-        <v>0.504</v>
+        <v>0.98</v>
       </c>
       <c r="E54" s="7" t="n">
-        <v>0.466</v>
+        <v>0.93</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>0.08154506437768236</v>
+        <v>0.05376344086021498</v>
       </c>
       <c r="G54" s="9" t="n">
         <v>0.06</v>
       </c>
       <c r="H54" s="10" t="n">
-        <v>46592</v>
+        <v>46594</v>
       </c>
       <c r="I54" s="14" t="n">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="J54" s="10" t="n">
         <v>46613</v>
       </c>
       <c r="K54" s="12" t="inlineStr">
         <is>
-          <t>yfinance</t>
+          <t>Notion + yfinance</t>
         </is>
       </c>
       <c r="L54" s="9" t="n">
-        <v>0.02292730261599521</v>
+        <v>0.01592686642965973</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>SWK</t>
+          <t>AWR</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
@@ -2915,29 +2915,29 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>Aug</t>
         </is>
       </c>
       <c r="D55" s="7" t="n">
-        <v>0.83</v>
+        <v>0.546</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>0.82</v>
+        <v>0.504</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>0.01219512195121952</v>
+        <v>0.08333333333333341</v>
       </c>
       <c r="G55" s="9" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="H55" s="10" t="n">
-        <v>46592</v>
+        <v>46595</v>
       </c>
       <c r="I55" s="14" t="n">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="J55" s="10" t="n">
-        <v>46632</v>
+        <v>46614</v>
       </c>
       <c r="K55" s="12" t="inlineStr">
         <is>
@@ -2945,7 +2945,7 @@
         </is>
       </c>
       <c r="L55" s="9" t="n">
-        <v>0.03327320144935559</v>
+        <v>0.02452830163458748</v>
       </c>
     </row>
     <row r="56">
@@ -2980,7 +2980,7 @@
         <v>46597</v>
       </c>
       <c r="I56" s="14" t="n">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="J56" s="10" t="n">
         <v>46611</v>
@@ -2991,7 +2991,7 @@
         </is>
       </c>
       <c r="L56" s="9" t="n">
-        <v>0.04719207309125793</v>
+        <v>0.04599181500645778</v>
       </c>
     </row>
     <row r="57">
@@ -3026,7 +3026,7 @@
         <v>46598</v>
       </c>
       <c r="I57" s="14" t="n">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="J57" s="10" t="n">
         <v>46629</v>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="L57" s="9" t="n">
-        <v>0.02417982284616581</v>
+        <v>0.02484172353559332</v>
       </c>
     </row>
   </sheetData>
@@ -3072,7 +3072,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Expected Increase Announcements by Month - 08/17/2026</t>
+          <t>Expected Increase Announcements by Month - 08/24/2026</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
         <v>46280</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>46303</v>
+        <v>46668</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0.708</v>
@@ -3725,16 +3725,16 @@
         </is>
       </c>
       <c r="B38" s="10" t="n">
-        <v>46373</v>
+        <v>46380</v>
       </c>
       <c r="C38" s="10" t="n">
         <v>46436</v>
       </c>
       <c r="D38" s="7" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>0.0454545454545455</v>
+        <v>0.04347826086956513</v>
       </c>
       <c r="F38" s="12" t="inlineStr">
         <is>
@@ -3929,7 +3929,7 @@
         <v>46473</v>
       </c>
       <c r="D49" s="7" t="n">
-        <v>1.275</v>
+        <v>0.579</v>
       </c>
       <c r="E49" s="8" t="n">
         <v>1.183219178082192</v>
@@ -4651,20 +4651,20 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>RGA</t>
+          <t>UNP</t>
         </is>
       </c>
       <c r="B85" s="10" t="n">
-        <v>46583</v>
+        <v>46585</v>
       </c>
       <c r="C85" s="10" t="n">
-        <v>46613</v>
+        <v>46629</v>
       </c>
       <c r="D85" s="7" t="n">
-        <v>0.93</v>
+        <v>1.38</v>
       </c>
       <c r="E85" s="8" t="n">
-        <v>0.04494382022471914</v>
+        <v>0.02985074626865658</v>
       </c>
       <c r="F85" s="12" t="inlineStr">
         <is>
@@ -4675,20 +4675,20 @@
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>UNP</t>
+          <t>SWK</t>
         </is>
       </c>
       <c r="B86" s="10" t="n">
-        <v>46585</v>
+        <v>46592</v>
       </c>
       <c r="C86" s="10" t="n">
-        <v>46629</v>
+        <v>46632</v>
       </c>
       <c r="D86" s="7" t="n">
-        <v>1.38</v>
+        <v>0.83</v>
       </c>
       <c r="E86" s="8" t="n">
-        <v>0.02985074626865658</v>
+        <v>0.01219512195121952</v>
       </c>
       <c r="F86" s="12" t="inlineStr">
         <is>
@@ -4699,44 +4699,44 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>AWR</t>
+          <t>RGA</t>
         </is>
       </c>
       <c r="B87" s="10" t="n">
-        <v>46592</v>
+        <v>46594</v>
       </c>
       <c r="C87" s="10" t="n">
         <v>46613</v>
       </c>
       <c r="D87" s="7" t="n">
-        <v>0.504</v>
+        <v>0.98</v>
       </c>
       <c r="E87" s="8" t="n">
-        <v>0.08154506437768236</v>
+        <v>0.05376344086021498</v>
       </c>
       <c r="F87" s="12" t="inlineStr">
         <is>
-          <t>yfinance</t>
+          <t>Notion + yfinance</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>SWK</t>
+          <t>AWR</t>
         </is>
       </c>
       <c r="B88" s="10" t="n">
-        <v>46592</v>
+        <v>46595</v>
       </c>
       <c r="C88" s="10" t="n">
-        <v>46632</v>
+        <v>46614</v>
       </c>
       <c r="D88" s="7" t="n">
-        <v>0.83</v>
+        <v>0.546</v>
       </c>
       <c r="E88" s="8" t="n">
-        <v>0.01219512195121952</v>
+        <v>0.08333333333333341</v>
       </c>
       <c r="F88" s="12" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete Holdings Dividend Summary - 08/17/2026</t>
+          <t>Complete Holdings Dividend Summary - 08/24/2026</t>
         </is>
       </c>
     </row>
@@ -4935,10 +4935,10 @@
         <v>1.16</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.009264435815684403</v>
+        <v>0.008765169347060732</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>46160</v>
+        <v>46255</v>
       </c>
       <c r="J5" s="8" t="n">
         <v>0.07407407407407393</v>
@@ -4988,10 +4988,10 @@
         <v>10.08</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.02422494557111912</v>
+        <v>0.02286760765227264</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>46157</v>
+        <v>46255</v>
       </c>
       <c r="J6" s="8" t="n">
         <v>0.05882352941176476</v>
@@ -5041,7 +5041,7 @@
         <v>8.552</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.004565912598123347</v>
+        <v>0.004937215292389725</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>46231</v>
@@ -5088,29 +5088,29 @@
         </is>
       </c>
       <c r="F8" s="7" t="n">
-        <v>0.504</v>
+        <v>0.546</v>
       </c>
       <c r="G8" s="25" t="n">
-        <v>2.016</v>
+        <v>2.184</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.02292730261599521</v>
+        <v>0.02452830163458748</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>46160</v>
+        <v>46251</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>0.08154506437768236</v>
+        <v>0.08333333333333341</v>
       </c>
       <c r="K8" s="10" t="n">
-        <v>46592</v>
+        <v>46595</v>
       </c>
       <c r="L8" s="10" t="n">
-        <v>46613</v>
+        <v>46614</v>
       </c>
       <c r="M8" s="12" t="inlineStr">
         <is>
-          <t>yfinance</t>
+          <t>Notion + yfinance</t>
         </is>
       </c>
     </row>
@@ -5147,10 +5147,10 @@
         <v>2.812</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.03830540607167161</v>
+        <v>0.03921896959116871</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>46157</v>
+        <v>46251</v>
       </c>
       <c r="J9" s="8" t="n">
         <v>0.03994082840236673</v>
@@ -5200,7 +5200,7 @@
         <v>4.12</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.02417982284616581</v>
+        <v>0.02484172353559332</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>46171</v>
@@ -5253,7 +5253,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.04719207309125793</v>
+        <v>0.04599181500645778</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>46246</v>
@@ -5306,7 +5306,7 @@
         <v>5.2</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.01919782524635881</v>
+        <v>0.01873873873873874</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>46182</v>
@@ -5353,22 +5353,22 @@
         </is>
       </c>
       <c r="F13" s="7" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="G13" s="25" t="n">
-        <v>0.92</v>
+        <v>0.96</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0.02266568111706065</v>
+        <v>0.02475502914436672</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>46163</v>
+        <v>46254</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>0.0454545454545455</v>
+        <v>0.04347826086956513</v>
       </c>
       <c r="K13" s="10" t="n">
-        <v>46373</v>
+        <v>46380</v>
       </c>
       <c r="L13" s="10" t="n">
         <v>46436</v>
@@ -5412,7 +5412,7 @@
         <v>2.4</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0.007609022827010429</v>
+        <v>0.007486664208023313</v>
       </c>
       <c r="I14" s="10" t="n">
         <v>46248</v>
@@ -5465,7 +5465,7 @@
         <v>1.68</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.01483181822008854</v>
+        <v>0.01533686311811834</v>
       </c>
       <c r="I15" s="10" t="n">
         <v>46209</v>
@@ -5518,10 +5518,10 @@
         <v>7.12</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.03536482359929009</v>
+        <v>0.03486606809614539</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>46161</v>
+        <v>46253</v>
       </c>
       <c r="J16" s="8" t="n">
         <v>0.04093567251461992</v>
@@ -5571,7 +5571,7 @@
         <v>3.44</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.01465139102332933</v>
+        <v>0.01403680539107752</v>
       </c>
       <c r="I17" s="10" t="n">
         <v>46211</v>
@@ -5624,7 +5624,7 @@
         <v>1.28</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.02756838233010548</v>
+        <v>0.02629956951214198</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>46188</v>
@@ -5677,7 +5677,7 @@
         <v>3.36</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.04597386662229366</v>
+        <v>0.04544224897291059</v>
       </c>
       <c r="I19" s="10" t="n">
         <v>46188</v>
@@ -5730,7 +5730,7 @@
         <v>2.56</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.02370150865075563</v>
+        <v>0.02439024411518612</v>
       </c>
       <c r="I20" s="10" t="n">
         <v>46247</v>
@@ -5783,7 +5783,7 @@
         <v>6.36</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.01617867832665757</v>
+        <v>0.01650469054964427</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>46205</v>
@@ -5836,7 +5836,7 @@
         <v>1.18</v>
       </c>
       <c r="H22" s="19" t="n">
-        <v>0.01451950349133763</v>
+        <v>0.01450522461134869</v>
       </c>
       <c r="I22" s="20" t="n">
         <v>46223</v>
@@ -5889,7 +5889,7 @@
         <v>9.32</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.02797286813397985</v>
+        <v>0.02728536827029688</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>46177</v>
@@ -5942,7 +5942,7 @@
         <v>5.52</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>0.01696165179016014</v>
+        <v>0.01876465903400463</v>
       </c>
       <c r="I24" s="10" t="n">
         <v>46171</v>
@@ -5995,7 +5995,7 @@
         <v>1.172</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.04853002147050658</v>
+        <v>0.04855012550259507</v>
       </c>
       <c r="I25" s="10" t="n">
         <v>46216</v>
@@ -6048,7 +6048,7 @@
         <v>3.28</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>0.03160531931567462</v>
+        <v>0.03052582683254938</v>
       </c>
       <c r="I26" s="10" t="n">
         <v>46204</v>
@@ -6101,7 +6101,7 @@
         <v>2.44</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.01620777860226065</v>
+        <v>0.01436646286276235</v>
       </c>
       <c r="I27" s="10" t="n">
         <v>46174</v>
@@ -6154,7 +6154,7 @@
         <v>5.36</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0.02049948359267303</v>
+        <v>0.01976911409091994</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>46168</v>
@@ -6207,7 +6207,7 @@
         <v>6</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.01644962302947224</v>
+        <v>0.01681119631420541</v>
       </c>
       <c r="I29" s="10" t="n">
         <v>46209</v>
@@ -6260,7 +6260,7 @@
         <v>2.25</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.02073541568246589</v>
+        <v>0.01991679185347889</v>
       </c>
       <c r="I30" s="10" t="n">
         <v>46216</v>
@@ -6313,7 +6313,7 @@
         <v>3.16</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0.0111426505629441</v>
+        <v>0.01113362059047492</v>
       </c>
       <c r="I31" s="10" t="n">
         <v>46203</v>
@@ -6366,7 +6366,7 @@
         <v>2.88</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.03158933923266214</v>
+        <v>0.03071017314446581</v>
       </c>
       <c r="I32" s="10" t="n">
         <v>46199</v>
@@ -6419,7 +6419,7 @@
         <v>1.92</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0.03505248647218896</v>
+        <v>0.03417038972317595</v>
       </c>
       <c r="I33" s="10" t="n">
         <v>46209</v>
@@ -6472,10 +6472,10 @@
         <v>3.64</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0.007508715643487043</v>
+        <v>0.00746459939730233</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>46163</v>
+        <v>46254</v>
       </c>
       <c r="J34" s="8" t="n">
         <v>0.09638554216867479</v>
@@ -6525,7 +6525,7 @@
         <v>3.48</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0.02817585571864528</v>
+        <v>0.02885811514786943</v>
       </c>
       <c r="I35" s="10" t="n">
         <v>46211</v>
@@ -6578,7 +6578,7 @@
         <v>1.64</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0.04146261970446818</v>
+        <v>0.03991199823387459</v>
       </c>
       <c r="I36" s="10" t="n">
         <v>46174</v>
@@ -6625,16 +6625,16 @@
         </is>
       </c>
       <c r="F37" s="7" t="n">
-        <v>1.275</v>
+        <v>0.579</v>
       </c>
       <c r="G37" s="25" t="n">
-        <v>2.55</v>
+        <v>1.158</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.05646589921647503</v>
+        <v>0.02462781771004423</v>
       </c>
       <c r="I37" s="10" t="n">
-        <v>46111</v>
+        <v>46251</v>
       </c>
       <c r="J37" s="8" t="n">
         <v>1.183219178082192</v>
@@ -6684,7 +6684,7 @@
         <v>3.252</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0.05213627254509019</v>
+        <v>0.05137432770585006</v>
       </c>
       <c r="I38" s="10" t="n">
         <v>46234</v>
@@ -6737,7 +6737,7 @@
         <v>4.76</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.0397644202597149</v>
+        <v>0.03756016628985256</v>
       </c>
       <c r="I39" s="10" t="n">
         <v>46231</v>
@@ -6790,7 +6790,7 @@
         <v>2.68</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.03547319512567042</v>
+        <v>0.03663203753211416</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>46182</v>
@@ -6843,7 +6843,7 @@
         <v>5.92</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0.04272208766034556</v>
+        <v>0.04064538447016642</v>
       </c>
       <c r="I41" s="10" t="n">
         <v>46178</v>
@@ -6896,7 +6896,7 @@
         <v>1.72</v>
       </c>
       <c r="H42" s="9" t="n">
-        <v>0.06420689396395274</v>
+        <v>0.06156357035591447</v>
       </c>
       <c r="I42" s="10" t="n">
         <v>46227</v>
@@ -6949,7 +6949,7 @@
         <v>3.28</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0.02844752743438886</v>
+        <v>0.02919292176686114</v>
       </c>
       <c r="I43" s="10" t="n">
         <v>46174</v>
@@ -7002,7 +7002,7 @@
         <v>4.356</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.03035751504105644</v>
+        <v>0.02976222999340377</v>
       </c>
       <c r="I44" s="10" t="n">
         <v>46227</v>
@@ -7055,7 +7055,7 @@
         <v>2.204</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>0.04340291557664582</v>
+        <v>0.04455225279189258</v>
       </c>
       <c r="I45" s="10" t="n">
         <v>46198</v>
@@ -7108,10 +7108,10 @@
         <v>5.08</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.02132393103767646</v>
+        <v>0.02090879099284308</v>
       </c>
       <c r="I46" s="10" t="n">
-        <v>46160</v>
+        <v>46252</v>
       </c>
       <c r="J46" s="8" t="n">
         <v>0.05833333333333339</v>
@@ -7155,22 +7155,22 @@
         </is>
       </c>
       <c r="F47" s="7" t="n">
-        <v>0.93</v>
+        <v>0.98</v>
       </c>
       <c r="G47" s="25" t="n">
-        <v>3.72</v>
+        <v>3.92</v>
       </c>
       <c r="H47" s="9" t="n">
-        <v>0.01490384578939962</v>
+        <v>0.01592686642965973</v>
       </c>
       <c r="I47" s="10" t="n">
-        <v>46161</v>
+        <v>46252</v>
       </c>
       <c r="J47" s="8" t="n">
-        <v>0.04494382022471914</v>
+        <v>0.05376344086021498</v>
       </c>
       <c r="K47" s="10" t="n">
-        <v>46583</v>
+        <v>46594</v>
       </c>
       <c r="L47" s="10" t="n">
         <v>46613</v>
@@ -7214,10 +7214,10 @@
         <v>9.76</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>0.02426351771286513</v>
+        <v>0.02453370826079572</v>
       </c>
       <c r="I48" s="10" t="n">
-        <v>46162</v>
+        <v>46253</v>
       </c>
       <c r="J48" s="8" t="n">
         <v>0.1401869158878504</v>
@@ -7267,7 +7267,7 @@
         <v>3.32</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.03327320144935559</v>
+        <v>0.03298231550978693</v>
       </c>
       <c r="I49" s="10" t="n">
         <v>46181</v>
@@ -7320,7 +7320,7 @@
         <v>5.2</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.0471762310908162</v>
+        <v>0.04661168979740114</v>
       </c>
       <c r="I50" s="10" t="n">
         <v>46188</v>
@@ -7373,7 +7373,7 @@
         <v>3.896</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.04405993627978225</v>
+        <v>0.04394062597018357</v>
       </c>
       <c r="I51" s="10" t="n">
         <v>46112</v>
@@ -7426,7 +7426,7 @@
         <v>5.68</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.0199848708660232</v>
+        <v>0.02203856655366886</v>
       </c>
       <c r="I52" s="10" t="n">
         <v>46234</v>
@@ -7479,7 +7479,7 @@
         <v>2.124</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>0.03470021290261385</v>
+        <v>0.03261921323323592</v>
       </c>
       <c r="I53" s="10" t="n">
         <v>46241</v>
@@ -7532,7 +7532,7 @@
         <v>5.52</v>
       </c>
       <c r="H54" s="9" t="n">
-        <v>0.01846030433687031</v>
+        <v>0.01778722342210357</v>
       </c>
       <c r="I54" s="10" t="n">
         <v>46171</v>
@@ -7585,7 +7585,7 @@
         <v>2.832</v>
       </c>
       <c r="H55" s="9" t="n">
-        <v>0.05849970615865919</v>
+        <v>0.05682182968157457</v>
       </c>
       <c r="I55" s="10" t="n">
         <v>46213</v>
@@ -7597,7 +7597,7 @@
         <v>46280</v>
       </c>
       <c r="L55" s="10" t="n">
-        <v>46303</v>
+        <v>46668</v>
       </c>
       <c r="M55" s="12" t="inlineStr">
         <is>
@@ -7638,10 +7638,10 @@
         <v>4.12</v>
       </c>
       <c r="H56" s="9" t="n">
-        <v>0.02567218110309963</v>
+        <v>0.02511582643638334</v>
       </c>
       <c r="I56" s="10" t="n">
-        <v>46157</v>
+        <v>46251</v>
       </c>
       <c r="J56" s="8" t="n">
         <v>0.04040404040404044</v>

</xml_diff>

<commit_message>
Update dividend calendar 2026-08-31
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estimated Dividend Calendar: Anticipated Announcements - 08/24/2026</t>
+          <t>Estimated Dividend Calendar: Anticipated Announcements - 08/31/2026</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
         <v>46048</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-210</v>
+        <v>-217</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>46413</v>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="L6" s="9" t="n">
-        <v>0.06156357035591447</v>
+        <v>0.06160458435888048</v>
       </c>
     </row>
     <row r="7">
@@ -725,11 +725,11 @@
       <c r="H7" s="10" t="n">
         <v>46263</v>
       </c>
-      <c r="I7" s="13" t="n">
-        <v>5</v>
+      <c r="I7" s="11" t="n">
+        <v>-2</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>46297</v>
+        <v>46662</v>
       </c>
       <c r="K7" s="12" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.03052582683254938</v>
+        <v>0.03150967828940907</v>
       </c>
     </row>
     <row r="8">
@@ -771,8 +771,8 @@
       <c r="H8" s="10" t="n">
         <v>46278</v>
       </c>
-      <c r="I8" s="14" t="n">
-        <v>20</v>
+      <c r="I8" s="13" t="n">
+        <v>13</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>46344</v>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.00746459939730233</v>
+        <v>0.007159787328081065</v>
       </c>
     </row>
     <row r="9">
@@ -818,7 +818,7 @@
         <v>46280</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>46668</v>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>0.05682182968157457</v>
+        <v>0.05667400301816825</v>
       </c>
     </row>
     <row r="10">
@@ -864,7 +864,7 @@
         <v>46285</v>
       </c>
       <c r="I10" s="14" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>46325</v>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.02203856655366886</v>
+        <v>0.02174245985426699</v>
       </c>
     </row>
     <row r="11">
@@ -910,7 +910,7 @@
         <v>46305</v>
       </c>
       <c r="I11" s="14" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46339</v>
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.02885811514786943</v>
+        <v>0.02914084787605498</v>
       </c>
     </row>
     <row r="12">
@@ -956,7 +956,7 @@
         <v>46311</v>
       </c>
       <c r="I12" s="14" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>46386</v>
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0.01113362059047492</v>
+        <v>0.01116568280612038</v>
       </c>
     </row>
     <row r="13">
@@ -999,13 +999,13 @@
         <v>0.06</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>46351</v>
+        <v>46352</v>
       </c>
       <c r="K13" s="12" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>0.01876465903400463</v>
+        <v>0.01894530978330544</v>
       </c>
     </row>
     <row r="14">
@@ -1048,7 +1048,7 @@
         <v>46322</v>
       </c>
       <c r="I14" s="14" t="n">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>46338</v>
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.02439024411518612</v>
+        <v>0.02424242459271785</v>
       </c>
     </row>
     <row r="15">
@@ -1094,7 +1094,7 @@
         <v>46329</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>46338</v>
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>0.007486664208023313</v>
+        <v>0.007418397878032125</v>
       </c>
     </row>
     <row r="16">
@@ -1140,7 +1140,7 @@
         <v>46332</v>
       </c>
       <c r="I16" s="14" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>46346</v>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="L16" s="9" t="n">
-        <v>0.02453370826079572</v>
+        <v>0.02506741966611176</v>
       </c>
     </row>
     <row r="17">
@@ -1186,7 +1186,7 @@
         <v>46341</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>46340</v>
@@ -1197,7 +1197,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.02511582643638334</v>
+        <v>0.02559562696073051</v>
       </c>
     </row>
     <row r="18">
@@ -1232,7 +1232,7 @@
         <v>46344</v>
       </c>
       <c r="I18" s="14" t="n">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>46385</v>
@@ -1243,7 +1243,7 @@
         </is>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.03417038972317595</v>
+        <v>0.03562152032738169</v>
       </c>
     </row>
     <row r="19">
@@ -1278,7 +1278,7 @@
         <v>46347</v>
       </c>
       <c r="I19" s="14" t="n">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>46358</v>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0.03991199823387459</v>
+        <v>0.04176747804642418</v>
       </c>
     </row>
     <row r="20">
@@ -1324,7 +1324,7 @@
         <v>46352</v>
       </c>
       <c r="I20" s="14" t="n">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>46400</v>
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0.04855012550259507</v>
+        <v>0.05415896640739416</v>
       </c>
     </row>
     <row r="21">
@@ -1370,7 +1370,7 @@
         <v>46360</v>
       </c>
       <c r="I21" s="14" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46371</v>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.04544224897291059</v>
+        <v>0.04620144476449378</v>
       </c>
     </row>
     <row r="22">
@@ -1416,7 +1416,7 @@
         <v>46366</v>
       </c>
       <c r="I22" s="14" t="n">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="J22" s="10" t="n">
         <v>46432</v>
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="L22" s="9" t="n">
-        <v>0.02286760765227264</v>
+        <v>0.02340050090881113</v>
       </c>
     </row>
     <row r="23">
@@ -1462,7 +1462,7 @@
         <v>46380</v>
       </c>
       <c r="I23" s="14" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>46436</v>
@@ -1473,7 +1473,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0.02475502914436672</v>
+        <v>0.02447730673433134</v>
       </c>
     </row>
     <row r="24">
@@ -1508,7 +1508,7 @@
         <v>46383</v>
       </c>
       <c r="I24" s="21" t="n">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="J24" s="20" t="n">
         <v>46404</v>
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="L24" s="19" t="n">
-        <v>0.01450522461134869</v>
+        <v>0.01495185032156178</v>
       </c>
     </row>
     <row r="25">
@@ -1554,7 +1554,7 @@
         <v>46402</v>
       </c>
       <c r="I25" s="14" t="n">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>46483</v>
@@ -1565,7 +1565,7 @@
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>0.01403680539107752</v>
+        <v>0.01430829392812274</v>
       </c>
     </row>
     <row r="26">
@@ -1600,7 +1600,7 @@
         <v>46411</v>
       </c>
       <c r="I26" s="14" t="n">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>46435</v>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0.03921896959116871</v>
+        <v>0.03917525839818</v>
       </c>
     </row>
     <row r="27">
@@ -1646,7 +1646,7 @@
         <v>46417</v>
       </c>
       <c r="I27" s="14" t="n">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>46433</v>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="L27" s="9" t="n">
-        <v>0.03486606809614539</v>
+        <v>0.0344027820304614</v>
       </c>
     </row>
     <row r="28">
@@ -1692,7 +1692,7 @@
         <v>46423</v>
       </c>
       <c r="I28" s="14" t="n">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>46473</v>
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="L28" s="9" t="n">
-        <v>0.02462781771004423</v>
+        <v>0.02566432573547334</v>
       </c>
     </row>
     <row r="29">
@@ -1738,7 +1738,7 @@
         <v>46428</v>
       </c>
       <c r="I29" s="14" t="n">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>46452</v>
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>0.01436646286276235</v>
+        <v>0.01460247154118745</v>
       </c>
     </row>
     <row r="30">
@@ -1784,7 +1784,7 @@
         <v>46428</v>
       </c>
       <c r="I30" s="14" t="n">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="J30" s="10" t="n">
         <v>46460</v>
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="L30" s="9" t="n">
-        <v>0.04661168979740114</v>
+        <v>0.04735452249896756</v>
       </c>
     </row>
     <row r="31">
@@ -1830,7 +1830,7 @@
         <v>46431</v>
       </c>
       <c r="I31" s="14" t="n">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>46480</v>
@@ -1841,7 +1841,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="n">
-        <v>0.01533686311811834</v>
+        <v>0.0152091256013432</v>
       </c>
     </row>
     <row r="32">
@@ -1876,7 +1876,7 @@
         <v>46432</v>
       </c>
       <c r="I32" s="14" t="n">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>46455</v>
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="L32" s="9" t="n">
-        <v>0.03663203753211416</v>
+        <v>0.03662953552196622</v>
       </c>
     </row>
     <row r="33">
@@ -1922,7 +1922,7 @@
         <v>46433</v>
       </c>
       <c r="I33" s="14" t="n">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>46425</v>
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>0.004937215292389725</v>
+        <v>0.005040431742740933</v>
       </c>
     </row>
     <row r="34">
@@ -1968,7 +1968,7 @@
         <v>46433</v>
       </c>
       <c r="I34" s="14" t="n">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>46383</v>
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="L34" s="9" t="n">
-        <v>0.01873873873873874</v>
+        <v>0.0181735571637435</v>
       </c>
     </row>
     <row r="35">
@@ -2014,7 +2014,7 @@
         <v>46433</v>
       </c>
       <c r="I35" s="14" t="n">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>46368</v>
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0.02629956951214198</v>
+        <v>0.02618390189114882</v>
       </c>
     </row>
     <row r="36">
@@ -2060,7 +2060,7 @@
         <v>46433</v>
       </c>
       <c r="I36" s="14" t="n">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>46635</v>
@@ -2071,7 +2071,7 @@
         </is>
       </c>
       <c r="L36" s="9" t="n">
-        <v>0.02919292176686114</v>
+        <v>0.02949242555414726</v>
       </c>
     </row>
     <row r="37">
@@ -2106,7 +2106,7 @@
         <v>46433</v>
       </c>
       <c r="I37" s="14" t="n">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>46608</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>0.03261921323323592</v>
+        <v>0.03273988439306359</v>
       </c>
     </row>
     <row r="38">
@@ -2152,7 +2152,7 @@
         <v>46440</v>
       </c>
       <c r="I38" s="14" t="n">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>46450</v>
@@ -2163,7 +2163,7 @@
         </is>
       </c>
       <c r="L38" s="9" t="n">
-        <v>0.008765169347060732</v>
+        <v>0.009220619189905729</v>
       </c>
     </row>
     <row r="39">
@@ -2198,7 +2198,7 @@
         <v>46441</v>
       </c>
       <c r="I39" s="14" t="n">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>46456</v>
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.02728536827029688</v>
+        <v>0.02854692381271174</v>
       </c>
     </row>
     <row r="40">
@@ -2244,7 +2244,7 @@
         <v>46452</v>
       </c>
       <c r="I40" s="14" t="n">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="J40" s="10" t="n">
         <v>46487</v>
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.01650469054964427</v>
+        <v>0.01721244925575102</v>
       </c>
     </row>
     <row r="41">
@@ -2290,7 +2290,7 @@
         <v>46461</v>
       </c>
       <c r="I41" s="14" t="n">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>46300</v>
@@ -2301,7 +2301,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>0.01681119631420541</v>
+        <v>0.01680531053556927</v>
       </c>
     </row>
     <row r="42">
@@ -2336,7 +2336,7 @@
         <v>46461</v>
       </c>
       <c r="I42" s="14" t="n">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="J42" s="10" t="n">
         <v>46386</v>
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="L42" s="9" t="n">
-        <v>0.05137432770585006</v>
+        <v>0.05300301563463215</v>
       </c>
     </row>
     <row r="43">
@@ -2382,7 +2382,7 @@
         <v>46488</v>
       </c>
       <c r="I43" s="14" t="n">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>46498</v>
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>0.02976222999340377</v>
+        <v>0.03034905620460662</v>
       </c>
     </row>
     <row r="44">
@@ -2428,7 +2428,7 @@
         <v>46492</v>
       </c>
       <c r="I44" s="14" t="n">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="J44" s="10" t="n">
         <v>46501</v>
@@ -2439,7 +2439,7 @@
         </is>
       </c>
       <c r="L44" s="9" t="n">
-        <v>0.01991679185347889</v>
+        <v>0.02015045608281234</v>
       </c>
     </row>
     <row r="45">
@@ -2474,7 +2474,7 @@
         <v>46492</v>
       </c>
       <c r="I45" s="14" t="n">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="J45" s="10" t="n">
         <v>46376</v>
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="L45" s="9" t="n">
-        <v>0.04394062597018357</v>
+        <v>0.04408486562942009</v>
       </c>
     </row>
     <row r="46">
@@ -2520,7 +2520,7 @@
         <v>46493</v>
       </c>
       <c r="I46" s="14" t="n">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="J46" s="10" t="n">
         <v>46531</v>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="L46" s="9" t="n">
-        <v>0.01976911409091994</v>
+        <v>0.02003326473707467</v>
       </c>
     </row>
     <row r="47">
@@ -2566,7 +2566,7 @@
         <v>46499</v>
       </c>
       <c r="I47" s="14" t="n">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="J47" s="10" t="n">
         <v>46526</v>
@@ -2577,7 +2577,7 @@
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>0.02090879099284308</v>
+        <v>0.02048428436065614</v>
       </c>
     </row>
     <row r="48">
@@ -2612,7 +2612,7 @@
         <v>46504</v>
       </c>
       <c r="I48" s="14" t="n">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="J48" s="10" t="n">
         <v>46562</v>
@@ -2623,7 +2623,7 @@
         </is>
       </c>
       <c r="L48" s="9" t="n">
-        <v>0.04455225279189258</v>
+        <v>0.04505775240209334</v>
       </c>
     </row>
     <row r="49">
@@ -2658,7 +2658,7 @@
         <v>46508</v>
       </c>
       <c r="I49" s="14" t="n">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>46518</v>
@@ -2669,7 +2669,7 @@
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>0.03756016628985256</v>
+        <v>0.03790865215187018</v>
       </c>
     </row>
     <row r="50">
@@ -2704,7 +2704,7 @@
         <v>46515</v>
       </c>
       <c r="I50" s="14" t="n">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="J50" s="10" t="n">
         <v>46542</v>
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="L50" s="9" t="n">
-        <v>0.04064538447016642</v>
+        <v>0.04233409721847894</v>
       </c>
     </row>
     <row r="51">
@@ -2750,7 +2750,7 @@
         <v>46532</v>
       </c>
       <c r="I51" s="14" t="n">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="J51" s="10" t="n">
         <v>46563</v>
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>0.03071017314446581</v>
+        <v>0.03186898210102054</v>
       </c>
     </row>
     <row r="52">
@@ -2796,7 +2796,7 @@
         <v>46585</v>
       </c>
       <c r="I52" s="14" t="n">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="J52" s="10" t="n">
         <v>46629</v>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="L52" s="9" t="n">
-        <v>0.01778722342210357</v>
+        <v>0.01816536404771699</v>
       </c>
     </row>
     <row r="53">
@@ -2842,7 +2842,7 @@
         <v>46592</v>
       </c>
       <c r="I53" s="14" t="n">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="J53" s="10" t="n">
         <v>46632</v>
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="L53" s="9" t="n">
-        <v>0.03298231550978693</v>
+        <v>0.03444519299078828</v>
       </c>
     </row>
     <row r="54">
@@ -2888,7 +2888,7 @@
         <v>46594</v>
       </c>
       <c r="I54" s="14" t="n">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="J54" s="10" t="n">
         <v>46613</v>
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="L54" s="9" t="n">
-        <v>0.01592686642965973</v>
+        <v>0.01600457321365694</v>
       </c>
     </row>
     <row r="55">
@@ -2934,7 +2934,7 @@
         <v>46595</v>
       </c>
       <c r="I55" s="14" t="n">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="J55" s="10" t="n">
         <v>46614</v>
@@ -2945,7 +2945,7 @@
         </is>
       </c>
       <c r="L55" s="9" t="n">
-        <v>0.02452830163458748</v>
+        <v>0.02444046536574221</v>
       </c>
     </row>
     <row r="56">
@@ -2980,7 +2980,7 @@
         <v>46597</v>
       </c>
       <c r="I56" s="14" t="n">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="J56" s="10" t="n">
         <v>46611</v>
@@ -2991,7 +2991,7 @@
         </is>
       </c>
       <c r="L56" s="9" t="n">
-        <v>0.04599181500645778</v>
+        <v>0.05033725871166542</v>
       </c>
     </row>
     <row r="57">
@@ -3026,7 +3026,7 @@
         <v>46598</v>
       </c>
       <c r="I57" s="14" t="n">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="J57" s="10" t="n">
         <v>46629</v>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="L57" s="9" t="n">
-        <v>0.02484172353559332</v>
+        <v>0.02572588296608385</v>
       </c>
     </row>
   </sheetData>
@@ -3072,7 +3072,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Expected Increase Announcements by Month - 08/24/2026</t>
+          <t>Expected Increase Announcements by Month - 08/31/2026</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
         <v>46263</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>46297</v>
+        <v>46662</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>0.82</v>
@@ -3407,10 +3407,10 @@
         </is>
       </c>
       <c r="B22" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="C22" s="10" t="n">
-        <v>46351</v>
+        <v>46352</v>
       </c>
       <c r="D22" s="7" t="n">
         <v>1.38</v>
@@ -4831,7 +4831,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete Holdings Dividend Summary - 08/24/2026</t>
+          <t>Complete Holdings Dividend Summary - 08/31/2026</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4935,7 @@
         <v>1.16</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.008765169347060732</v>
+        <v>0.009220619189905729</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>46255</v>
@@ -4988,7 +4988,7 @@
         <v>10.08</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.02286760765227264</v>
+        <v>0.02340050090881113</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>46255</v>
@@ -5041,7 +5041,7 @@
         <v>8.552</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.004937215292389725</v>
+        <v>0.005040431742740933</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>46231</v>
@@ -5094,7 +5094,7 @@
         <v>2.184</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.02452830163458748</v>
+        <v>0.02444046536574221</v>
       </c>
       <c r="I8" s="10" t="n">
         <v>46251</v>
@@ -5147,7 +5147,7 @@
         <v>2.812</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.03921896959116871</v>
+        <v>0.03917525839818</v>
       </c>
       <c r="I9" s="10" t="n">
         <v>46251</v>
@@ -5200,7 +5200,7 @@
         <v>4.12</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.02484172353559332</v>
+        <v>0.02572588296608385</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>46171</v>
@@ -5253,7 +5253,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.04599181500645778</v>
+        <v>0.05033725871166542</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>46246</v>
@@ -5306,7 +5306,7 @@
         <v>5.2</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.01873873873873874</v>
+        <v>0.0181735571637435</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>46182</v>
@@ -5359,7 +5359,7 @@
         <v>0.96</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0.02475502914436672</v>
+        <v>0.02447730673433134</v>
       </c>
       <c r="I13" s="10" t="n">
         <v>46254</v>
@@ -5412,7 +5412,7 @@
         <v>2.4</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0.007486664208023313</v>
+        <v>0.007418397878032125</v>
       </c>
       <c r="I14" s="10" t="n">
         <v>46248</v>
@@ -5465,7 +5465,7 @@
         <v>1.68</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.01533686311811834</v>
+        <v>0.0152091256013432</v>
       </c>
       <c r="I15" s="10" t="n">
         <v>46209</v>
@@ -5518,7 +5518,7 @@
         <v>7.12</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.03486606809614539</v>
+        <v>0.0344027820304614</v>
       </c>
       <c r="I16" s="10" t="n">
         <v>46253</v>
@@ -5571,7 +5571,7 @@
         <v>3.44</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.01403680539107752</v>
+        <v>0.01430829392812274</v>
       </c>
       <c r="I17" s="10" t="n">
         <v>46211</v>
@@ -5624,7 +5624,7 @@
         <v>1.28</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.02629956951214198</v>
+        <v>0.02618390189114882</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>46188</v>
@@ -5677,7 +5677,7 @@
         <v>3.36</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.04544224897291059</v>
+        <v>0.04620144476449378</v>
       </c>
       <c r="I19" s="10" t="n">
         <v>46188</v>
@@ -5730,7 +5730,7 @@
         <v>2.56</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.02439024411518612</v>
+        <v>0.02424242459271785</v>
       </c>
       <c r="I20" s="10" t="n">
         <v>46247</v>
@@ -5783,7 +5783,7 @@
         <v>6.36</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.01650469054964427</v>
+        <v>0.01721244925575102</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>46205</v>
@@ -5836,7 +5836,7 @@
         <v>1.18</v>
       </c>
       <c r="H22" s="19" t="n">
-        <v>0.01450522461134869</v>
+        <v>0.01495185032156178</v>
       </c>
       <c r="I22" s="20" t="n">
         <v>46223</v>
@@ -5889,7 +5889,7 @@
         <v>9.32</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.02728536827029688</v>
+        <v>0.02854692381271174</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>46177</v>
@@ -5942,19 +5942,19 @@
         <v>5.52</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>0.01876465903400463</v>
+        <v>0.01894530978330544</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>46171</v>
+        <v>46262</v>
       </c>
       <c r="J24" s="8" t="n">
         <v>0.02222222222222208</v>
       </c>
       <c r="K24" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="L24" s="10" t="n">
-        <v>46351</v>
+        <v>46352</v>
       </c>
       <c r="M24" s="12" t="inlineStr">
         <is>
@@ -5995,7 +5995,7 @@
         <v>1.172</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.04855012550259507</v>
+        <v>0.05415896640739416</v>
       </c>
       <c r="I25" s="10" t="n">
         <v>46216</v>
@@ -6048,7 +6048,7 @@
         <v>3.28</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>0.03052582683254938</v>
+        <v>0.03150967828940907</v>
       </c>
       <c r="I26" s="10" t="n">
         <v>46204</v>
@@ -6060,7 +6060,7 @@
         <v>46263</v>
       </c>
       <c r="L26" s="10" t="n">
-        <v>46297</v>
+        <v>46662</v>
       </c>
       <c r="M26" s="12" t="inlineStr">
         <is>
@@ -6101,7 +6101,7 @@
         <v>2.44</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.01436646286276235</v>
+        <v>0.01460247154118745</v>
       </c>
       <c r="I27" s="10" t="n">
         <v>46174</v>
@@ -6154,10 +6154,10 @@
         <v>5.36</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0.01976911409091994</v>
+        <v>0.02003326473707467</v>
       </c>
       <c r="I28" s="10" t="n">
-        <v>46168</v>
+        <v>46259</v>
       </c>
       <c r="J28" s="8" t="n">
         <v>0.0307692307692308</v>
@@ -6207,7 +6207,7 @@
         <v>6</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.01681119631420541</v>
+        <v>0.01680531053556927</v>
       </c>
       <c r="I29" s="10" t="n">
         <v>46209</v>
@@ -6260,7 +6260,7 @@
         <v>2.25</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.01991679185347889</v>
+        <v>0.02015045608281234</v>
       </c>
       <c r="I30" s="10" t="n">
         <v>46216</v>
@@ -6313,7 +6313,7 @@
         <v>3.16</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0.01113362059047492</v>
+        <v>0.01116568280612038</v>
       </c>
       <c r="I31" s="10" t="n">
         <v>46203</v>
@@ -6366,7 +6366,7 @@
         <v>2.88</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.03071017314446581</v>
+        <v>0.03186898210102054</v>
       </c>
       <c r="I32" s="10" t="n">
         <v>46199</v>
@@ -6419,7 +6419,7 @@
         <v>1.92</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0.03417038972317595</v>
+        <v>0.03562152032738169</v>
       </c>
       <c r="I33" s="10" t="n">
         <v>46209</v>
@@ -6472,7 +6472,7 @@
         <v>3.64</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0.00746459939730233</v>
+        <v>0.007159787328081065</v>
       </c>
       <c r="I34" s="10" t="n">
         <v>46254</v>
@@ -6525,7 +6525,7 @@
         <v>3.48</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0.02885811514786943</v>
+        <v>0.02914084787605498</v>
       </c>
       <c r="I35" s="10" t="n">
         <v>46211</v>
@@ -6578,7 +6578,7 @@
         <v>1.64</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0.03991199823387459</v>
+        <v>0.04176747804642418</v>
       </c>
       <c r="I36" s="10" t="n">
         <v>46174</v>
@@ -6631,7 +6631,7 @@
         <v>1.158</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.02462781771004423</v>
+        <v>0.02566432573547334</v>
       </c>
       <c r="I37" s="10" t="n">
         <v>46251</v>
@@ -6684,7 +6684,7 @@
         <v>3.252</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0.05137432770585006</v>
+        <v>0.05300301563463215</v>
       </c>
       <c r="I38" s="10" t="n">
         <v>46234</v>
@@ -6737,7 +6737,7 @@
         <v>4.76</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.03756016628985256</v>
+        <v>0.03790865215187018</v>
       </c>
       <c r="I39" s="10" t="n">
         <v>46231</v>
@@ -6790,7 +6790,7 @@
         <v>2.68</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.03663203753211416</v>
+        <v>0.03662953552196622</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>46182</v>
@@ -6843,7 +6843,7 @@
         <v>5.92</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0.04064538447016642</v>
+        <v>0.04233409721847894</v>
       </c>
       <c r="I41" s="10" t="n">
         <v>46178</v>
@@ -6896,7 +6896,7 @@
         <v>1.72</v>
       </c>
       <c r="H42" s="9" t="n">
-        <v>0.06156357035591447</v>
+        <v>0.06160458435888048</v>
       </c>
       <c r="I42" s="10" t="n">
         <v>46227</v>
@@ -6949,7 +6949,7 @@
         <v>3.28</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0.02919292176686114</v>
+        <v>0.02949242555414726</v>
       </c>
       <c r="I43" s="10" t="n">
         <v>46174</v>
@@ -7002,7 +7002,7 @@
         <v>4.356</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.02976222999340377</v>
+        <v>0.03034905620460662</v>
       </c>
       <c r="I44" s="10" t="n">
         <v>46227</v>
@@ -7055,7 +7055,7 @@
         <v>2.204</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>0.04455225279189258</v>
+        <v>0.04505775240209334</v>
       </c>
       <c r="I45" s="10" t="n">
         <v>46198</v>
@@ -7108,7 +7108,7 @@
         <v>5.08</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.02090879099284308</v>
+        <v>0.02048428436065614</v>
       </c>
       <c r="I46" s="10" t="n">
         <v>46252</v>
@@ -7161,7 +7161,7 @@
         <v>3.92</v>
       </c>
       <c r="H47" s="9" t="n">
-        <v>0.01592686642965973</v>
+        <v>0.01600457321365694</v>
       </c>
       <c r="I47" s="10" t="n">
         <v>46252</v>
@@ -7214,7 +7214,7 @@
         <v>9.76</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>0.02453370826079572</v>
+        <v>0.02506741966611176</v>
       </c>
       <c r="I48" s="10" t="n">
         <v>46253</v>
@@ -7267,7 +7267,7 @@
         <v>3.32</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.03298231550978693</v>
+        <v>0.03444519299078828</v>
       </c>
       <c r="I49" s="10" t="n">
         <v>46181</v>
@@ -7320,7 +7320,7 @@
         <v>5.2</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.04661168979740114</v>
+        <v>0.04735452249896756</v>
       </c>
       <c r="I50" s="10" t="n">
         <v>46188</v>
@@ -7373,7 +7373,7 @@
         <v>3.896</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.04394062597018357</v>
+        <v>0.04408486562942009</v>
       </c>
       <c r="I51" s="10" t="n">
         <v>46112</v>
@@ -7426,7 +7426,7 @@
         <v>5.68</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.02203856655366886</v>
+        <v>0.02174245985426699</v>
       </c>
       <c r="I52" s="10" t="n">
         <v>46234</v>
@@ -7479,7 +7479,7 @@
         <v>2.124</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>0.03261921323323592</v>
+        <v>0.03273988439306359</v>
       </c>
       <c r="I53" s="10" t="n">
         <v>46241</v>
@@ -7532,7 +7532,7 @@
         <v>5.52</v>
       </c>
       <c r="H54" s="9" t="n">
-        <v>0.01778722342210357</v>
+        <v>0.01816536404771699</v>
       </c>
       <c r="I54" s="10" t="n">
         <v>46171</v>
@@ -7585,7 +7585,7 @@
         <v>2.832</v>
       </c>
       <c r="H55" s="9" t="n">
-        <v>0.05682182968157457</v>
+        <v>0.05667400301816825</v>
       </c>
       <c r="I55" s="10" t="n">
         <v>46213</v>
@@ -7638,7 +7638,7 @@
         <v>4.12</v>
       </c>
       <c r="H56" s="9" t="n">
-        <v>0.02511582643638334</v>
+        <v>0.02559562696073051</v>
       </c>
       <c r="I56" s="10" t="n">
         <v>46251</v>

</xml_diff>